<commit_message>
data: refresh models and pricing for 2026-09-07
</commit_message>
<xml_diff>
--- a/public/AI模型厂商全景_2023-2026.xlsx
+++ b/public/AI模型厂商全景_2023-2026.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Re8dba41062f04036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="厂商地图" sheetId="2" r:id="R7a89739aa8824de0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型时间轴" sheetId="3" r:id="R1be871a31d6b4ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前定价" sheetId="4" r:id="R3b69c52b724f47d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本计算器" sheetId="5" r:id="Rdfab913af245456a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用案例" sheetId="6" r:id="R8f088369bcbf4f6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景选型" sheetId="7" r:id="R8a5b61ebc9b24abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料来源" sheetId="8" r:id="R4bbb141beaaa4850"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R9ac234d8b78b4553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="厂商地图" sheetId="2" r:id="Rf7836ba07e7f4b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型时间轴" sheetId="3" r:id="R6b216b3527914c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前定价" sheetId="4" r:id="R0a228ce26e544ce3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本计算器" sheetId="5" r:id="R7c654cef0df84228"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用案例" sheetId="6" r:id="R0005ff6b4aeb4c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景选型" sheetId="7" r:id="Rf815e41ab1d04810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料来源" sheetId="8" r:id="Re97935fc9c4f448e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -719,8 +719,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PricesTable" displayName="PricesTable" ref="A2:O46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A2:O46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PricesTable" displayName="PricesTable" ref="A2:O54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A2:O54"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="区域"/>
     <x:tableColumn id="2" name="厂商"/>
@@ -743,8 +743,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CostCalculatorTable" displayName="CostCalculatorTable" ref="A9:O51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A9:O51"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CostCalculatorTable" displayName="CostCalculatorTable" ref="A9:O59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A9:O59"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="区域"/>
     <x:tableColumn id="2" name="厂商"/>
@@ -803,8 +803,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SourcesTable" displayName="SourcesTable" ref="A12:F153" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A12:F153"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SourcesTable" displayName="SourcesTable" ref="A12:F161" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A12:F161"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="类别"/>
     <x:tableColumn id="2" name="厂商/对象"/>
@@ -1066,7 +1066,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>研究日：2026-08-24｜范围：24 家代表厂商｜价格与产品为查询日快照，采购前请复核来源</x:v>
+        <x:v>研究日：2026-09-07｜范围：24 家代表厂商｜价格与产品为查询日快照，采购前请复核来源</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1099,8 +1099,7 @@
         <x:v>当前价格行</x:v>
       </x:c>
       <x:c r="H4" s="15" t="n">
-        <x:f>COUNTA('当前定价'!$C$3:$C$90)</x:f>
-        <x:v>44</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="J4" s="14" t="str">
         <x:v>公开案例</x:v>
@@ -1243,7 +1242,7 @@
       <x:c r="B14" s="64"/>
       <x:c r="C14" s="64"/>
       <x:c r="D14" s="64" t="str">
-        <x:v>GPT-5.6 Sol；Claude；Grok 4.6；GLM-5.2；DeepSeek V4 Pro；Kimi K3</x:v>
+        <x:v>GPT-6 Astra；Claude Fable 5.1 / Opus；GLM-5.3；DeepSeek V4 Pro；Kimi K3</x:v>
       </x:c>
       <x:c r="E14" s="64"/>
       <x:c r="F14" s="64"/>
@@ -1504,10 +1503,10 @@
         <x:v>OpenAI</x:v>
       </x:c>
       <x:c r="C3" s="88" t="str">
-        <x:v>从 GPT-4 的多模态能力，演进到 GPT-4o 的实时多模态、o1 的推理范式，再到 GPT-5/5.6 的统一推理与 Agent 工具栈。</x:v>
+        <x:v>从 GPT-4 的多模态能力，演进到 GPT-4o 的实时多模态、o1 的推理范式、GPT-5/5.6 的统一推理与 Agent 工具栈，并在 2026-09 推出 GPT-6 Astra。</x:v>
       </x:c>
       <x:c r="D3" s="88" t="str">
-        <x:v>GPT-5.6 Sol / Terra / Luna；GPT-Realtime-2.1；GPT-Image-2</x:v>
+        <x:v>GPT-6 Astra；GPT-5.6 Sol / Terra / Luna；GPT-Realtime-2.1；GPT-Image-2</x:v>
       </x:c>
       <x:c r="E3" s="88" t="str">
         <x:v>ChatGPT、Responses API、Codex、Sora</x:v>
@@ -1522,16 +1521,16 @@
         <x:v>第一方 API；云市场渠道</x:v>
       </x:c>
       <x:c r="I3" s="88" t="str">
-        <x:v>Sol $4/$20；Terra $2/$12；Luna $0.2/$1.2（输入/输出，USD/百万tokens）</x:v>
+        <x:v>Astra $10/$50；Sol $4/$20；Luna $0.2/$1.2（输入/输出，USD/百万tokens）</x:v>
       </x:c>
       <x:c r="J3" s="88" t="str">
         <x:v>高难知识工作、代码 Agent、通用智能体、高并发分层路由</x:v>
       </x:c>
       <x:c r="K3" s="95" t="str">
-        <x:v>https://developers.openai.com/api/docs/models</x:v>
+        <x:v>https://developers.openai.com/api/docs/models/gpt-6-astra</x:v>
       </x:c>
       <x:c r="L3" s="89" t="str">
-        <x:v>【公开事实】当前目录与价格按查询日快照</x:v>
+        <x:v>【公开事实】Astra &gt;272K 整次请求升价；Batch/Flex 与 Fast 档另计</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
@@ -1542,10 +1541,10 @@
         <x:v>Anthropic</x:v>
       </x:c>
       <x:c r="C4" s="64" t="str">
-        <x:v>从 Claude 2 的长上下文与安全定位，发展到 Claude 3/3.5 的分层模型，再到 Claude 4/5 的长周期 Agent 与编码能力。</x:v>
+        <x:v>从 Claude 2 的长上下文与安全定位，发展到 Claude 3/3.5 的分层模型、Claude 4/5 的长周期 Agent，并在 2026-09 推出 Fable 5.1。</x:v>
       </x:c>
       <x:c r="D4" s="64" t="str">
-        <x:v>Claude Fable 5 / Opus 5 / Sonnet 5 / Haiku 4.5</x:v>
+        <x:v>Claude Fable 5.1 / Opus 5 / Sonnet 5 / Haiku 4.5</x:v>
       </x:c>
       <x:c r="E4" s="64" t="str">
         <x:v>Claude、Claude Code、Claude Platform、Managed Agents</x:v>
@@ -1560,16 +1559,16 @@
         <x:v>Claude API；AWS、Google Cloud、Microsoft Foundry</x:v>
       </x:c>
       <x:c r="I4" s="64" t="str">
-        <x:v>Sonnet 5 $2/$10；Opus 5 $5/$25；缓存读约基础输入价 0.1×</x:v>
+        <x:v>Fable 5.1 $10/$50；Sonnet 5 $2/$10；缓存读约基础输入价 0.1×</x:v>
       </x:c>
       <x:c r="J4" s="64" t="str">
         <x:v>复杂编码、企业 Agent、知识工作、需强安全控制的应用</x:v>
       </x:c>
       <x:c r="K4" s="96" t="str">
-        <x:v>https://platform.claude.com/docs/en/home</x:v>
+        <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
       </x:c>
       <x:c r="L4" s="91" t="str">
-        <x:v>【公开事实】注意缓存写入与地域溢价</x:v>
+        <x:v>【公开事实】Fable 缓存写入与 US-only inference、Batch 档需单独核算</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
@@ -1580,10 +1579,10 @@
         <x:v>Google DeepMind</x:v>
       </x:c>
       <x:c r="C5" s="64" t="str">
-        <x:v>以 Gemini 1 建立原生多模态路线，Gemini 1.5 扩展长上下文，2.x/3.x 进一步强化推理、搜索 Grounding、实时与 Agent。</x:v>
+        <x:v>以 Gemini 1 建立原生多模态路线，Gemini 1.5 扩展长上下文，2.x/3.x 强化推理、搜索与 Agent；2026-09 推出 3.8 Flash 与 Lyria 3.5。</x:v>
       </x:c>
       <x:c r="D5" s="64" t="str">
-        <x:v>Gemini 3.1 Pro / 3.7 Flash / 3.5 Flash-Lite；Gemma</x:v>
+        <x:v>Gemini 3.8 Flash / 3.7 Flash / 3.5 Flash-Lite；Lyria 3.5；Gemma</x:v>
       </x:c>
       <x:c r="E5" s="64" t="str">
         <x:v>Gemini、AI Studio、Vertex AI、Workspace、Android/Pixel</x:v>
@@ -1598,16 +1597,16 @@
         <x:v>Gemini API、Vertex AI、端侧</x:v>
       </x:c>
       <x:c r="I5" s="64" t="str">
-        <x:v>3.7 Flash 促销 $0.75/$3.75；3.5 Flash-Lite $0.30/$2.50</x:v>
+        <x:v>3.8 Flash 促销 $0.75/$3.75（至 2026-12-31）；之后 $1.5/$7.5</x:v>
       </x:c>
       <x:c r="J5" s="64" t="str">
         <x:v>搜索增强、多模态文档、Workspace、端侧与高吞吐</x:v>
       </x:c>
       <x:c r="K5" s="96" t="str">
-        <x:v>https://ai.google.dev/gemini-api/docs/models</x:v>
+        <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
       </x:c>
       <x:c r="L5" s="91" t="str">
-        <x:v>【公开事实】搜索/地图 Grounding 另收费</x:v>
+        <x:v>【公开事实】搜索/地图 Grounding、音视频与区域价格另计</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -1618,13 +1617,13 @@
         <x:v>Meta</x:v>
       </x:c>
       <x:c r="C6" s="64" t="str">
-        <x:v>以 Llama 2/3/4 建立开放权重生态，支持微调、私有化与云端托管；消费产品由 Meta AI 和眼镜等终端承接。</x:v>
+        <x:v>以 Llama 2/3/4 建立开放权重生态；2026 年扩展 Muse Spark 1.3、Muse Voice、Muse Image 与第一方 Model API。</x:v>
       </x:c>
       <x:c r="D6" s="64" t="str">
-        <x:v>Llama 4 Scout/Maverick；Muse Spark</x:v>
+        <x:v>Llama 4 Scout/Maverick；Muse Spark 1.3；Muse Voice；Muse Image</x:v>
       </x:c>
       <x:c r="E6" s="64" t="str">
-        <x:v>Meta AI、WhatsApp/Instagram/Facebook、Ray-Ban Meta</x:v>
+        <x:v>Meta AI、Model API、WhatsApp/Instagram/Facebook、Ray-Ban Meta</x:v>
       </x:c>
       <x:c r="F6" s="64" t="str">
         <x:v>开放生态、可控私有化、微调、端侧与云端可移植性</x:v>
@@ -1633,19 +1632,19 @@
         <x:v>开放权重（许可证有条件）+ 部分闭源</x:v>
       </x:c>
       <x:c r="H6" s="64" t="str">
-        <x:v>自建、云厂商托管、端侧</x:v>
+        <x:v>第一方 Model API、自建、云厂商托管、端侧</x:v>
       </x:c>
       <x:c r="I6" s="64" t="str">
-        <x:v>无统一第一方 API 标价；权重不收费但需承担算力和运维</x:v>
+        <x:v>Voice Transcribe $0.18/小时；Muse Image $0.01/张；文本 token 价以控制台为准</x:v>
       </x:c>
       <x:c r="J6" s="64" t="str">
         <x:v>行业微调、私有部署、客服、端侧助手、合成数据</x:v>
       </x:c>
       <x:c r="K6" s="96" t="str">
-        <x:v>https://ai.meta.com/llama/</x:v>
+        <x:v>https://developer.meta.com/ai</x:v>
       </x:c>
       <x:c r="L6" s="91" t="str">
-        <x:v>【公开事实】开放权重不等于零成本</x:v>
+        <x:v>【公开事实】开放权重与第一方 API 为不同成本口径</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -1718,10 +1717,10 @@
         <x:v>低成本 Agent、文档智能、代码、欧洲数据主权</x:v>
       </x:c>
       <x:c r="K8" s="96" t="str">
-        <x:v>https://docs.mistral.ai/models</x:v>
+        <x:v>https://docs.mistral.ai/getting-started/changelog/</x:v>
       </x:c>
       <x:c r="L8" s="91" t="str">
-        <x:v>【公开事实】兼顾 API 与权重部署</x:v>
+        <x:v>【公开事实】OCR 4.1 已 GA；Leanstral 1.5 将于 2026-09-30 退役</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -1750,16 +1749,16 @@
         <x:v>API、云市场、VPC/本地 Vault</x:v>
       </x:c>
       <x:c r="I9" s="64" t="str">
-        <x:v>Command A+ 约 $2.5/$10；私有 Vault 按实例/承诺计费</x:v>
+        <x:v>Command A+ 自助 API 免费至触发限速；生产私有 Vault 按实例/承诺计费</x:v>
       </x:c>
       <x:c r="J9" s="64" t="str">
         <x:v>企业搜索、知识库、客服、主权/保密部署</x:v>
       </x:c>
       <x:c r="K9" s="96" t="str">
-        <x:v>https://docs.cohere.com/docs/models</x:v>
+        <x:v>https://docs.cohere.com/docs/command-a-plus</x:v>
       </x:c>
       <x:c r="L9" s="91" t="str">
-        <x:v>【公开事实】适合把生成与检索组件组合评测</x:v>
+        <x:v>【公开事实】免费限速档不等于生产 SLA 或无限额度</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -1773,7 +1772,7 @@
         <x:v>Bedrock 作为多模型托管入口，Amazon 自研从 Titan 扩展至 Nova 的理解、创作、实时语音与定制模型。</x:v>
       </x:c>
       <x:c r="D10" s="64" t="str">
-        <x:v>Nova 2 Lite / Sonic；Nova Premier；Nova Forge</x:v>
+        <x:v>Nova 2 Lite / Sonic；Nova Premier / Forge；Claude Fable 5.1</x:v>
       </x:c>
       <x:c r="E10" s="64" t="str">
         <x:v>Amazon Bedrock、Amazon Q、Nova Act/Forge</x:v>
@@ -1794,10 +1793,10 @@
         <x:v>AWS 既有客户、客服/RAG、多模型路由、语音应用</x:v>
       </x:c>
       <x:c r="K10" s="96" t="str">
-        <x:v>https://aws.amazon.com/bedrock/</x:v>
+        <x:v>https://aws.amazon.com/about-aws/whats-new/2026/09/claude-fable-5-1-aws/</x:v>
       </x:c>
       <x:c r="L10" s="91" t="str">
-        <x:v>【公开事实】Bedrock 案例常使用第三方底模</x:v>
+        <x:v>【公开事实】Bedrock 同时提供自研与第三方模型，价格随区域/档位变化</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -1811,7 +1810,7 @@
         <x:v>Phi 路线强调小模型与端侧；MAI 路线面向 Copilot 的自研闭源前沿模型，并与 Azure 模型目录形成组合。</x:v>
       </x:c>
       <x:c r="D11" s="64" t="str">
-        <x:v>Phi-4 Reasoning Vision；MAI-1 / MAI-Voice</x:v>
+        <x:v>Phi-4 Reasoning Vision；MAI-1；MAI-Voice；MAI-Transcribe-2；GPT-6 Astra</x:v>
       </x:c>
       <x:c r="E11" s="64" t="str">
         <x:v>Microsoft Copilot、Azure AI Foundry、Windows/Edge</x:v>
@@ -1826,16 +1825,16 @@
         <x:v>本地/端侧、Azure、Copilot</x:v>
       </x:c>
       <x:c r="I11" s="64" t="str">
-        <x:v>Phi 权重无按 token 许可费；托管成本按 Azure 部署计</x:v>
+        <x:v>Foundry Astra 短上下文 $10/$50；Phi/MAI 与语音模型按服务计费</x:v>
       </x:c>
       <x:c r="J11" s="64" t="str">
         <x:v>端侧、离线、轻量代码/视觉、微软生态应用</x:v>
       </x:c>
       <x:c r="K11" s="96" t="str">
-        <x:v>https://microsoft.ai/news/introducing-mai-1-preview-and-mai-voice-1/</x:v>
+        <x:v>https://azure.microsoft.com/en-us/blog/gpt-6-astra-frontier-intelligence-for-work-now-generally-available-in-microsoft-foundry/</x:v>
       </x:c>
       <x:c r="L11" s="91" t="str">
-        <x:v>【公开事实】MAI 生产 API 价未统一公开</x:v>
+        <x:v>【公开事实】MAI-Transcribe-2 于 2026-09-03 发布；区域可用性需核验</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -1902,13 +1901,13 @@
         <x:v>百炼 API、开源自建、专属部署</x:v>
       </x:c>
       <x:c r="I13" s="64" t="str">
-        <x:v>Qwen3.8-Max ¥12/¥36；Qwen3-Max ≤32K ¥2.5/¥10</x:v>
+        <x:v>Qwen3.8-Max ¥12/¥36；Qwen3.8-Max Prime ¥24/¥72；Qwen3-Max ≤32K ¥2.5/¥10</x:v>
       </x:c>
       <x:c r="J13" s="64" t="str">
         <x:v>中文 Agent、代码、企业知识、私有化、底模微调</x:v>
       </x:c>
       <x:c r="K13" s="96" t="str">
-        <x:v>https://qwenlm.github.io/</x:v>
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
       </x:c>
       <x:c r="L13" s="91" t="str">
         <x:v>【公开事实】上下文长度会触发阶梯价</x:v>
@@ -1940,13 +1939,13 @@
         <x:v>千帆 API、专属资源、私有化</x:v>
       </x:c>
       <x:c r="I14" s="64" t="str">
-        <x:v>ERNIE 5.1 ≤32K ¥4/¥18；4.5 Turbo ¥0.8/¥3.2</x:v>
+        <x:v>ERNIE 5.1 ≤32K ¥4/¥18；32K—128K ¥6/¥22；4.5 Turbo ¥0.8/¥3.2</x:v>
       </x:c>
       <x:c r="J14" s="64" t="str">
         <x:v>政企知识库、客服、搜索、内容与多模态应用</x:v>
       </x:c>
       <x:c r="K14" s="96" t="str">
-        <x:v>https://cloud.baidu.com/product-s/qianfan_home</x:v>
+        <x:v>https://cloud.baidu.com/doc/qianfan/s/wmh4sv6ya</x:v>
       </x:c>
       <x:c r="L14" s="91" t="str">
         <x:v>【公开事实】千帆还托管第三方模型</x:v>
@@ -1998,10 +1997,10 @@
         <x:v>腾讯 / 混元 Hy</x:v>
       </x:c>
       <x:c r="C16" s="64" t="str">
-        <x:v>从 2023 通用大模型，发展到 T1/Turbo S 推理与 Hy3 Agent；同时延伸图片、视频、3D 等生成能力。</x:v>
+        <x:v>从 2023 通用大模型，发展到 T1/Turbo S 推理与 Hy3 Agent；2026-09 推出 Hy4 Preview，并延伸图片、视频和 3D。</x:v>
       </x:c>
       <x:c r="D16" s="64" t="str">
-        <x:v>Hy3；混元图像/视频/3D；腾讯代码模型</x:v>
+        <x:v>Hy4 Preview；Hy3；混元图像/视频/3D；腾讯代码模型</x:v>
       </x:c>
       <x:c r="E16" s="64" t="str">
         <x:v>腾讯元宝、ima、WorkBuddy、CodeBuddy、TokenHub、微信/腾讯云生态</x:v>
@@ -2016,16 +2015,16 @@
         <x:v>TokenHub API、专属部署、腾讯云</x:v>
       </x:c>
       <x:c r="I16" s="64" t="str">
-        <x:v>Hy3 约 ¥1/¥4，缓存约 ¥0.25；生成模型按次/Token</x:v>
+        <x:v>Hy4 Preview ¥6/¥18，缓存 ¥0.3；Hy3 约 ¥1/¥4，缓存约 ¥0.25</x:v>
       </x:c>
       <x:c r="J16" s="64" t="str">
         <x:v>企业 Agent、办公/代码、微信生态客服、多媒体生成</x:v>
       </x:c>
       <x:c r="K16" s="96" t="str">
-        <x:v>https://cloud.tencent.com/product/tokenhub</x:v>
+        <x:v>https://cloud.tencent.com/document/product/1823/130055</x:v>
       </x:c>
       <x:c r="L16" s="91" t="str">
-        <x:v>【公开事实】原混元售卖入口逐步迁移 TokenHub</x:v>
+        <x:v>【公开事实】Hy4 为 Preview；原混元售卖入口逐步迁移 TokenHub</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -2039,7 +2038,7 @@
         <x:v>以 ChatGLM 开源生态和 BigModel MaaS 切入，GLM-4.5 后重点转向代码、Agent 与长周期工程任务。</x:v>
       </x:c>
       <x:c r="D17" s="64" t="str">
-        <x:v>GLM-5.2 / 5.1；GLM-5V-Turbo；GLM-4.7-FlashX</x:v>
+        <x:v>GLM-5.3 / 5.2；GLM-5V-Turbo；GLM-4.7-FlashX</x:v>
       </x:c>
       <x:c r="E17" s="64" t="str">
         <x:v>智谱清言、AutoGLM、GLM Coding Plan、开放平台</x:v>
@@ -2054,13 +2053,13 @@
         <x:v>BigModel API、私有化、代码订阅</x:v>
       </x:c>
       <x:c r="I17" s="64" t="str">
-        <x:v>GLM-5.2 ¥8/¥28；GLM-4.7-FlashX ¥0.5/¥3</x:v>
+        <x:v>GLM-5.3 ¥8/¥28，缓存 ¥2；GLM-4.7-FlashX ¥0.5/¥3</x:v>
       </x:c>
       <x:c r="J17" s="64" t="str">
         <x:v>代码 Agent、企业知识库、工单/合同、视觉操作</x:v>
       </x:c>
       <x:c r="K17" s="96" t="str">
-        <x:v>https://docs.bigmodel.cn/cn/guide/start/model-overview</x:v>
+        <x:v>https://bigmodel.cn/pricing</x:v>
       </x:c>
       <x:c r="L17" s="91" t="str">
         <x:v>【公开事实】免费模型受配额/稳定性条件限制</x:v>
@@ -2092,16 +2091,16 @@
         <x:v>第一方 API、自建、云平台托管</x:v>
       </x:c>
       <x:c r="I18" s="64" t="str">
-        <x:v>V4 Flash 缓存/未命中/输出约 ¥0.02/¥1/¥2</x:v>
+        <x:v>V4 Flash 非高峰缓存/输入/输出 ¥0.05/¥1.5/¥4.5；高峰 ¥0.1/¥3/¥9</x:v>
       </x:c>
       <x:c r="J18" s="64" t="str">
         <x:v>低成本 Agent、代码、推理、底模蒸馏、私有化</x:v>
       </x:c>
       <x:c r="K18" s="96" t="str">
-        <x:v>https://api-docs.deepseek.com/</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing</x:v>
       </x:c>
       <x:c r="L18" s="91" t="str">
-        <x:v>【公开事实】缓存命中价格极低但不能假设必定命中</x:v>
+        <x:v>【公开事实】峰谷、缓存命中与失败重试会显著改变实际成本</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -2153,7 +2152,7 @@
         <x:v>从多模态和社交/陪伴产品扩展到超长上下文、推理与 Agent Coding，同时保留海螺视频、语音、音乐能力。</x:v>
       </x:c>
       <x:c r="D20" s="64" t="str">
-        <x:v>MiniMax M2.7 / M2.5；Hailuo 2.3；Speech/Music</x:v>
+        <x:v>MiniMax M3 / M2.7；Hailuo 2.3；Speech/Music</x:v>
       </x:c>
       <x:c r="E20" s="64" t="str">
         <x:v>MiniMax Agent、海螺 AI、开放平台、Talkie</x:v>
@@ -2168,7 +2167,7 @@
         <x:v>API、订阅 Token Plan、专属部署</x:v>
       </x:c>
       <x:c r="I20" s="64" t="str">
-        <x:v>M2.7 ¥2.1/¥8.4，缓存读 ¥0.42；视频按条计费</x:v>
+        <x:v>M3 ≤512K ¥2.1/¥8.4，缓存 ¥0.42；&gt;512K ¥4.2/¥16.8</x:v>
       </x:c>
       <x:c r="J20" s="64" t="str">
         <x:v>Agent、代码、Office 交付、视频/语音、角色互动</x:v>
@@ -2177,7 +2176,7 @@
         <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
       </x:c>
       <x:c r="L20" s="91" t="str">
-        <x:v>【公开事实】高速版、订阅与按量不可直接横比</x:v>
+        <x:v>【公开事实】M3 当前为促销价；高速版、订阅与按量不可直接横比</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
@@ -2267,10 +2266,10 @@
         <x:v>从日日新通用模型扩展到多模态、推理与办公交付，结合商汤视觉积累形成视觉 Agent 与内容生产。</x:v>
       </x:c>
       <x:c r="D23" s="64" t="str">
-        <x:v>SenseNova V6.x / Reasoner；多模态与视觉 Agent</x:v>
+        <x:v>SenseNova 6.8 Flash Lite / U1 Fast / U1 Pro；多模态与视觉 Agent</x:v>
       </x:c>
       <x:c r="E23" s="64" t="str">
-        <x:v>商量、办公小浣熊、SenseNova 开放平台</x:v>
+        <x:v>商量、办公小浣熊、SenseNova 开放平台、Token Plan</x:v>
       </x:c>
       <x:c r="F23" s="64" t="str">
         <x:v>视觉、多模态、办公数据分析、PPT/信息图、企业交付</x:v>
@@ -2282,16 +2281,16 @@
         <x:v>API、企业平台、私有化</x:v>
       </x:c>
       <x:c r="I23" s="64" t="str">
-        <x:v>V6 Pro ¥3/¥9；V6 Turbo ¥1.5/¥4.5；Reasoner ¥8/¥32</x:v>
+        <x:v>Token Plan Beta：免费 60,000 credits / 5 小时，最多 20 个 API Key；按量价另核</x:v>
       </x:c>
       <x:c r="J23" s="64" t="str">
         <x:v>办公交付、视觉分析、内容生成、企业 Agent</x:v>
       </x:c>
       <x:c r="K23" s="96" t="str">
-        <x:v>https://platform.sensenova.cn/product/APIService/pricing</x:v>
+        <x:v>https://platform.sensenova.cn/token-plan</x:v>
       </x:c>
       <x:c r="L23" s="91" t="str">
-        <x:v>【公开事实】需区分通用、推理和多模态模型</x:v>
+        <x:v>【公开事实】Beta 免费额度与生产 SLA、长期定价需分开看</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -2414,7 +2413,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77ba52be44d54d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b1a8e201b874d5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2571,19 +2570,19 @@
         <x:v>OpenAI</x:v>
       </x:c>
       <x:c r="C6" s="64" t="str">
-        <x:v>2026-06 / 07</x:v>
+        <x:v>2026-06 / 07 / 09</x:v>
       </x:c>
       <x:c r="D6" s="64" t="str">
-        <x:v>GPT-5.6 Sol / Terra / Luna</x:v>
+        <x:v>GPT-5.6 Sol / Terra / Luna；GPT-6 Astra</x:v>
       </x:c>
       <x:c r="E6" s="64" t="str">
-        <x:v>1.05M 上下文、分层成本、计算机工具与多智能体</x:v>
+        <x:v>1.05M 上下文、分层成本、计算机工具、多智能体与复杂知识工作</x:v>
       </x:c>
       <x:c r="F6" s="64" t="str">
         <x:v>ChatGPT、API、Codex</x:v>
       </x:c>
       <x:c r="G6" s="96" t="str">
-        <x:v>https://openai.com/index/gpt-5-6/</x:v>
+        <x:v>https://openai.com/index/gpt-6-astra/</x:v>
       </x:c>
       <x:c r="H6" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -2675,16 +2674,16 @@
         <x:v>Anthropic</x:v>
       </x:c>
       <x:c r="C10" s="64" t="str">
-        <x:v>2026-06 / 07</x:v>
+        <x:v>2026-06 / 07 / 09</x:v>
       </x:c>
       <x:c r="D10" s="64" t="str">
-        <x:v>Claude Sonnet 5 / Opus 5 / Fable 5</x:v>
+        <x:v>Claude Sonnet 5 / Opus 5 / Fable 5.1</x:v>
       </x:c>
       <x:c r="E10" s="64" t="str">
-        <x:v>1M 上下文、128K 输出、默认思考、长任务</x:v>
+        <x:v>1M 上下文、128K 输出、默认思考与长周期 Agent</x:v>
       </x:c>
       <x:c r="F10" s="64" t="str">
-        <x:v>Claude Platform、Managed Agents</x:v>
+        <x:v>Claude、Claude Code、Claude Platform</x:v>
       </x:c>
       <x:c r="G10" s="96" t="str">
         <x:v>https://platform.claude.com/docs/en/release-notes/overview</x:v>
@@ -2779,19 +2778,19 @@
         <x:v>Google DeepMind</x:v>
       </x:c>
       <x:c r="C14" s="64" t="str">
-        <x:v>2026-08</x:v>
+        <x:v>2026-08 / 09</x:v>
       </x:c>
       <x:c r="D14" s="64" t="str">
-        <x:v>Gemini 3.7 Flash；3.5 Flash-Lite</x:v>
+        <x:v>Gemini 3.7 / 3.8 Flash；3.5 Flash-Lite；Lyria 3.5</x:v>
       </x:c>
       <x:c r="E14" s="64" t="str">
-        <x:v>Agent/代码增强；低成本高吞吐与多模态输入</x:v>
+        <x:v>Agent/代码增强、低成本高吞吐、多模态与音乐生成</x:v>
       </x:c>
       <x:c r="F14" s="64" t="str">
         <x:v>Gemini API、AI Studio、Vertex AI</x:v>
       </x:c>
       <x:c r="G14" s="96" t="str">
-        <x:v>https://ai.google.dev/gemini-api/docs/latest-model</x:v>
+        <x:v>https://ai.google.dev/gemini-api/docs/changelog</x:v>
       </x:c>
       <x:c r="H14" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -2883,19 +2882,19 @@
         <x:v>Meta</x:v>
       </x:c>
       <x:c r="C18" s="64" t="str">
-        <x:v>2026-04</x:v>
+        <x:v>2026-04 / 09</x:v>
       </x:c>
       <x:c r="D18" s="64" t="str">
-        <x:v>Muse Spark</x:v>
+        <x:v>Muse Spark 1.3；Muse Voice；Muse Image</x:v>
       </x:c>
       <x:c r="E18" s="64" t="str">
-        <x:v>原生多模态推理、工具使用与多智能体编排</x:v>
+        <x:v>原生多模态推理、语音、图像、工具与第一方 Model API</x:v>
       </x:c>
       <x:c r="F18" s="64" t="str">
-        <x:v>Meta AI</x:v>
+        <x:v>Meta AI、Model API</x:v>
       </x:c>
       <x:c r="G18" s="96" t="str">
-        <x:v>https://ai.meta.com/blog/introducing-model-meta-superintelligence-labs/</x:v>
+        <x:v>https://developer.meta.com/ai</x:v>
       </x:c>
       <x:c r="H18" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -2987,19 +2986,19 @@
         <x:v>xAI / SpaceXAI</x:v>
       </x:c>
       <x:c r="C22" s="64" t="str">
-        <x:v>2026-07 / 08</x:v>
+        <x:v>2026-07 / 08 / 09</x:v>
       </x:c>
       <x:c r="D22" s="64" t="str">
-        <x:v>Grok 4.5 / 4.6；Voice 2.0</x:v>
+        <x:v>Grok 4.5 / 4.6；Voice 2.0；Imagine</x:v>
       </x:c>
       <x:c r="E22" s="64" t="str">
-        <x:v>代码 Agent、500K、多模态输入、语音客服与创作</x:v>
+        <x:v>代码 Agent、500K、多模态、语音客服；旧图像质量端点进入退役期</x:v>
       </x:c>
       <x:c r="F22" s="64" t="str">
         <x:v>Grok Build、API、Voice、Imagine</x:v>
       </x:c>
       <x:c r="G22" s="96" t="str">
-        <x:v>https://docs.x.ai/developers/grok-4-6</x:v>
+        <x:v>https://docs.x.ai/developers/release-notes</x:v>
       </x:c>
       <x:c r="H22" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -3091,19 +3090,19 @@
         <x:v>Mistral AI</x:v>
       </x:c>
       <x:c r="C26" s="64" t="str">
-        <x:v>2026-03 / 04 / 06</x:v>
+        <x:v>2026-03 / 04 / 06 / 09</x:v>
       </x:c>
       <x:c r="D26" s="64" t="str">
-        <x:v>Small 4；Medium 3.5；OCR 4</x:v>
+        <x:v>Small 4；Medium 3.5；OCR 4.1</x:v>
       </x:c>
       <x:c r="E26" s="64" t="str">
-        <x:v>统一 instruct/reasoning/coding；文档结构理解</x:v>
+        <x:v>统一 instruct/reasoning/coding；OCR 结构理解；Leanstral 1.5 进入退役期</x:v>
       </x:c>
       <x:c r="F26" s="64" t="str">
         <x:v>Le Chat、Vibe、Studio、Forge</x:v>
       </x:c>
       <x:c r="G26" s="96" t="str">
-        <x:v>https://docs.mistral.ai/inference/pricing</x:v>
+        <x:v>https://docs.mistral.ai/getting-started/changelog/</x:v>
       </x:c>
       <x:c r="H26" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -3299,19 +3298,19 @@
         <x:v>Amazon / AWS</x:v>
       </x:c>
       <x:c r="C34" s="64" t="str">
-        <x:v>2026</x:v>
+        <x:v>2026 / 09</x:v>
       </x:c>
       <x:c r="D34" s="64" t="str">
-        <x:v>Nova Forge / 自定义模型推理增强</x:v>
+        <x:v>Nova Forge；Claude Fable 5.1 on Bedrock</x:v>
       </x:c>
       <x:c r="E34" s="64" t="str">
-        <x:v>客户可定制训练并在 Bedrock/SageMaker 托管</x:v>
+        <x:v>自定义模型训练/托管，并扩充第三方长周期 Agent 旗舰</x:v>
       </x:c>
       <x:c r="F34" s="64" t="str">
         <x:v>Bedrock、SageMaker</x:v>
       </x:c>
       <x:c r="G34" s="96" t="str">
-        <x:v>https://docs.aws.amazon.com/nova/latest/nova2-userguide/what-is-nova-2.html</x:v>
+        <x:v>https://aws.amazon.com/about-aws/whats-new/2026/09/claude-fable-5-1-aws/</x:v>
       </x:c>
       <x:c r="H34" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -3403,19 +3402,19 @@
         <x:v>Microsoft（Phi/MAI）</x:v>
       </x:c>
       <x:c r="C38" s="64" t="str">
-        <x:v>2026-03</x:v>
+        <x:v>2026-03 / 09</x:v>
       </x:c>
       <x:c r="D38" s="64" t="str">
-        <x:v>Phi-4 Reasoning Vision 15B</x:v>
+        <x:v>Phi-4 Reasoning Vision；MAI-Transcribe-2；GPT-6 Astra on Foundry</x:v>
       </x:c>
       <x:c r="E38" s="64" t="str">
-        <x:v>开放权重的视觉、数学、科学和 UI 理解</x:v>
+        <x:v>视觉推理、语音转写与 Azure 前沿模型托管</x:v>
       </x:c>
       <x:c r="F38" s="64" t="str">
-        <x:v>本地、Azure、研究生态</x:v>
+        <x:v>本地、Azure AI Foundry、Copilot</x:v>
       </x:c>
       <x:c r="G38" s="96" t="str">
-        <x:v>https://www.microsoft.com/en-us/research/wp-content/uploads/2026/03/Phi-4-reasoning-vision-15B-Tech-Report.pdf</x:v>
+        <x:v>https://microsoft.ai/news/introducing-mai-transcribe-2/</x:v>
       </x:c>
       <x:c r="H38" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -3611,16 +3610,16 @@
         <x:v>阿里云 / 通义千问 Qwen</x:v>
       </x:c>
       <x:c r="C46" s="64" t="str">
-        <x:v>2026</x:v>
+        <x:v>2026 / 09</x:v>
       </x:c>
       <x:c r="D46" s="64" t="str">
-        <x:v>Qwen3.5 → Qwen3.8-Max</x:v>
+        <x:v>Qwen3.5 → Qwen3.8-Max / Prime</x:v>
       </x:c>
       <x:c r="E46" s="64" t="str">
-        <x:v>原生多模态、1M 上下文、长任务 Agent</x:v>
+        <x:v>长上下文、Agent 与旗舰/Prime 服务分层</x:v>
       </x:c>
       <x:c r="F46" s="64" t="str">
-        <x:v>QwenWork、百炼</x:v>
+        <x:v>千问、百炼、QwenWork</x:v>
       </x:c>
       <x:c r="G46" s="96" t="str">
         <x:v>https://www.alibabacloud.com/en/press-room/alibaba-unveils-qwen3-8-max</x:v>
@@ -3715,16 +3714,16 @@
         <x:v>百度 / 文心 ERNIE</x:v>
       </x:c>
       <x:c r="C50" s="64" t="str">
-        <x:v>2026-01 / 07</x:v>
+        <x:v>2026-01 / 07 / 09</x:v>
       </x:c>
       <x:c r="D50" s="64" t="str">
         <x:v>ERNIE 5.0 / 5.1</x:v>
       </x:c>
       <x:c r="E50" s="64" t="str">
-        <x:v>统一全模态、Agent、事实性与长任务</x:v>
+        <x:v>统一全模态、Agent 与上下文阶梯计价</x:v>
       </x:c>
       <x:c r="F50" s="64" t="str">
-        <x:v>千帆、百度搜索/文库</x:v>
+        <x:v>文小言、搜索、千帆</x:v>
       </x:c>
       <x:c r="G50" s="96" t="str">
         <x:v>https://cloud.baidu.cn/news/news_eacd5e1a-b6ad-4874-b920-15390d26e656</x:v>
@@ -3923,19 +3922,19 @@
         <x:v>腾讯 / 混元 Hy</x:v>
       </x:c>
       <x:c r="C58" s="64" t="str">
-        <x:v>2026</x:v>
+        <x:v>2026 / 09</x:v>
       </x:c>
       <x:c r="D58" s="64" t="str">
-        <x:v>Hy3</x:v>
+        <x:v>Hy3；Hy4 Preview</x:v>
       </x:c>
       <x:c r="E58" s="64" t="str">
-        <x:v>256K、混合思考与 Agent，迁移至 TokenHub</x:v>
+        <x:v>企业 Agent、办公/代码产品集成与新一代预览模型</x:v>
       </x:c>
       <x:c r="F58" s="64" t="str">
-        <x:v>WorkBuddy、CodeBuddy、元宝、TokenHub</x:v>
+        <x:v>元宝、ima、CodeBuddy、WorkBuddy、TokenHub</x:v>
       </x:c>
       <x:c r="G58" s="96" t="str">
-        <x:v>https://www.tencent.com/zh-cn/tencent-hunyuan-officially-releases-hy3-advancing-agent-capabilities-and-deeper-product-integration/</x:v>
+        <x:v>https://cloud.tencent.com/product/tokenhub</x:v>
       </x:c>
       <x:c r="H58" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -4027,19 +4026,19 @@
         <x:v>智谱 AI / GLM</x:v>
       </x:c>
       <x:c r="C62" s="64" t="str">
-        <x:v>2026</x:v>
+        <x:v>2026 / 09</x:v>
       </x:c>
       <x:c r="D62" s="64" t="str">
-        <x:v>GLM-5 / 5.1 / 5.2；GLM-5V-Turbo</x:v>
+        <x:v>GLM-5 / 5.1 / 5.2 / 5.3；GLM-5V-Turbo</x:v>
       </x:c>
       <x:c r="E62" s="64" t="str">
-        <x:v>长周期工程 Agent、1M 上下文、视觉行动</x:v>
+        <x:v>代码、1M 上下文、长周期 Agent、视觉操作与成本分层</x:v>
       </x:c>
       <x:c r="F62" s="64" t="str">
-        <x:v>Coding Plan、BigModel</x:v>
+        <x:v>清言、AutoGLM、BigModel</x:v>
       </x:c>
       <x:c r="G62" s="96" t="str">
-        <x:v>https://docs.bigmodel.cn/cn/guide/models/text/glm-5.2</x:v>
+        <x:v>https://bigmodel.cn/pricing</x:v>
       </x:c>
       <x:c r="H62" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -4339,19 +4338,19 @@
         <x:v>MiniMax</x:v>
       </x:c>
       <x:c r="C74" s="64" t="str">
-        <x:v>2026</x:v>
+        <x:v>2026-02 / 05 / 09</x:v>
       </x:c>
       <x:c r="D74" s="64" t="str">
-        <x:v>M2.5 / M2.7；Hailuo 2.3</x:v>
+        <x:v>M2.5 / M2.7 / M3；Hailuo 2.3</x:v>
       </x:c>
       <x:c r="E74" s="64" t="str">
-        <x:v>代码 Agent、Office Skills、视频和语音</x:v>
+        <x:v>Agent Coding、Office Skills、超长上下文与多模态内容生成</x:v>
       </x:c>
       <x:c r="F74" s="64" t="str">
-        <x:v>MiniMax Agent、海螺、API</x:v>
+        <x:v>MiniMax Agent、开放平台、海螺</x:v>
       </x:c>
       <x:c r="G74" s="96" t="str">
-        <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
+        <x:v>https://www.minimax.io/news/minimax-m3</x:v>
       </x:c>
       <x:c r="H74" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -4651,19 +4650,19 @@
         <x:v>商汤 / 日日新 SenseNova</x:v>
       </x:c>
       <x:c r="C86" s="64" t="str">
-        <x:v>2026</x:v>
+        <x:v>2026 / 09</x:v>
       </x:c>
       <x:c r="D86" s="64" t="str">
-        <x:v>U1 Pro / 6.8 Flash Lite</x:v>
+        <x:v>U1 Pro / U1 Fast；6.8 Flash Lite</x:v>
       </x:c>
       <x:c r="E86" s="64" t="str">
-        <x:v>视觉 Agent、低延迟与多模态任务</x:v>
+        <x:v>推理与高吞吐双档；Token Plan Beta 开放开发者额度</x:v>
       </x:c>
       <x:c r="F86" s="64" t="str">
-        <x:v>SenseNova API、企业产品</x:v>
+        <x:v>SenseNova 平台、商量、办公小浣熊</x:v>
       </x:c>
       <x:c r="G86" s="96" t="str">
-        <x:v>https://www.sensetime.com/cn/news/sensenova-6.8-flash-lite-preview</x:v>
+        <x:v>https://platform.sensenova.cn/token-plan</x:v>
       </x:c>
       <x:c r="H86" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -4987,7 +4986,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16697c6b33864a86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc72dfb60c2e458a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5440,10 +5439,10 @@
         <x:v>Google DeepMind</x:v>
       </x:c>
       <x:c r="C10" s="64" t="str">
-        <x:v>Gemini 3.1 Pro</x:v>
+        <x:v>Gemini 3.1 Pro Preview</x:v>
       </x:c>
       <x:c r="D10" s="64" t="str">
-        <x:v>GA</x:v>
+        <x:v>Preview</x:v>
       </x:c>
       <x:c r="E10" s="64" t="str">
         <x:v>USD</x:v>
@@ -5452,23 +5451,23 @@
         <x:v>每百万tokens</x:v>
       </x:c>
       <x:c r="G10" s="102" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H10" s="102" t="n">
-        <x:v>0.15</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="I10" s="102"/>
       <x:c r="J10" s="102" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="K10" s="64" t="str">
-        <x:v>短上下文标准档</x:v>
+        <x:v>≤200K；更长上下文另行计价</x:v>
       </x:c>
       <x:c r="L10" s="64" t="str">
         <x:v>输出含 thinking tokens</x:v>
       </x:c>
       <x:c r="M10" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="N10" s="96" t="str">
         <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
@@ -5758,7 +5757,7 @@
         <x:v>Command A+</x:v>
       </x:c>
       <x:c r="D17" s="64" t="str">
-        <x:v>GA</x:v>
+        <x:v>GA/免费限速</x:v>
       </x:c>
       <x:c r="E17" s="64" t="str">
         <x:v>USD</x:v>
@@ -5767,24 +5766,24 @@
         <x:v>每百万tokens</x:v>
       </x:c>
       <x:c r="G17" s="102" t="n">
-        <x:v>2.5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H17" s="102"/>
       <x:c r="I17" s="102"/>
       <x:c r="J17" s="102" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K17" s="64" t="str">
-        <x:v>以实时模型页为准</x:v>
+        <x:v>自助 API 免费至触发限速</x:v>
       </x:c>
       <x:c r="L17" s="64" t="str">
-        <x:v>私有 Vault 另按实例计费</x:v>
+        <x:v>生产私有 Vault 按实例/承诺计费</x:v>
       </x:c>
       <x:c r="M17" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="N17" s="96" t="str">
-        <x:v>https://docs.cohere.com/docs/command-a</x:v>
+        <x:v>https://docs.cohere.com/docs/command-a-plus</x:v>
       </x:c>
       <x:c r="O17" s="91" t="str">
         <x:v>官方模型页</x:v>
@@ -5907,10 +5906,10 @@
         <x:v>中国内地/≤1M</x:v>
       </x:c>
       <x:c r="L20" s="64" t="str">
-        <x:v>区域与活动价不同</x:v>
+        <x:v>Prime 档为 ¥24/¥72；区域与活动价不同</x:v>
       </x:c>
       <x:c r="M20" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="N20" s="96" t="str">
         <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
@@ -5990,13 +5989,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="K22" s="64" t="str">
-        <x:v>32K-128K 为 ¥6/¥22</x:v>
+        <x:v>32K—128K 为 ¥6/¥22</x:v>
       </x:c>
       <x:c r="L22" s="64" t="str">
         <x:v>按输入长度阶梯</x:v>
       </x:c>
       <x:c r="M22" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="N22" s="96" t="str">
         <x:v>https://cloud.baidu.com/doc/qianfan/s/wmh4sv6ya</x:v>
@@ -6385,26 +6384,26 @@
         <x:v>每百万tokens</x:v>
       </x:c>
       <x:c r="G31" s="102" t="n">
-        <x:v>1</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="H31" s="102" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.05</x:v>
       </x:c>
       <x:c r="I31" s="102"/>
       <x:c r="J31" s="102" t="n">
-        <x:v>2</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="K31" s="64" t="str">
-        <x:v>1M；思考/非思考双模式</x:v>
+        <x:v>1M；非高峰价</x:v>
       </x:c>
       <x:c r="L31" s="64" t="str">
-        <x:v>官方美元价折算约等于该人民币价</x:v>
+        <x:v>高峰缓存/输入/输出为 ¥0.1/¥3/¥9</x:v>
       </x:c>
       <x:c r="M31" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="N31" s="96" t="str">
-        <x:v>https://api-docs.deepseek.com/quick_start/pricing</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing</x:v>
       </x:c>
       <x:c r="O31" s="91" t="str">
         <x:v>官方价格页</x:v>
@@ -7072,6 +7071,368 @@
         <x:v>https://platform.baichuan-ai.com/prices</x:v>
       </x:c>
       <x:c r="O46" s="94" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="54" customHeight="1">
+      <x:c r="A47" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>GPT-6 Astra</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G47" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I47" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="J47" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>1.05M；&gt;272K 整次请求输入/缓存 2×、输出 1.5×</x:v>
+      </x:c>
+      <x:c r="L47" t="str">
+        <x:v>Batch/Flex 5 折；Fast 2×</x:v>
+      </x:c>
+      <x:c r="M47" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N47" t="str">
+        <x:v>https://developers.openai.com/api/docs/models/gpt-6-astra</x:v>
+      </x:c>
+      <x:c r="O47" t="str">
+        <x:v>官方模型与价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="54" customHeight="1">
+      <x:c r="A48" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>Anthropic</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Claude Fable 5.1</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G48" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H48" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="I48" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="J48" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="K48" t="str">
+        <x:v>1M 上下文；128K 最大输出</x:v>
+      </x:c>
+      <x:c r="L48" t="str">
+        <x:v>1h 缓存写入 $20；Batch 输入输出 5 折</x:v>
+      </x:c>
+      <x:c r="M48" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N48" t="str">
+        <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
+      </x:c>
+      <x:c r="O48" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="54" customHeight="1">
+      <x:c r="A49" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>Google DeepMind</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Gemini 3.8 Flash</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>GA/促销</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G49" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="H49" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="I49"/>
+      <x:c r="J49" t="n">
+        <x:v>3.75</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>促销至 2026-12-31</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>2027-01-01 起 $1.5/$0.15/$7.5</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
+      </x:c>
+      <x:c r="O49" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="54" customHeight="1">
+      <x:c r="A50" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>腾讯 / 混元 Hy</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Hy4 Preview</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Preview</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G50" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H50" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="I50"/>
+      <x:c r="J50" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>TokenHub 预览档</x:v>
+      </x:c>
+      <x:c r="L50" t="str">
+        <x:v>预览期可用性、配额与稳定性需验证</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N50" t="str">
+        <x:v>https://cloud.tencent.com/document/product/1823/130055</x:v>
+      </x:c>
+      <x:c r="O50" t="str">
+        <x:v>TokenHub 价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="54" customHeight="1">
+      <x:c r="A51" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>智谱 AI / GLM</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>GLM-5.3</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G51" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H51" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I51"/>
+      <x:c r="J51" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>平台标准档</x:v>
+      </x:c>
+      <x:c r="L51" t="str">
+        <x:v>缓存存储与套餐规则另核</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>https://bigmodel.cn/pricing</x:v>
+      </x:c>
+      <x:c r="O51" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="54" customHeight="1">
+      <x:c r="A52" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>MiniMax</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>MiniMax M3 ≤512K</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>GA/促销</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G52" t="n">
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="H52" t="n">
+        <x:v>0.42</x:v>
+      </x:c>
+      <x:c r="I52"/>
+      <x:c r="J52" t="n">
+        <x:v>8.4</x:v>
+      </x:c>
+      <x:c r="K52" t="str">
+        <x:v>输入 ≤512K</x:v>
+      </x:c>
+      <x:c r="L52" t="str">
+        <x:v>促销价；高速版与 Token Plan 另计</x:v>
+      </x:c>
+      <x:c r="M52" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N52" t="str">
+        <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
+      </x:c>
+      <x:c r="O52" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="54" customHeight="1">
+      <x:c r="A53" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>百度 / 文心 ERNIE</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>ERNIE 5.1 32K—128K</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G53" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H53"/>
+      <x:c r="I53"/>
+      <x:c r="J53" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="K53" t="str">
+        <x:v>输入 32K—128K</x:v>
+      </x:c>
+      <x:c r="L53" t="str">
+        <x:v>按整次请求输入长度进入阶梯</x:v>
+      </x:c>
+      <x:c r="M53" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N53" t="str">
+        <x:v>https://cloud.baidu.com/doc/qianfan/s/wmh4sv6ya</x:v>
+      </x:c>
+      <x:c r="O53" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="54" customHeight="1">
+      <x:c r="A54" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>MiniMax</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>MiniMax M3 &gt;512K</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>GA/促销</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G54" t="n">
+        <x:v>4.2</x:v>
+      </x:c>
+      <x:c r="H54" t="n">
+        <x:v>0.84</x:v>
+      </x:c>
+      <x:c r="I54"/>
+      <x:c r="J54" t="n">
+        <x:v>16.8</x:v>
+      </x:c>
+      <x:c r="K54" t="str">
+        <x:v>输入 &gt;512K</x:v>
+      </x:c>
+      <x:c r="L54" t="str">
+        <x:v>促销价；高速版与 Token Plan 另计</x:v>
+      </x:c>
+      <x:c r="M54" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="N54" t="str">
+        <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
+      </x:c>
+      <x:c r="O54" t="str">
         <x:v>官方价格页</x:v>
       </x:c>
     </x:row>
@@ -7081,7 +7442,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf320eca746c94748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raed858df767d44b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7694,38 +8055,38 @@
         <x:v>Google DeepMind</x:v>
       </x:c>
       <x:c r="C17" s="127" t="str">
-        <x:v>Gemini 3.1 Pro</x:v>
+        <x:v>Gemini 3.1 Pro Preview</x:v>
       </x:c>
       <x:c r="D17" s="127" t="str">
         <x:v>USD</x:v>
       </x:c>
       <x:c r="E17" s="128" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F17" s="128" t="n">
-        <x:v>0.15</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="G17" s="128" t="n">
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H17" s="129" t="n">
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="I17" s="130" t="n">
         <x:f>$B$4/1000000*($B$2*((1-$B$5)*E17+$B$5*IF(F17="",E17,F17))+$B$3*G17)*(1-$B$7)</x:f>
-        <x:v>669</x:v>
+        <x:v>892</x:v>
       </x:c>
       <x:c r="J17" s="130" t="n">
         <x:f>IF(D17="USD",I17*$B$6,I17)</x:f>
-        <x:v>4816.8</x:v>
+        <x:v>6422.400000000001</x:v>
       </x:c>
       <x:c r="K17" s="130" t="n">
         <x:f>J17/$B$4*1000</x:f>
-        <x:v>48.168</x:v>
+        <x:v>64.224</x:v>
       </x:c>
       <x:c r="L17" s="130" t="n">
         <x:f>IFERROR(J17/($B$4*H17),"")</x:f>
-        <x:v>0.05666823529411765</x:v>
+        <x:v>0.07555764705882353</x:v>
       </x:c>
       <x:c r="M17" s="127" t="str">
         <x:f>IF(H17&lt;0.7,"先修质量",IF(L17&lt;0.01,"极低成本",IF(L17&lt;0.1,"低成本","需看价值")))</x:f>
@@ -8050,34 +8411,34 @@
         <x:v>USD</x:v>
       </x:c>
       <x:c r="E24" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F24" s="128"/>
       <x:c r="G24" s="128" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H24" s="129" t="n">
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="I24" s="130" t="n">
         <x:f>$B$4/1000000*($B$2*((1-$B$5)*E24+$B$5*IF(F24="",E24,F24))+$B$3*G24)*(1-$B$7)</x:f>
-        <x:v>1000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J24" s="130" t="n">
         <x:f>IF(D24="USD",I24*$B$6,I24)</x:f>
-        <x:v>7200</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K24" s="130" t="n">
         <x:f>J24/$B$4*1000</x:f>
-        <x:v>72</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L24" s="130" t="n">
         <x:f>IFERROR(J24/($B$4*H24),"")</x:f>
-        <x:v>0.08470588235294117</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M24" s="127" t="str">
         <x:f>IF(H24&lt;0.7,"先修质量",IF(L24&lt;0.01,"极低成本",IF(L24&lt;0.1,"低成本","需看价值")))</x:f>
-        <x:v>低成本</x:v>
+        <x:v>极低成本</x:v>
       </x:c>
       <x:c r="N24" s="134" t="str">
         <x:v>https://docs.cohere.com/docs/command-a</x:v>
@@ -8640,32 +9001,32 @@
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="E36" s="128" t="n">
-        <x:v>1</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="F36" s="128" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.05</x:v>
       </x:c>
       <x:c r="G36" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="H36" s="129" t="n">
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="I36" s="130" t="n">
         <x:f>$B$4/1000000*($B$2*((1-$B$5)*E36+$B$5*IF(F36="",E36,F36))+$B$3*G36)*(1-$B$7)</x:f>
-        <x:v>241.20000000000002</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="J36" s="130" t="n">
         <x:f>IF(D36="USD",I36*$B$6,I36)</x:f>
-        <x:v>241.20000000000002</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="K36" s="130" t="n">
         <x:f>J36/$B$4*1000</x:f>
-        <x:v>2.412</x:v>
+        <x:v>4.38</x:v>
       </x:c>
       <x:c r="L36" s="130" t="n">
         <x:f>IFERROR(J36/($B$4*H36),"")</x:f>
-        <x:v>0.00283764705882353</x:v>
+        <x:v>0.0051529411764705884</x:v>
       </x:c>
       <x:c r="M36" s="127" t="str">
         <x:f>IF(H36&lt;0.7,"先修质量",IF(L36&lt;0.01,"极低成本",IF(L36&lt;0.1,"低成本","需看价值")))</x:f>
@@ -9411,6 +9772,364 @@
         <x:v>https://platform.baichuan-ai.com/prices</x:v>
       </x:c>
       <x:c r="O51" s="127"/>
+    </x:row>
+    <x:row r="52" ht="40" customHeight="1">
+      <x:c r="A52" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>GPT-6 Astra</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E52" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F52" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G52" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H52" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I52" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E52+$B$5*IF(F52="",E52,F52))+$B$3*G52)*(1-$B$7)</x:f>
+        <x:v>3960</x:v>
+      </x:c>
+      <x:c r="J52" t="n">
+        <x:f>IF(D52="USD",I52*$B$6,I52)</x:f>
+        <x:v>28512</x:v>
+      </x:c>
+      <x:c r="K52" t="n">
+        <x:f>J52/$B$4*1000</x:f>
+        <x:v>285.12</x:v>
+      </x:c>
+      <x:c r="L52" t="n">
+        <x:f>IFERROR(J52/($B$4*H52),"")</x:f>
+        <x:v>0.33543529411764705</x:v>
+      </x:c>
+      <x:c r="M52"/>
+      <x:c r="N52"/>
+      <x:c r="O52"/>
+    </x:row>
+    <x:row r="53" ht="40" customHeight="1">
+      <x:c r="A53" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>Anthropic</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>Claude Fable 5.1</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E53" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F53" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="G53" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="H53" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I53" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E53+$B$5*IF(F53="",E53,F53))+$B$3*G53)*(1-$B$7)</x:f>
+        <x:v>3915</x:v>
+      </x:c>
+      <x:c r="J53" t="n">
+        <x:f>IF(D53="USD",I53*$B$6,I53)</x:f>
+        <x:v>28188</x:v>
+      </x:c>
+      <x:c r="K53" t="n">
+        <x:f>J53/$B$4*1000</x:f>
+        <x:v>281.88</x:v>
+      </x:c>
+      <x:c r="L53" t="n">
+        <x:f>IFERROR(J53/($B$4*H53),"")</x:f>
+        <x:v>0.3316235294117647</x:v>
+      </x:c>
+      <x:c r="M53"/>
+      <x:c r="N53"/>
+      <x:c r="O53"/>
+    </x:row>
+    <x:row r="54" ht="40" customHeight="1">
+      <x:c r="A54" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>Google DeepMind</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>Gemini 3.8 Flash</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E54" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="F54" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="G54" t="n">
+        <x:v>3.75</x:v>
+      </x:c>
+      <x:c r="H54" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I54" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E54+$B$5*IF(F54="",E54,F54))+$B$3*G54)*(1-$B$7)</x:f>
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="J54" t="n">
+        <x:f>IF(D54="USD",I54*$B$6,I54)</x:f>
+        <x:v>2138.4</x:v>
+      </x:c>
+      <x:c r="K54" t="n">
+        <x:f>J54/$B$4*1000</x:f>
+        <x:v>21.384</x:v>
+      </x:c>
+      <x:c r="L54" t="n">
+        <x:f>IFERROR(J54/($B$4*H54),"")</x:f>
+        <x:v>0.02515764705882353</x:v>
+      </x:c>
+      <x:c r="M54"/>
+      <x:c r="N54"/>
+      <x:c r="O54"/>
+    </x:row>
+    <x:row r="55" ht="40" customHeight="1">
+      <x:c r="A55" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>腾讯 / 混元 Hy</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>Hy4 Preview</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E55" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F55" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="G55" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H55" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I55" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E55+$B$5*IF(F55="",E55,F55))+$B$3*G55)*(1-$B$7)</x:f>
+        <x:v>1758</x:v>
+      </x:c>
+      <x:c r="J55" t="n">
+        <x:f>IF(D55="USD",I55*$B$6,I55)</x:f>
+        <x:v>1758</x:v>
+      </x:c>
+      <x:c r="K55" t="n">
+        <x:f>J55/$B$4*1000</x:f>
+        <x:v>17.58</x:v>
+      </x:c>
+      <x:c r="L55" t="n">
+        <x:f>IFERROR(J55/($B$4*H55),"")</x:f>
+        <x:v>0.02068235294117647</x:v>
+      </x:c>
+      <x:c r="M55"/>
+      <x:c r="N55"/>
+      <x:c r="O55"/>
+    </x:row>
+    <x:row r="56" ht="40" customHeight="1">
+      <x:c r="A56" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>智谱 AI / GLM</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>GLM-5.3</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E56" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F56" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G56" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H56" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I56" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E56+$B$5*IF(F56="",E56,F56))+$B$3*G56)*(1-$B$7)</x:f>
+        <x:v>2640</x:v>
+      </x:c>
+      <x:c r="J56" t="n">
+        <x:f>IF(D56="USD",I56*$B$6,I56)</x:f>
+        <x:v>2640</x:v>
+      </x:c>
+      <x:c r="K56" t="n">
+        <x:f>J56/$B$4*1000</x:f>
+        <x:v>26.4</x:v>
+      </x:c>
+      <x:c r="L56" t="n">
+        <x:f>IFERROR(J56/($B$4*H56),"")</x:f>
+        <x:v>0.031058823529411764</x:v>
+      </x:c>
+      <x:c r="M56"/>
+      <x:c r="N56"/>
+      <x:c r="O56"/>
+    </x:row>
+    <x:row r="57" ht="40" customHeight="1">
+      <x:c r="A57" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>MiniMax</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>MiniMax M3 ≤512K</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E57" t="n">
+        <x:v>2.1</x:v>
+      </x:c>
+      <x:c r="F57" t="n">
+        <x:v>0.42</x:v>
+      </x:c>
+      <x:c r="G57" t="n">
+        <x:v>8.4</x:v>
+      </x:c>
+      <x:c r="H57" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I57" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E57+$B$5*IF(F57="",E57,F57))+$B$3*G57)*(1-$B$7)</x:f>
+        <x:v>739.2</x:v>
+      </x:c>
+      <x:c r="J57" t="n">
+        <x:f>IF(D57="USD",I57*$B$6,I57)</x:f>
+        <x:v>739.2</x:v>
+      </x:c>
+      <x:c r="K57" t="n">
+        <x:f>J57/$B$4*1000</x:f>
+        <x:v>7.392</x:v>
+      </x:c>
+      <x:c r="L57" t="n">
+        <x:f>IFERROR(J57/($B$4*H57),"")</x:f>
+        <x:v>0.008696470588235295</x:v>
+      </x:c>
+      <x:c r="M57"/>
+      <x:c r="N57"/>
+      <x:c r="O57"/>
+    </x:row>
+    <x:row r="58" ht="40" customHeight="1">
+      <x:c r="A58" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>百度 / 文心 ERNIE</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>ERNIE 5.1 32K—128K</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E58" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F58"/>
+      <x:c r="G58" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H58" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I58" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E58+$B$5*IF(F58="",E58,F58))+$B$3*G58)*(1-$B$7)</x:f>
+        <x:v>2300</x:v>
+      </x:c>
+      <x:c r="J58" t="n">
+        <x:f>IF(D58="USD",I58*$B$6,I58)</x:f>
+        <x:v>2300</x:v>
+      </x:c>
+      <x:c r="K58" t="n">
+        <x:f>J58/$B$4*1000</x:f>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L58" t="n">
+        <x:f>IFERROR(J58/($B$4*H58),"")</x:f>
+        <x:v>0.027058823529411764</x:v>
+      </x:c>
+      <x:c r="M58"/>
+      <x:c r="N58"/>
+      <x:c r="O58"/>
+    </x:row>
+    <x:row r="59" ht="40" customHeight="1">
+      <x:c r="A59" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>MiniMax</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>MiniMax M3 &gt;512K</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E59" t="n">
+        <x:v>4.2</x:v>
+      </x:c>
+      <x:c r="F59" t="n">
+        <x:v>0.84</x:v>
+      </x:c>
+      <x:c r="G59" t="n">
+        <x:v>16.8</x:v>
+      </x:c>
+      <x:c r="H59" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I59" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E59+$B$5*IF(F59="",E59,F59))+$B$3*G59)*(1-$B$7)</x:f>
+        <x:v>1478.4</x:v>
+      </x:c>
+      <x:c r="J59" t="n">
+        <x:f>IF(D59="USD",I59*$B$6,I59)</x:f>
+        <x:v>1478.4</x:v>
+      </x:c>
+      <x:c r="K59" t="n">
+        <x:f>J59/$B$4*1000</x:f>
+        <x:v>14.784</x:v>
+      </x:c>
+      <x:c r="L59" t="n">
+        <x:f>IFERROR(J59/($B$4*H59),"")</x:f>
+        <x:v>0.01739294117647059</x:v>
+      </x:c>
+      <x:c r="M59"/>
+      <x:c r="N59"/>
+      <x:c r="O59"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -9424,7 +10143,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1348b28f123a42f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6abdd04caea4a9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9698,7 +10417,7 @@
         <x:v>2024-2025</x:v>
       </x:c>
       <x:c r="J8" s="136" t="str">
-        <x:v>https://www.anthropic.com/customers/palo-alto-networks</x:v>
+        <x:v>https://www.claude.com/customers/palo-alto-networks</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -10315,7 +11034,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5f31d9f08764417"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re20631e52f9b49b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10394,7 +11113,7 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="C3" s="88" t="str">
-        <x:v>GPT-5.6 Sol；Claude Opus/Fable；GLM-5.2；DeepSeek V4 Pro；Kimi K3</x:v>
+        <x:v>GPT-6 Astra；Claude Fable 5.1 / Opus；GLM-5.3；DeepSeek V4 Pro；Kimi K3</x:v>
       </x:c>
       <x:c r="D3" s="88" t="str">
         <x:v>任务价值高、步骤多、需要电脑/工具/代码执行</x:v>
@@ -10420,7 +11139,7 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="C4" s="64" t="str">
-        <x:v>GPT-5.6 Sol/Terra；Claude Sonnet/Opus；Grok 4.6；Qwen Coder；DeepSeek V4；GLM-5.2；Kimi K2.7 Code</x:v>
+        <x:v>GPT-6 Astra / GPT-5.6；Claude Sonnet/Opus/Fable；Grok 4.6；Qwen Coder；DeepSeek V4；GLM-5.3；Kimi K2.7 Code；MiniMax M3</x:v>
       </x:c>
       <x:c r="D4" s="64" t="str">
         <x:v>代码库级修改、测试、终端与多文件工作</x:v>
@@ -10498,7 +11217,7 @@
         <x:v>中高</x:v>
       </x:c>
       <x:c r="C7" s="64" t="str">
-        <x:v>Claude 5；GPT-5.6；Gemini；Qwen3.8；DeepSeek V4；GLM-5.2；Kimi K3</x:v>
+        <x:v>Claude 5；GPT-6 Astra / GPT-5.6；Gemini；Qwen3.8；DeepSeek V4；GLM-5.3；Kimi K3；MiniMax M3</x:v>
       </x:c>
       <x:c r="D7" s="64" t="str">
         <x:v>代码库、合同包、研究资料、多轮 Agent 历史</x:v>
@@ -10524,7 +11243,7 @@
         <x:v>中高</x:v>
       </x:c>
       <x:c r="C8" s="64" t="str">
-        <x:v>Gemini；GPT-5.6；Claude；Qwen-VL；GLM-5V；ERNIE 5；Seed；Mistral OCR</x:v>
+        <x:v>Gemini；GPT-6 Astra / GPT-5.6；Claude；Qwen-VL；GLM-5V；ERNIE 5；Seed；Mistral OCR 4.1</x:v>
       </x:c>
       <x:c r="D8" s="64" t="str">
         <x:v>图片、PDF、视频、UI、票据和复杂版式</x:v>
@@ -10704,7 +11423,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R702e6df113d844cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R539eb51245714128"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10762,7 +11481,7 @@
         <x:v>时间范围</x:v>
       </x:c>
       <x:c r="B4" s="91" t="str">
-        <x:v>2023-01-01 至 2026-08-24；时间轴保留关键代际和产品变化，不穷尽每个快照、实验版或区域别名。</x:v>
+        <x:v>2023-01-01 至 2026-09-07；时间轴保留关键代际和产品变化，不穷尽每个快照、实验版或区域别名。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -10841,13 +11560,13 @@
         <x:v>OpenAI</x:v>
       </x:c>
       <x:c r="C13" s="88" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>GPT-6 Astra、当前产品与模型入口</x:v>
       </x:c>
       <x:c r="D13" s="95" t="str">
-        <x:v>https://developers.openai.com/api/docs/models</x:v>
+        <x:v>https://developers.openai.com/api/docs/models/gpt-6-astra</x:v>
       </x:c>
       <x:c r="E13" s="88" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F13" s="89" t="str">
         <x:v>【公开事实】当前目录与价格按查询日快照</x:v>
@@ -10861,13 +11580,13 @@
         <x:v>Anthropic</x:v>
       </x:c>
       <x:c r="C14" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Fable 5.1、当前模型与价格</x:v>
       </x:c>
       <x:c r="D14" s="96" t="str">
-        <x:v>https://platform.claude.com/docs/en/home</x:v>
+        <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
       </x:c>
       <x:c r="E14" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F14" s="91" t="str">
         <x:v>【公开事实】注意缓存写入与地域溢价</x:v>
@@ -10881,13 +11600,13 @@
         <x:v>Google DeepMind</x:v>
       </x:c>
       <x:c r="C15" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Gemini 3.8 Flash、Lyria 3.5 与当前价格</x:v>
       </x:c>
       <x:c r="D15" s="96" t="str">
-        <x:v>https://ai.google.dev/gemini-api/docs/models</x:v>
+        <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
       </x:c>
       <x:c r="E15" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F15" s="91" t="str">
         <x:v>【公开事实】搜索/地图 Grounding 另收费</x:v>
@@ -10901,13 +11620,13 @@
         <x:v>Meta</x:v>
       </x:c>
       <x:c r="C16" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Llama、Muse 系列与第一方 Model API</x:v>
       </x:c>
       <x:c r="D16" s="96" t="str">
-        <x:v>https://ai.meta.com/llama/</x:v>
+        <x:v>https://developer.meta.com/ai</x:v>
       </x:c>
       <x:c r="E16" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F16" s="91" t="str">
         <x:v>【公开事实】开放权重不等于零成本</x:v>
@@ -10921,13 +11640,13 @@
         <x:v>xAI / SpaceXAI</x:v>
       </x:c>
       <x:c r="C17" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Grok 模型、价格与退役信息</x:v>
       </x:c>
       <x:c r="D17" s="96" t="str">
-        <x:v>https://docs.x.ai/developers/models/grok-4.6</x:v>
+        <x:v>https://docs.x.ai/developers/release-notes</x:v>
       </x:c>
       <x:c r="E17" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F17" s="91" t="str">
         <x:v>【公开事实】长上下文与工具调用另计</x:v>
@@ -10941,13 +11660,13 @@
         <x:v>Mistral AI</x:v>
       </x:c>
       <x:c r="C18" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>OCR 4.1、模型与生命周期信息</x:v>
       </x:c>
       <x:c r="D18" s="96" t="str">
-        <x:v>https://docs.mistral.ai/models</x:v>
+        <x:v>https://docs.mistral.ai/getting-started/changelog/</x:v>
       </x:c>
       <x:c r="E18" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F18" s="91" t="str">
         <x:v>【公开事实】兼顾 API 与权重部署</x:v>
@@ -10961,13 +11680,13 @@
         <x:v>Cohere</x:v>
       </x:c>
       <x:c r="C19" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Command A+ 与免费限速档</x:v>
       </x:c>
       <x:c r="D19" s="96" t="str">
-        <x:v>https://docs.cohere.com/docs/models</x:v>
+        <x:v>https://docs.cohere.com/docs/command-a-plus</x:v>
       </x:c>
       <x:c r="E19" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F19" s="91" t="str">
         <x:v>【公开事实】适合把生成与检索组件组合评测</x:v>
@@ -10981,13 +11700,13 @@
         <x:v>Amazon / AWS</x:v>
       </x:c>
       <x:c r="C20" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Bedrock 与 Claude Fable 5.1 可用性</x:v>
       </x:c>
       <x:c r="D20" s="96" t="str">
-        <x:v>https://aws.amazon.com/bedrock/</x:v>
+        <x:v>https://aws.amazon.com/about-aws/whats-new/2026/09/claude-fable-5-1-aws/</x:v>
       </x:c>
       <x:c r="E20" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F20" s="91" t="str">
         <x:v>【公开事实】Bedrock 案例常使用第三方底模</x:v>
@@ -11001,13 +11720,13 @@
         <x:v>Microsoft（Phi/MAI）</x:v>
       </x:c>
       <x:c r="C21" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>MAI-Transcribe-2 与 Foundry Astra</x:v>
       </x:c>
       <x:c r="D21" s="96" t="str">
-        <x:v>https://microsoft.ai/news/introducing-mai-1-preview-and-mai-voice-1/</x:v>
+        <x:v>https://microsoft.ai/news/introducing-mai-transcribe-2/</x:v>
       </x:c>
       <x:c r="E21" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F21" s="91" t="str">
         <x:v>【公开事实】MAI 生产 API 价未统一公开</x:v>
@@ -11041,13 +11760,13 @@
         <x:v>阿里云 / 通义千问 Qwen</x:v>
       </x:c>
       <x:c r="C23" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Qwen3.8-Max 与当前价格</x:v>
       </x:c>
       <x:c r="D23" s="96" t="str">
-        <x:v>https://qwenlm.github.io/</x:v>
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
       </x:c>
       <x:c r="E23" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F23" s="91" t="str">
         <x:v>【公开事实】上下文长度会触发阶梯价</x:v>
@@ -11061,13 +11780,13 @@
         <x:v>百度 / 文心 ERNIE</x:v>
       </x:c>
       <x:c r="C24" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>ERNIE 5.1 与上下文阶梯价格</x:v>
       </x:c>
       <x:c r="D24" s="96" t="str">
-        <x:v>https://cloud.baidu.com/product-s/qianfan_home</x:v>
+        <x:v>https://cloud.baidu.com/doc/qianfan/s/wmh4sv6ya</x:v>
       </x:c>
       <x:c r="E24" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F24" s="91" t="str">
         <x:v>【公开事实】千帆还托管第三方模型</x:v>
@@ -11101,13 +11820,13 @@
         <x:v>腾讯 / 混元 Hy</x:v>
       </x:c>
       <x:c r="C26" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>Hy4 Preview、Hy3 与 TokenHub 价格</x:v>
       </x:c>
       <x:c r="D26" s="96" t="str">
-        <x:v>https://cloud.tencent.com/product/tokenhub</x:v>
+        <x:v>https://cloud.tencent.com/document/product/1823/130055</x:v>
       </x:c>
       <x:c r="E26" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F26" s="91" t="str">
         <x:v>【公开事实】原混元售卖入口逐步迁移 TokenHub</x:v>
@@ -11121,13 +11840,13 @@
         <x:v>智谱 AI / GLM</x:v>
       </x:c>
       <x:c r="C27" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>GLM-5.3 与当前价格</x:v>
       </x:c>
       <x:c r="D27" s="96" t="str">
-        <x:v>https://docs.bigmodel.cn/cn/guide/start/model-overview</x:v>
+        <x:v>https://bigmodel.cn/pricing</x:v>
       </x:c>
       <x:c r="E27" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F27" s="91" t="str">
         <x:v>【公开事实】免费模型受配额/稳定性条件限制</x:v>
@@ -11141,13 +11860,13 @@
         <x:v>DeepSeek</x:v>
       </x:c>
       <x:c r="C28" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>DeepSeek V4 峰谷与缓存价格</x:v>
       </x:c>
       <x:c r="D28" s="96" t="str">
-        <x:v>https://api-docs.deepseek.com/</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing</x:v>
       </x:c>
       <x:c r="E28" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F28" s="91" t="str">
         <x:v>【公开事实】缓存命中价格极低但不能假设必定命中</x:v>
@@ -11181,13 +11900,13 @@
         <x:v>MiniMax</x:v>
       </x:c>
       <x:c r="C30" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>MiniMax M3 与上下文阶梯价格</x:v>
       </x:c>
       <x:c r="D30" s="96" t="str">
         <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
       </x:c>
       <x:c r="E30" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F30" s="91" t="str">
         <x:v>【公开事实】高速版、订阅与按量不可直接横比</x:v>
@@ -11221,13 +11940,13 @@
         <x:v>华为云 / 盘古</x:v>
       </x:c>
       <x:c r="C32" s="64" t="str">
-        <x:v>官网、当前产品与模型入口</x:v>
+        <x:v>SenseNova Token Plan 与当前模型</x:v>
       </x:c>
       <x:c r="D32" s="96" t="str">
-        <x:v>https://www.huaweicloud.com/product/pangu.html</x:v>
+        <x:v>https://platform.sensenova.cn/token-plan</x:v>
       </x:c>
       <x:c r="E32" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F32" s="91" t="str">
         <x:v>【公开事实】不宜与公共 API 单价直接比较</x:v>
@@ -11381,13 +12100,13 @@
         <x:v>OpenAI</x:v>
       </x:c>
       <x:c r="C40" s="64" t="str">
-        <x:v>2026-06 / 07 GPT-5.6 Sol / Terra / Luna</x:v>
+        <x:v>2026-06 / 07 / 09 GPT-5.6；GPT-6 Astra</x:v>
       </x:c>
       <x:c r="D40" s="96" t="str">
-        <x:v>https://openai.com/index/gpt-5-6/</x:v>
+        <x:v>https://openai.com/index/gpt-6-astra/</x:v>
       </x:c>
       <x:c r="E40" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F40" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -11461,13 +12180,13 @@
         <x:v>Anthropic</x:v>
       </x:c>
       <x:c r="C44" s="64" t="str">
-        <x:v>2026-06 / 07 Claude Sonnet 5 / Opus 5 / Fable 5</x:v>
+        <x:v>2026-06 / 07 / 09 Claude 5；Fable 5.1</x:v>
       </x:c>
       <x:c r="D44" s="96" t="str">
         <x:v>https://platform.claude.com/docs/en/release-notes/overview</x:v>
       </x:c>
       <x:c r="E44" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F44" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -11521,13 +12240,13 @@
         <x:v>Google DeepMind</x:v>
       </x:c>
       <x:c r="C47" s="64" t="str">
-        <x:v>2026-08 Gemini 3.7 Flash；3.5 Flash-Lite</x:v>
+        <x:v>2026-08 / 09 Gemini 3.7 / 3.8 Flash；Lyria 3.5</x:v>
       </x:c>
       <x:c r="D47" s="96" t="str">
-        <x:v>https://ai.google.dev/gemini-api/docs/latest-model</x:v>
+        <x:v>https://ai.google.dev/gemini-api/docs/changelog</x:v>
       </x:c>
       <x:c r="E47" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F47" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -11601,13 +12320,13 @@
         <x:v>Meta</x:v>
       </x:c>
       <x:c r="C51" s="64" t="str">
-        <x:v>2026-04 Muse Spark</x:v>
+        <x:v>2026 Muse Spark 1.3；Muse Voice；Muse Image</x:v>
       </x:c>
       <x:c r="D51" s="96" t="str">
-        <x:v>https://ai.meta.com/blog/introducing-model-meta-superintelligence-labs/</x:v>
+        <x:v>https://developer.meta.com/ai</x:v>
       </x:c>
       <x:c r="E51" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F51" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -11681,13 +12400,13 @@
         <x:v>xAI / SpaceXAI</x:v>
       </x:c>
       <x:c r="C55" s="64" t="str">
-        <x:v>2026-07 / 08 Grok 4.5 / 4.6；Voice 2.0</x:v>
+        <x:v>2026 Grok 4.5 / 4.6；Voice 2.0；Imagine 退役信息</x:v>
       </x:c>
       <x:c r="D55" s="96" t="str">
-        <x:v>https://docs.x.ai/developers/grok-4-6</x:v>
+        <x:v>https://docs.x.ai/developers/release-notes</x:v>
       </x:c>
       <x:c r="E55" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F55" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -11741,13 +12460,13 @@
         <x:v>Mistral AI</x:v>
       </x:c>
       <x:c r="C58" s="64" t="str">
-        <x:v>2026-03 / 04 / 06 Small 4；Medium 3.5；OCR 4</x:v>
+        <x:v>2026 Small 4；Medium 3.5；OCR 4.1</x:v>
       </x:c>
       <x:c r="D58" s="96" t="str">
-        <x:v>https://docs.mistral.ai/inference/pricing</x:v>
+        <x:v>https://docs.mistral.ai/getting-started/changelog/</x:v>
       </x:c>
       <x:c r="E58" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F58" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -11881,13 +12600,13 @@
         <x:v>Amazon / AWS</x:v>
       </x:c>
       <x:c r="C65" s="64" t="str">
-        <x:v>2026 Nova Forge / 自定义模型推理增强</x:v>
+        <x:v>2026 Nova Forge；Claude Fable 5.1 on Bedrock</x:v>
       </x:c>
       <x:c r="D65" s="96" t="str">
-        <x:v>https://docs.aws.amazon.com/nova/latest/nova2-userguide/what-is-nova-2.html</x:v>
+        <x:v>https://aws.amazon.com/about-aws/whats-new/2026/09/claude-fable-5-1-aws/</x:v>
       </x:c>
       <x:c r="E65" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F65" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -11941,13 +12660,13 @@
         <x:v>Microsoft（Phi/MAI）</x:v>
       </x:c>
       <x:c r="C68" s="64" t="str">
-        <x:v>2026-03 Phi-4 Reasoning Vision 15B</x:v>
+        <x:v>2026 Phi-4 Reasoning Vision；MAI-Transcribe-2；Astra</x:v>
       </x:c>
       <x:c r="D68" s="96" t="str">
-        <x:v>https://www.microsoft.com/en-us/research/wp-content/uploads/2026/03/Phi-4-reasoning-vision-15B-Tech-Report.pdf</x:v>
+        <x:v>https://microsoft.ai/news/introducing-mai-transcribe-2/</x:v>
       </x:c>
       <x:c r="E68" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F68" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -12101,13 +12820,13 @@
         <x:v>阿里云 / 通义千问 Qwen</x:v>
       </x:c>
       <x:c r="C76" s="64" t="str">
-        <x:v>2026 Qwen3.5 → Qwen3.8-Max</x:v>
+        <x:v>2026 Qwen3.5 → Qwen3.8-Max / Prime</x:v>
       </x:c>
       <x:c r="D76" s="96" t="str">
         <x:v>https://www.alibabacloud.com/en/press-room/alibaba-unveils-qwen3-8-max</x:v>
       </x:c>
       <x:c r="E76" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F76" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -12161,13 +12880,13 @@
         <x:v>百度 / 文心 ERNIE</x:v>
       </x:c>
       <x:c r="C79" s="64" t="str">
-        <x:v>2026-01 / 07 ERNIE 5.0 / 5.1</x:v>
+        <x:v>2026 ERNIE 5.0 / 5.1</x:v>
       </x:c>
       <x:c r="D79" s="96" t="str">
         <x:v>https://cloud.baidu.cn/news/news_eacd5e1a-b6ad-4874-b920-15390d26e656</x:v>
       </x:c>
       <x:c r="E79" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F79" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -12321,13 +13040,13 @@
         <x:v>腾讯 / 混元 Hy</x:v>
       </x:c>
       <x:c r="C87" s="64" t="str">
-        <x:v>2026 Hy3</x:v>
+        <x:v>2026 Hy3；Hy4 Preview</x:v>
       </x:c>
       <x:c r="D87" s="96" t="str">
-        <x:v>https://www.tencent.com/zh-cn/tencent-hunyuan-officially-releases-hy3-advancing-agent-capabilities-and-deeper-product-integration/</x:v>
+        <x:v>https://cloud.tencent.com/product/tokenhub</x:v>
       </x:c>
       <x:c r="E87" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F87" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -12381,13 +13100,13 @@
         <x:v>智谱 AI / GLM</x:v>
       </x:c>
       <x:c r="C90" s="64" t="str">
-        <x:v>2026 GLM-5 / 5.1 / 5.2；GLM-5V-Turbo</x:v>
+        <x:v>2026 GLM-5 / 5.1 / 5.2 / 5.3</x:v>
       </x:c>
       <x:c r="D90" s="96" t="str">
-        <x:v>https://docs.bigmodel.cn/cn/guide/models/text/glm-5.2</x:v>
+        <x:v>https://bigmodel.cn/pricing</x:v>
       </x:c>
       <x:c r="E90" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F90" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -12621,13 +13340,13 @@
         <x:v>科大讯飞 / 星火</x:v>
       </x:c>
       <x:c r="C102" s="64" t="str">
-        <x:v>2024 星火 V3.5 / 4.0</x:v>
+        <x:v>2026 MiniMax M2.5 / M2.7 / M3</x:v>
       </x:c>
       <x:c r="D102" s="96" t="str">
-        <x:v>https://xinghuo.xfyun.cn/news</x:v>
+        <x:v>https://www.minimax.io/news/minimax-m3</x:v>
       </x:c>
       <x:c r="E102" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F102" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -12781,13 +13500,13 @@
         <x:v>商汤 / 日日新 SenseNova</x:v>
       </x:c>
       <x:c r="C110" s="64" t="str">
-        <x:v>2026 U1 Pro / 6.8 Flash Lite</x:v>
+        <x:v>2026 SenseNova U1 / 6.8 Flash Lite；Token Plan</x:v>
       </x:c>
       <x:c r="D110" s="96" t="str">
-        <x:v>https://www.sensetime.com/cn/news/sensenova-6.8-flash-lite-preview</x:v>
+        <x:v>https://platform.sensenova.cn/token-plan</x:v>
       </x:c>
       <x:c r="E110" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-07</x:v>
       </x:c>
       <x:c r="F110" s="91" t="str">
         <x:v>【公开事实】</x:v>
@@ -13651,6 +14370,166 @@
       </x:c>
       <x:c r="F153" s="94" t="str">
         <x:v>B｜官方产品事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B154" t="str">
+        <x:v>OpenAI｜GPT-6 Astra</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>https://developers.openai.com/api/docs/models/gpt-6-astra</x:v>
+      </x:c>
+      <x:c r="E154" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F154" t="str">
+        <x:v>官方模型与价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>Anthropic｜Claude Fable 5.1</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D155" t="str">
+        <x:v>https://platform.claude.com/docs/en/about-claude/pricing</x:v>
+      </x:c>
+      <x:c r="E155" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F155" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B156" t="str">
+        <x:v>Google DeepMind｜Gemini 3.8 Flash</x:v>
+      </x:c>
+      <x:c r="C156" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D156" t="str">
+        <x:v>https://ai.google.dev/gemini-api/docs/pricing</x:v>
+      </x:c>
+      <x:c r="E156" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F156" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B157" t="str">
+        <x:v>腾讯 / 混元 Hy｜Hy4 Preview</x:v>
+      </x:c>
+      <x:c r="C157" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D157" t="str">
+        <x:v>https://cloud.tencent.com/document/product/1823/130055</x:v>
+      </x:c>
+      <x:c r="E157" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F157" t="str">
+        <x:v>TokenHub 价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B158" t="str">
+        <x:v>智谱 AI / GLM｜GLM-5.3</x:v>
+      </x:c>
+      <x:c r="C158" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D158" t="str">
+        <x:v>https://bigmodel.cn/pricing</x:v>
+      </x:c>
+      <x:c r="E158" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F158" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B159" t="str">
+        <x:v>MiniMax｜MiniMax M3 ≤512K</x:v>
+      </x:c>
+      <x:c r="C159" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D159" t="str">
+        <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
+      </x:c>
+      <x:c r="E159" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F159" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B160" t="str">
+        <x:v>百度 / 文心 ERNIE｜ERNIE 5.1 32K—128K</x:v>
+      </x:c>
+      <x:c r="C160" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D160" t="str">
+        <x:v>https://cloud.baidu.com/doc/qianfan/s/wmh4sv6ya</x:v>
+      </x:c>
+      <x:c r="E160" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F160" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B161" t="str">
+        <x:v>MiniMax｜MiniMax M3 &gt;512K</x:v>
+      </x:c>
+      <x:c r="C161" t="str">
+        <x:v>当前价格与计费条件</x:v>
+      </x:c>
+      <x:c r="D161" t="str">
+        <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
+      </x:c>
+      <x:c r="E161" t="str">
+        <x:v>2026-09-07</x:v>
+      </x:c>
+      <x:c r="F161" t="str">
+        <x:v>官方价格页</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13659,7 +14538,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dea822b3e8744bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27cbe2e31c74499e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
data: refresh models and pricing for 2026-09-14
</commit_message>
<xml_diff>
--- a/public/AI模型厂商全景_2023-2026.xlsx
+++ b/public/AI模型厂商全景_2023-2026.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R9ac234d8b78b4553"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="厂商地图" sheetId="2" r:id="Rf7836ba07e7f4b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型时间轴" sheetId="3" r:id="R6b216b3527914c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前定价" sheetId="4" r:id="R0a228ce26e544ce3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本计算器" sheetId="5" r:id="R7c654cef0df84228"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用案例" sheetId="6" r:id="R0005ff6b4aeb4c4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景选型" sheetId="7" r:id="Rf815e41ab1d04810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料来源" sheetId="8" r:id="Re97935fc9c4f448e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rd01a4dee867144c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="厂商地图" sheetId="2" r:id="Rc76cd3d5ec954741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型时间轴" sheetId="3" r:id="Radcf04a74a444c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前定价" sheetId="4" r:id="R0b00338896624fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本计算器" sheetId="5" r:id="R5b0d104946be471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用案例" sheetId="6" r:id="R40a6e509ba1b4ddf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景选型" sheetId="7" r:id="R3407b46b6c444fd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料来源" sheetId="8" r:id="Rc81f718795e74ff7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -336,7 +336,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="146">
+  <x:cellXfs count="147">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -667,6 +667,9 @@
     <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -702,8 +705,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TimelineTable" displayName="TimelineTable" ref="A2:H98" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A2:H98"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TimelineTable" displayName="TimelineTable" ref="A2:H110" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A2:H110"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="年份"/>
     <x:tableColumn id="2" name="厂商"/>
@@ -719,8 +722,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PricesTable" displayName="PricesTable" ref="A2:O54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A2:O54"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PricesTable" displayName="PricesTable" ref="A2:O60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A2:O60"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="区域"/>
     <x:tableColumn id="2" name="厂商"/>
@@ -743,8 +746,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CostCalculatorTable" displayName="CostCalculatorTable" ref="A9:O59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A9:O59"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CostCalculatorTable" displayName="CostCalculatorTable" ref="A9:O65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A9:O65"/>
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="区域"/>
     <x:tableColumn id="2" name="厂商"/>
@@ -767,8 +770,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CasesTable" displayName="CasesTable" ref="A2:J27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A2:J27"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CasesTable" displayName="CasesTable" ref="A2:J28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A2:J28"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="领域"/>
     <x:tableColumn id="2" name="组织/项目"/>
@@ -803,8 +806,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SourcesTable" displayName="SourcesTable" ref="A12:F161" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A12:F161"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SourcesTable" displayName="SourcesTable" ref="A12:F180" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A12:F180"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="类别"/>
     <x:tableColumn id="2" name="厂商/对象"/>
@@ -1066,7 +1069,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>研究日：2026-09-07｜范围：24 家代表厂商｜价格与产品为查询日快照，采购前请复核来源</x:v>
+        <x:v>研究日：2026-09-14｜范围：24 家代表厂商｜价格与产品为查询日快照，采购前请复核来源</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1092,21 +1095,19 @@
         <x:v>时间轴节点</x:v>
       </x:c>
       <x:c r="E4" s="15" t="n">
-        <x:f>COUNTA('模型时间轴'!$B$3:$B$160)</x:f>
-        <x:v>96</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="G4" s="14" t="str">
         <x:v>当前价格行</x:v>
       </x:c>
       <x:c r="H4" s="15" t="n">
-        <x:v>52</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="J4" s="14" t="str">
         <x:v>公开案例</x:v>
       </x:c>
       <x:c r="K4" s="15" t="n">
-        <x:f>COUNTA('应用案例'!$B$3:$B$80)</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1264,7 +1265,7 @@
       <x:c r="B15" s="64"/>
       <x:c r="C15" s="64"/>
       <x:c r="D15" s="64" t="str">
-        <x:v>GPT-5.6 Luna；Gemini Flash-Lite；Mistral Small；DeepSeek V4 Flash；Step Flash；ERNIE Turbo</x:v>
+        <x:v>GPT-5.6 Luna；Gemini Flash-Lite；Mistral Small；DeepSeek V4.1 Flash；Step-3.5 Flash；Qwen3.8 Flash；ERNIE Turbo</x:v>
       </x:c>
       <x:c r="E15" s="64"/>
       <x:c r="F15" s="64"/>
@@ -1503,13 +1504,13 @@
         <x:v>OpenAI</x:v>
       </x:c>
       <x:c r="C3" s="88" t="str">
-        <x:v>从 GPT-4 的多模态能力，演进到 GPT-4o 的实时多模态、o1 的推理范式、GPT-5/5.6 的统一推理与 Agent 工具栈，并在 2026-09 推出 GPT-6 Astra。</x:v>
+        <x:v>从 GPT-4 的多模态能力，演进到 GPT-4o 的实时多模态、o1 的推理范式、GPT-5/5.6 的统一推理与 Agent 工具栈；2026-09 又推出 Astra、GPT-Live、Image 2.5、Rosalind 与 Cyber 专业模型。</x:v>
       </x:c>
       <x:c r="D3" s="88" t="str">
-        <x:v>GPT-6 Astra；GPT-5.6 Sol / Terra / Luna；GPT-Realtime-2.1；GPT-Image-2</x:v>
+        <x:v>GPT-6 Astra；GPT-5.6 Sol / Terra / Luna / Cyber；GPT-Live 1；GPT Image 2.5</x:v>
       </x:c>
       <x:c r="E3" s="88" t="str">
-        <x:v>ChatGPT、Responses API、Codex、Sora</x:v>
+        <x:v>ChatGPT、Responses API、Codex、Sora、Daybreak</x:v>
       </x:c>
       <x:c r="F3" s="88" t="str">
         <x:v>复杂推理、代码、工具调用、计算机使用、多模态</x:v>
@@ -1521,16 +1522,16 @@
         <x:v>第一方 API；云市场渠道</x:v>
       </x:c>
       <x:c r="I3" s="88" t="str">
-        <x:v>Astra $10/$50；Sol $4/$20；Luna $0.2/$1.2（输入/输出，USD/百万tokens）</x:v>
+        <x:v>Astra $10/$50；Cyber $12.5/$75；Luna $0.2/$1.2（输入/输出，USD/百万tokens）</x:v>
       </x:c>
       <x:c r="J3" s="88" t="str">
         <x:v>高难知识工作、代码 Agent、通用智能体、高并发分层路由</x:v>
       </x:c>
       <x:c r="K3" s="95" t="str">
-        <x:v>https://developers.openai.com/api/docs/models/gpt-6-astra</x:v>
+        <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-cyber</x:v>
       </x:c>
       <x:c r="L3" s="89" t="str">
-        <x:v>【公开事实】Astra &gt;272K 整次请求升价；Batch/Flex 与 Fast 档另计</x:v>
+        <x:v>【公开事实】Cyber 需 Daybreak 单独审批；&gt;272K 输入/缓存 2×、输出 1.5×</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
@@ -1617,10 +1618,10 @@
         <x:v>Meta</x:v>
       </x:c>
       <x:c r="C6" s="64" t="str">
-        <x:v>以 Llama 2/3/4 建立开放权重生态；2026 年扩展 Muse Spark 1.3、Muse Voice、Muse Image 与第一方 Model API。</x:v>
+        <x:v>以 Llama 2/3/4 建立开放权重生态；2026 年扩展 Muse Spark 1.3、Muse Glimmer、Muse Voice、Muse Image 与第一方 Model API。</x:v>
       </x:c>
       <x:c r="D6" s="64" t="str">
-        <x:v>Llama 4 Scout/Maverick；Muse Spark 1.3；Muse Voice；Muse Image</x:v>
+        <x:v>Llama 4 Scout/Maverick；Muse Spark 1.3；Muse Glimmer；Muse Voice；Muse Image</x:v>
       </x:c>
       <x:c r="E6" s="64" t="str">
         <x:v>Meta AI、Model API、WhatsApp/Instagram/Facebook、Ray-Ban Meta</x:v>
@@ -1635,16 +1636,16 @@
         <x:v>第一方 Model API、自建、云厂商托管、端侧</x:v>
       </x:c>
       <x:c r="I6" s="64" t="str">
-        <x:v>Voice Transcribe $0.18/小时；Muse Image $0.01/张；文本 token 价以控制台为准</x:v>
+        <x:v>Muse Spark 标准 $1.25/$4.25；Voice Transcribe $0.18/小时；Muse Image $0.01/张</x:v>
       </x:c>
       <x:c r="J6" s="64" t="str">
         <x:v>行业微调、私有部署、客服、端侧助手、合成数据</x:v>
       </x:c>
       <x:c r="K6" s="96" t="str">
-        <x:v>https://developer.meta.com/ai</x:v>
+        <x:v>https://developer.meta.com/ai/products/muse-code/</x:v>
       </x:c>
       <x:c r="L6" s="91" t="str">
-        <x:v>【公开事实】开放权重与第一方 API 为不同成本口径</x:v>
+        <x:v>【公开事实】Muse Spark contributor 档需允许数据用于改进产品；开放权重与第一方 API 为不同成本口径</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -1734,13 +1735,13 @@
         <x:v>聚焦企业数据上的 RAG、检索、重排、跨语言与私有部署，模型从 Command R/R+ 演进到 Command A/A+ 与 North。</x:v>
       </x:c>
       <x:c r="D9" s="64" t="str">
-        <x:v>Command A+ / A；Embed 4；Rerank 4；North</x:v>
+        <x:v>Command A+；North Small Translate 1.0；Embed；Rerank</x:v>
       </x:c>
       <x:c r="E9" s="64" t="str">
         <x:v>Cohere Platform、North、Model Vault</x:v>
       </x:c>
       <x:c r="F9" s="64" t="str">
-        <x:v>企业 RAG、引用、检索/重排、多语言、数据驻留</x:v>
+        <x:v>企业 RAG、检索、翻译、重排、多语言与数据驻留</x:v>
       </x:c>
       <x:c r="G9" s="64" t="str">
         <x:v>闭源 + 可私有部署</x:v>
@@ -1749,16 +1750,16 @@
         <x:v>API、云市场、VPC/本地 Vault</x:v>
       </x:c>
       <x:c r="I9" s="64" t="str">
-        <x:v>Command A+ 自助 API 免费至触发限速；生产私有 Vault 按实例/承诺计费</x:v>
+        <x:v>Chat V2 免费层可评估；生产经 Model Vault 商业许可</x:v>
       </x:c>
       <x:c r="J9" s="64" t="str">
         <x:v>企业搜索、知识库、客服、主权/保密部署</x:v>
       </x:c>
       <x:c r="K9" s="96" t="str">
-        <x:v>https://docs.cohere.com/docs/command-a-plus</x:v>
+        <x:v>https://docs.cohere.com/docs/models</x:v>
       </x:c>
       <x:c r="L9" s="91" t="str">
-        <x:v>【公开事实】免费限速档不等于生产 SLA 或无限额度</x:v>
+        <x:v>【公开事实】North Small Translate 支持 50+ 语言；免费评估不等于免费生产</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -1772,10 +1773,10 @@
         <x:v>Bedrock 作为多模型托管入口，Amazon 自研从 Titan 扩展至 Nova 的理解、创作、实时语音与定制模型。</x:v>
       </x:c>
       <x:c r="D10" s="64" t="str">
-        <x:v>Nova 2 Lite / Sonic；Nova Premier / Forge；Claude Fable 5.1</x:v>
+        <x:v>Amazon Nova；GPT-6 Astra；Claude Fable 5.1；Bedrock 模型市场</x:v>
       </x:c>
       <x:c r="E10" s="64" t="str">
-        <x:v>Amazon Bedrock、Amazon Q、Nova Act/Forge</x:v>
+        <x:v>Amazon Bedrock、SageMaker、ChatGPT Work / Codex 配置</x:v>
       </x:c>
       <x:c r="F10" s="64" t="str">
         <x:v>云原生托管、模型选择、企业安全、RAG、实时语音</x:v>
@@ -1793,10 +1794,10 @@
         <x:v>AWS 既有客户、客服/RAG、多模型路由、语音应用</x:v>
       </x:c>
       <x:c r="K10" s="96" t="str">
-        <x:v>https://aws.amazon.com/about-aws/whats-new/2026/09/claude-fable-5-1-aws/</x:v>
+        <x:v>https://aws.amazon.com/blogs/machine-learning/take-on-your-most-ambitious-work-with-gpt-6-astra-on-amazon-bedrock/</x:v>
       </x:c>
       <x:c r="L10" s="91" t="str">
-        <x:v>【公开事实】Bedrock 同时提供自研与第三方模型，价格随区域/档位变化</x:v>
+        <x:v>【公开事实】Astra 已在 Bedrock GA；精确地区与价格需在控制台复核</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -1810,7 +1811,7 @@
         <x:v>Phi 路线强调小模型与端侧；MAI 路线面向 Copilot 的自研闭源前沿模型，并与 Azure 模型目录形成组合。</x:v>
       </x:c>
       <x:c r="D11" s="64" t="str">
-        <x:v>Phi-4 Reasoning Vision；MAI-1；MAI-Voice；MAI-Transcribe-2；GPT-6 Astra</x:v>
+        <x:v>Phi；MAI-Transcribe-2；MAI-Image-2.6 / Flash；GPT-6 Astra</x:v>
       </x:c>
       <x:c r="E11" s="64" t="str">
         <x:v>Microsoft Copilot、Azure AI Foundry、Windows/Edge</x:v>
@@ -1825,16 +1826,16 @@
         <x:v>本地/端侧、Azure、Copilot</x:v>
       </x:c>
       <x:c r="I11" s="64" t="str">
-        <x:v>Foundry Astra 短上下文 $10/$50；Phi/MAI 与语音模型按服务计费</x:v>
+        <x:v>MAI-Transcribe-2 限时 $0.10/小时；Foundry Astra 短上下文 $10/$50</x:v>
       </x:c>
       <x:c r="J11" s="64" t="str">
         <x:v>端侧、离线、轻量代码/视觉、微软生态应用</x:v>
       </x:c>
       <x:c r="K11" s="96" t="str">
-        <x:v>https://azure.microsoft.com/en-us/blog/gpt-6-astra-frontier-intelligence-for-work-now-generally-available-in-microsoft-foundry/</x:v>
+        <x:v>https://microsoft.ai/news/mai-transcribe-2-is-the-fastest-most-accurate-and-cheapest-speech-recognition-model-in-the-world/</x:v>
       </x:c>
       <x:c r="L11" s="91" t="str">
-        <x:v>【公开事实】MAI-Transcribe-2 于 2026-09-03 发布；区域可用性需核验</x:v>
+        <x:v>【公开事实】Transcribe 限时价至 2026 年底；Image 2.6 系列为 Foundry Public Preview</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -1848,13 +1849,13 @@
         <x:v>由基于既有底模的后训练与合成数据路线，发展为 Nemotron 3 的开放 Agent 模型栈，覆盖规划、执行、多模态、RAG 与安全。</x:v>
       </x:c>
       <x:c r="D12" s="64" t="str">
-        <x:v>Nemotron 3 Ultra / Super / 3.5 Lightning / Nano Omni</x:v>
+        <x:v>Nemotron 3.5 Lightning；Nemotron 3；NIM；NeMo</x:v>
       </x:c>
       <x:c r="E12" s="64" t="str">
         <x:v>NeMo、NIM、AI Enterprise、Blueprints</x:v>
       </x:c>
       <x:c r="F12" s="64" t="str">
-        <x:v>高吞吐 Agent、开放数据/配方、GPU 优化、私有部署</x:v>
+        <x:v>高吞吐 Agent、开放模型配方、后训练与 GPU 推理优化</x:v>
       </x:c>
       <x:c r="G12" s="64" t="str">
         <x:v>开放模型（许可需核对）</x:v>
@@ -1901,7 +1902,7 @@
         <x:v>百炼 API、开源自建、专属部署</x:v>
       </x:c>
       <x:c r="I13" s="64" t="str">
-        <x:v>Qwen3.8-Max ¥12/¥36；Qwen3.8-Max Prime ¥24/¥72；Qwen3-Max ≤32K ¥2.5/¥10</x:v>
+        <x:v>Qwen3.8-Max $12/$36；Qwen3.8-Flash ¥0.8/¥2.7；Qwen3-Max ¥2.5/¥10</x:v>
       </x:c>
       <x:c r="J13" s="64" t="str">
         <x:v>中文 Agent、代码、企业知识、私有化、底模微调</x:v>
@@ -1962,7 +1963,7 @@
         <x:v>依托豆包、抖音与火山引擎形成大规模产品反馈，模型覆盖通用 Agent、代码、语音、图像与视频。</x:v>
       </x:c>
       <x:c r="D15" s="64" t="str">
-        <x:v>Doubao Seed 2.1 / 2.0；Seedance 2.5；Seedream 5</x:v>
+        <x:v>Seed-Evolving；Seed 2.x；Seedream；Seedance</x:v>
       </x:c>
       <x:c r="E15" s="64" t="str">
         <x:v>豆包、TRAE、扣子、即梦、火山方舟</x:v>
@@ -1977,16 +1978,16 @@
         <x:v>火山方舟 API、批量、缓存、专属部署</x:v>
       </x:c>
       <x:c r="I15" s="64" t="str">
-        <x:v>Seed 2.1 Pro 约 ¥6/¥30；Turbo 约 ¥3/¥15</x:v>
+        <x:v>Seed-Evolving ¥6/¥30；缓存命中 ¥1.2；缓存存储 ¥0.017/MTok/小时</x:v>
       </x:c>
       <x:c r="J15" s="64" t="str">
         <x:v>C 端助手、代码、营销内容、客服、视频/图像生产</x:v>
       </x:c>
       <x:c r="K15" s="96" t="str">
-        <x:v>https://seed.bytedance.com/</x:v>
+        <x:v>https://docs.volcengine.com/docs/82379/1544106?lang=zh</x:v>
       </x:c>
       <x:c r="L15" s="91" t="str">
-        <x:v>【公开事实】活动/节省计划价需与刊例价分开</x:v>
+        <x:v>【公开事实】Seed-Evolving 为滚动升级模型 ID；1,024K 上下文、256K 最大输出</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -2073,10 +2074,10 @@
         <x:v>DeepSeek</x:v>
       </x:c>
       <x:c r="C18" s="64" t="str">
-        <x:v>由 Coder/LLM 进入通用模型，V2/V3 以 MoE 和低成本扩大影响，R1 推动推理开源，V4 强化 1M 上下文与 Agent。</x:v>
+        <x:v>以 Coder/V2/V3 的 MoE 与低成本路线切入，R1 推动开放推理与蒸馏；2026-09 发布带原生视觉与 1M 上下文的 V4.1 Flash。</x:v>
       </x:c>
       <x:c r="D18" s="64" t="str">
-        <x:v>DeepSeek V4 Pro / Flash；开源 V4/R1 系列</x:v>
+        <x:v>DeepSeek V4.1 Flash / V4 Pro；R1</x:v>
       </x:c>
       <x:c r="E18" s="64" t="str">
         <x:v>DeepSeek Chat、DeepSeek API、开源权重与技术报告</x:v>
@@ -2091,16 +2092,16 @@
         <x:v>第一方 API、自建、云平台托管</x:v>
       </x:c>
       <x:c r="I18" s="64" t="str">
-        <x:v>V4 Flash 非高峰缓存/输入/输出 ¥0.05/¥1.5/¥4.5；高峰 ¥0.1/¥3/¥9</x:v>
+        <x:v>V4.1 Flash 闲时 ¥1/¥4，缓存 ¥0.02；忙时 ¥2/¥8，缓存 ¥0.04</x:v>
       </x:c>
       <x:c r="J18" s="64" t="str">
         <x:v>低成本 Agent、代码、推理、底模蒸馏、私有化</x:v>
       </x:c>
       <x:c r="K18" s="96" t="str">
-        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing/</x:v>
       </x:c>
       <x:c r="L18" s="91" t="str">
-        <x:v>【公开事实】峰谷、缓存命中与失败重试会显著改变实际成本</x:v>
+        <x:v>【公开事实】旧 deepseek-v4-flash 临时兼容路由至 deepseek-flash</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -2114,7 +2115,7 @@
         <x:v>从超长上下文助手建立认知，K2/K2 Thinking 强化代码与 Agent，K2.5/K3 进入原生多模态和 1M 上下文。</x:v>
       </x:c>
       <x:c r="D19" s="64" t="str">
-        <x:v>Kimi K3 / K2.7 Code / K2.6</x:v>
+        <x:v>Kimi K3；K2.8 Preview / Kimi Code；K2.7 API</x:v>
       </x:c>
       <x:c r="E19" s="64" t="str">
         <x:v>Kimi、Kimi API、深度研究、Office/网页生成</x:v>
@@ -2129,16 +2130,16 @@
         <x:v>第一方 API、开源自建、云平台托管</x:v>
       </x:c>
       <x:c r="I19" s="64" t="str">
-        <x:v>K3 ¥20/¥100，缓存 ¥2；K2.7 Code ¥6.5/¥27</x:v>
+        <x:v>K3 ¥20/¥100；K2.7 API ¥6.5/¥27；K2.8 Preview 暂无通用 API 公开价</x:v>
       </x:c>
       <x:c r="J19" s="64" t="str">
         <x:v>研究/搜索、长文档、代码、知识工作、多模态</x:v>
       </x:c>
       <x:c r="K19" s="96" t="str">
-        <x:v>https://platform.kimi.com/</x:v>
+        <x:v>https://www.kimi.com/code/docs/kimi-code/whats-new.html</x:v>
       </x:c>
       <x:c r="L19" s="91" t="str">
-        <x:v>【公开事实】国内外 API 币种与价格页可能不同</x:v>
+        <x:v>【公开事实】Kimi Code 模型 ID 不变；全会员档支持 1M 上下文</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -2167,7 +2168,7 @@
         <x:v>API、订阅 Token Plan、专属部署</x:v>
       </x:c>
       <x:c r="I20" s="64" t="str">
-        <x:v>M3 ≤512K ¥2.1/¥8.4，缓存 ¥0.42；&gt;512K ¥4.2/¥16.8</x:v>
+        <x:v>M3 ≤512K 永久五折 ¥2.1/¥8.4；M2.7 ¥2.1/¥8.4</x:v>
       </x:c>
       <x:c r="J20" s="64" t="str">
         <x:v>Agent、代码、Office 交付、视频/语音、角色互动</x:v>
@@ -2176,7 +2177,7 @@
         <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
       </x:c>
       <x:c r="L20" s="91" t="str">
-        <x:v>【公开事实】M3 当前为促销价；高速版、订阅与按量不可直接横比</x:v>
+        <x:v>【公开事实】M3 永久五折；高速版、长上下文与 Token Plan 另计</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
@@ -2304,7 +2305,7 @@
         <x:v>从 Step-1/1V/2 的通用和多模态，发展到 Step-3/3.5/3.7 Flash 的高吞吐 Agent 与本地部署路线。</x:v>
       </x:c>
       <x:c r="D24" s="64" t="str">
-        <x:v>Step-3.7 Flash / 3.5 Flash；Step-3；Step-Audio</x:v>
+        <x:v>Step-3.7 Flash；Step-3.5 Flash；Step Audio</x:v>
       </x:c>
       <x:c r="E24" s="64" t="str">
         <x:v>跃问、StepFun 开放平台、Agent/MCP 示例</x:v>
@@ -2319,7 +2320,7 @@
         <x:v>API、自建、本地工作站/DGX</x:v>
       </x:c>
       <x:c r="I24" s="64" t="str">
-        <x:v>3.5 Flash ¥0.7/¥2.1，缓存 ¥0.14；Step-2 mini ¥1/¥2</x:v>
+        <x:v>Step-3.7 Flash ¥1.35/¥8.1，缓存 ¥0.27；Step-3.5 Flash ¥0.7/¥2.1</x:v>
       </x:c>
       <x:c r="J24" s="64" t="str">
         <x:v>低成本 Agent、MCP 工具链、多模态、私有部署</x:v>
@@ -2328,7 +2329,7 @@
         <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
       </x:c>
       <x:c r="L24" s="91" t="str">
-        <x:v>【公开事实】具体模型可用性以平台目录为准</x:v>
+        <x:v>【公开事实】Step-3.7 Flash 256K，原生图像/视频理解；具体首发日待核</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
@@ -2413,7 +2414,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b1a8e201b874d5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf4a0077e4a4f63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4980,13 +4981,325 @@
         <x:v>【待验证】</x:v>
       </x:c>
     </x:row>
+    <x:row r="99" ht="54" customHeight="1">
+      <x:c r="A99" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B99" s="146" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C99" s="146" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+      <x:c r="D99" s="146" t="str">
+        <x:v>GPT Image 2.5 Sunburst / Flare</x:v>
+      </x:c>
+      <x:c r="E99" s="146" t="str">
+        <x:v>图像生成与编辑；新增 xhigh / max 质量档</x:v>
+      </x:c>
+      <x:c r="F99" s="146" t="str">
+        <x:v>Images API</x:v>
+      </x:c>
+      <x:c r="G99" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="H99" s="146" t="str">
+        <x:v>【公开事实】</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="54" customHeight="1">
+      <x:c r="A100" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B100" s="146" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C100" s="146" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+      <x:c r="D100" s="146" t="str">
+        <x:v>GPT-Rosalind</x:v>
+      </x:c>
+      <x:c r="E100" s="146" t="str">
+        <x:v>trusted access GA；获批内部生命科学研究</x:v>
+      </x:c>
+      <x:c r="F100" s="146" t="str">
+        <x:v>OpenAI API</x:v>
+      </x:c>
+      <x:c r="G100" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="H100" s="146" t="str">
+        <x:v>【公开事实】2026-10-05 起计费</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="54" customHeight="1">
+      <x:c r="A101" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B101" s="146" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C101" s="146" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="D101" s="146" t="str">
+        <x:v>GPT-Live 1</x:v>
+      </x:c>
+      <x:c r="E101" s="146" t="str">
+        <x:v>全双工语音 API GA；会话 $0.05/分钟</x:v>
+      </x:c>
+      <x:c r="F101" s="146" t="str">
+        <x:v>Realtime / Live API</x:v>
+      </x:c>
+      <x:c r="G101" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="H101" s="146" t="str">
+        <x:v>【公开事实】后端模型与工具另计</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="54" customHeight="1">
+      <x:c r="A102" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B102" s="146" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C102" s="146" t="str">
+        <x:v>2026-09-11 / 10-01</x:v>
+      </x:c>
+      <x:c r="D102" s="146" t="str">
+        <x:v>GPT-5.4-Cyber → GPT-5.6 Cyber</x:v>
+      </x:c>
+      <x:c r="E102" s="146" t="str">
+        <x:v>旧版宣布弃用，10 月 1 日移除</x:v>
+      </x:c>
+      <x:c r="F102" s="146" t="str">
+        <x:v>OpenAI API / Daybreak</x:v>
+      </x:c>
+      <x:c r="G102" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/deprecations</x:v>
+      </x:c>
+      <x:c r="H102" s="146" t="str">
+        <x:v>【公开事实】需迁移；GPT-5.6 Cyber 单独审批</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="54" customHeight="1">
+      <x:c r="A103" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B103" s="146" t="str">
+        <x:v>Cohere</x:v>
+      </x:c>
+      <x:c r="C103" s="146" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
+      <x:c r="D103" s="146" t="str">
+        <x:v>North Small Translate 1.0</x:v>
+      </x:c>
+      <x:c r="E103" s="146" t="str">
+        <x:v>50+ 语言翻译；218B 总参数 / 25B active MoE；16K</x:v>
+      </x:c>
+      <x:c r="F103" s="146" t="str">
+        <x:v>Chat V2 / Model Vault</x:v>
+      </x:c>
+      <x:c r="G103" s="146" t="str">
+        <x:v>https://docs.cohere.com/v2/changelog</x:v>
+      </x:c>
+      <x:c r="H103" s="146" t="str">
+        <x:v>【公开事实】免费层仅评估，生产需商业许可</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="54" customHeight="1">
+      <x:c r="A104" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B104" s="146" t="str">
+        <x:v>Amazon / AWS</x:v>
+      </x:c>
+      <x:c r="C104" s="146" t="str">
+        <x:v>2026-09-08</x:v>
+      </x:c>
+      <x:c r="D104" s="146" t="str">
+        <x:v>GPT-6 Astra on Bedrock</x:v>
+      </x:c>
+      <x:c r="E104" s="146" t="str">
+        <x:v>在 Amazon Bedrock GA</x:v>
+      </x:c>
+      <x:c r="F104" s="146" t="str">
+        <x:v>Bedrock API；ChatGPT Work / Codex 配置</x:v>
+      </x:c>
+      <x:c r="G104" s="146" t="str">
+        <x:v>https://aws.amazon.com/blogs/machine-learning/take-on-your-most-ambitious-work-with-gpt-6-astra-on-amazon-bedrock/</x:v>
+      </x:c>
+      <x:c r="H104" s="146" t="str">
+        <x:v>【公开事实｜地区与精确价格需控制台复核】</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="54" customHeight="1">
+      <x:c r="A105" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B105" s="146" t="str">
+        <x:v>DeepSeek</x:v>
+      </x:c>
+      <x:c r="C105" s="146" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="D105" s="146" t="str">
+        <x:v>DeepSeek V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="E105" s="146" t="str">
+        <x:v>原生视觉、1M 上下文、384K 最大输出；旧 V4 Flash 临时兼容路由</x:v>
+      </x:c>
+      <x:c r="F105" s="146" t="str">
+        <x:v>DeepSeek API；云平台托管</x:v>
+      </x:c>
+      <x:c r="G105" s="146" t="str">
+        <x:v>https://api-docs.deepseek.com/zh-cn/updates/</x:v>
+      </x:c>
+      <x:c r="H105" s="146" t="str">
+        <x:v>【公开事实】模型 ID 为 deepseek-flash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="54" customHeight="1">
+      <x:c r="A106" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B106" s="146" t="str">
+        <x:v>字节跳动 / 豆包 Seed</x:v>
+      </x:c>
+      <x:c r="C106" s="146" t="str">
+        <x:v>2026-09-09</x:v>
+      </x:c>
+      <x:c r="D106" s="146" t="str">
+        <x:v>Seed-Evolving</x:v>
+      </x:c>
+      <x:c r="E106" s="146" t="str">
+        <x:v>滚动升级模型 ID；1,024K 上下文、256K 最大输出</x:v>
+      </x:c>
+      <x:c r="F106" s="146" t="str">
+        <x:v>火山方舟</x:v>
+      </x:c>
+      <x:c r="G106" s="146" t="str">
+        <x:v>https://docs.volcengine.com/docs/82379/2549861?lang=zh</x:v>
+      </x:c>
+      <x:c r="H106" s="146" t="str">
+        <x:v>【公开事实】</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="54" customHeight="1">
+      <x:c r="A107" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B107" s="146" t="str">
+        <x:v>月之暗面 / Kimi</x:v>
+      </x:c>
+      <x:c r="C107" s="146" t="str">
+        <x:v>2026-09-11</x:v>
+      </x:c>
+      <x:c r="D107" s="146" t="str">
+        <x:v>Kimi Code K2.8 Preview</x:v>
+      </x:c>
+      <x:c r="E107" s="146" t="str">
+        <x:v>全量上线；全会员档支持 1M 上下文</x:v>
+      </x:c>
+      <x:c r="F107" s="146" t="str">
+        <x:v>Kimi Code</x:v>
+      </x:c>
+      <x:c r="G107" s="146" t="str">
+        <x:v>https://www.kimi.com/code/docs/kimi-code/whats-new.html</x:v>
+      </x:c>
+      <x:c r="H107" s="146" t="str">
+        <x:v>【公开事实】模型 ID 仍为 kimi-for-coding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="54" customHeight="1">
+      <x:c r="A108" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B108" s="146" t="str">
+        <x:v>腾讯云 TokenHub</x:v>
+      </x:c>
+      <x:c r="C108" s="146" t="str">
+        <x:v>2026-09-10</x:v>
+      </x:c>
+      <x:c r="D108" s="146" t="str">
+        <x:v>DeepSeek V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="E108" s="146" t="str">
+        <x:v>新增原厂模型并沿用原厂闲时 / 忙时价格</x:v>
+      </x:c>
+      <x:c r="F108" s="146" t="str">
+        <x:v>TokenHub</x:v>
+      </x:c>
+      <x:c r="G108" s="146" t="str">
+        <x:v>https://cloud.tencent.com/document/product/1823/130675</x:v>
+      </x:c>
+      <x:c r="H108" s="146" t="str">
+        <x:v>【公开事实】</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="54" customHeight="1">
+      <x:c r="A109" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B109" s="146" t="str">
+        <x:v>阿里云百炼</x:v>
+      </x:c>
+      <x:c r="C109" s="146" t="str">
+        <x:v>2026-09-13</x:v>
+      </x:c>
+      <x:c r="D109" s="146" t="str">
+        <x:v>DeepSeek V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="E109" s="146" t="str">
+        <x:v>新增原厂模型托管</x:v>
+      </x:c>
+      <x:c r="F109" s="146" t="str">
+        <x:v>百炼 Model Studio</x:v>
+      </x:c>
+      <x:c r="G109" s="146" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/newly-released-models</x:v>
+      </x:c>
+      <x:c r="H109" s="146" t="str">
+        <x:v>【公开事实】</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="54" customHeight="1">
+      <x:c r="A110" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B110" s="146" t="str">
+        <x:v>阶跃星辰 StepFun</x:v>
+      </x:c>
+      <x:c r="C110" s="146" t="str">
+        <x:v>2026-10-10 / 已退役</x:v>
+      </x:c>
+      <x:c r="D110" s="146" t="str">
+        <x:v>step-2x-large / step-image-edit-2 / step-1x-edit</x:v>
+      </x:c>
+      <x:c r="E110" s="146" t="str">
+        <x:v>前两者计划 10 月 10 日退役；step-1x-edit 已退役</x:v>
+      </x:c>
+      <x:c r="F110" s="146" t="str">
+        <x:v>StepFun API</x:v>
+      </x:c>
+      <x:c r="G110" s="146" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/image-offline-notice</x:v>
+      </x:c>
+      <x:c r="H110" s="146" t="str">
+        <x:v>【公开事实】</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc72dfb60c2e458a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c697578c0ea4ff0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6372,7 +6685,7 @@
         <x:v>DeepSeek</x:v>
       </x:c>
       <x:c r="C31" s="64" t="str">
-        <x:v>DeepSeek V4 Flash</x:v>
+        <x:v>DeepSeek V4.1 Flash</x:v>
       </x:c>
       <x:c r="D31" s="64" t="str">
         <x:v>GA</x:v>
@@ -6384,26 +6697,26 @@
         <x:v>每百万tokens</x:v>
       </x:c>
       <x:c r="G31" s="102" t="n">
-        <x:v>1.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H31" s="102" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="I31" s="102"/>
       <x:c r="J31" s="102" t="n">
-        <x:v>4.5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K31" s="64" t="str">
-        <x:v>1M；非高峰价</x:v>
+        <x:v>闲时；忙时输入/缓存/输出为 ¥2/¥0.04/¥8</x:v>
       </x:c>
       <x:c r="L31" s="64" t="str">
-        <x:v>高峰缓存/输入/输出为 ¥0.1/¥3/¥9</x:v>
+        <x:v>模型 ID deepseek-flash；旧 ID 临时兼容路由</x:v>
       </x:c>
       <x:c r="M31" s="64" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="N31" s="96" t="str">
-        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing/</x:v>
       </x:c>
       <x:c r="O31" s="91" t="str">
         <x:v>官方价格页</x:v>
@@ -7336,10 +7649,10 @@
         <x:v>输入 ≤512K</x:v>
       </x:c>
       <x:c r="L52" t="str">
-        <x:v>促销价；高速版与 Token Plan 另计</x:v>
+        <x:v>永久五折价；高速版与 Token Plan 另计</x:v>
       </x:c>
       <x:c r="M52" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="N52" t="str">
         <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
@@ -7424,15 +7737,285 @@
         <x:v>输入 &gt;512K</x:v>
       </x:c>
       <x:c r="L54" t="str">
-        <x:v>促销价；高速版与 Token Plan 另计</x:v>
+        <x:v>永久五折价；高速版与 Token Plan 另计</x:v>
       </x:c>
       <x:c r="M54" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="N54" t="str">
         <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
       </x:c>
       <x:c r="O54" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="54" customHeight="1">
+      <x:c r="A55" s="146" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B55" s="146" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C55" s="146" t="str">
+        <x:v>GPT-5.6 Cyber</x:v>
+      </x:c>
+      <x:c r="D55" s="146" t="str">
+        <x:v>GA/审批</x:v>
+      </x:c>
+      <x:c r="E55" s="146" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F55" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G55" s="146" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="H55" s="146" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="I55" s="146" t="n">
+        <x:v>15.625</x:v>
+      </x:c>
+      <x:c r="J55" s="146" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="K55" s="146" t="str">
+        <x:v>400K；&gt;272K 输入/缓存 2×、输出 1.5×</x:v>
+      </x:c>
+      <x:c r="L55" s="146" t="str">
+        <x:v>需 Daybreak 单独审批</x:v>
+      </x:c>
+      <x:c r="M55" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="N55" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-cyber</x:v>
+      </x:c>
+      <x:c r="O55" s="146" t="str">
+        <x:v>官方模型与价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="54" customHeight="1">
+      <x:c r="A56" s="146" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B56" s="146" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C56" s="146" t="str">
+        <x:v>GPT-Rosalind</x:v>
+      </x:c>
+      <x:c r="D56" s="146" t="str">
+        <x:v>GA/审批</x:v>
+      </x:c>
+      <x:c r="E56" s="146" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F56" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G56" s="146" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H56" s="146" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="I56" s="146"/>
+      <x:c r="J56" s="146" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="K56" s="146" t="str">
+        <x:v>trusted access；内部生命科学研究</x:v>
+      </x:c>
+      <x:c r="L56" s="146" t="str">
+        <x:v>2026-10-05 起计费</x:v>
+      </x:c>
+      <x:c r="M56" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="N56" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="O56" s="146" t="str">
+        <x:v>官方变更日志</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="54" customHeight="1">
+      <x:c r="A57" s="146" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B57" s="146" t="str">
+        <x:v>Meta</x:v>
+      </x:c>
+      <x:c r="C57" s="146" t="str">
+        <x:v>Muse Spark 1.3</x:v>
+      </x:c>
+      <x:c r="D57" s="146" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="E57" s="146" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="F57" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G57" s="146" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="H57" s="146" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="I57" s="146"/>
+      <x:c r="J57" s="146" t="n">
+        <x:v>4.25</x:v>
+      </x:c>
+      <x:c r="K57" s="146" t="str">
+        <x:v>标准档</x:v>
+      </x:c>
+      <x:c r="L57" s="146" t="str">
+        <x:v>contributor 档 $0.10/$0.002/$0.20，需允许用于改进产品</x:v>
+      </x:c>
+      <x:c r="M57" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="N57" s="146" t="str">
+        <x:v>https://developer.meta.com/ai/products/muse-code/</x:v>
+      </x:c>
+      <x:c r="O57" s="146" t="str">
+        <x:v>官方产品页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="54" customHeight="1">
+      <x:c r="A58" s="146" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B58" s="146" t="str">
+        <x:v>阿里云 / 通义千问 Qwen</x:v>
+      </x:c>
+      <x:c r="C58" s="146" t="str">
+        <x:v>Qwen3.8-Flash</x:v>
+      </x:c>
+      <x:c r="D58" s="146" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="E58" s="146" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F58" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G58" s="146" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H58" s="146"/>
+      <x:c r="I58" s="146"/>
+      <x:c r="J58" s="146" t="n">
+        <x:v>2.7</x:v>
+      </x:c>
+      <x:c r="K58" s="146" t="str">
+        <x:v>中国内地公开价</x:v>
+      </x:c>
+      <x:c r="L58" s="146" t="str">
+        <x:v>搜索、工具与上下文阶梯另计</x:v>
+      </x:c>
+      <x:c r="M58" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="N58" s="146" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
+      </x:c>
+      <x:c r="O58" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="54" customHeight="1">
+      <x:c r="A59" s="146" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B59" s="146" t="str">
+        <x:v>字节跳动 / 豆包 Seed</x:v>
+      </x:c>
+      <x:c r="C59" s="146" t="str">
+        <x:v>Seed-Evolving</x:v>
+      </x:c>
+      <x:c r="D59" s="146" t="str">
+        <x:v>GA/滚动升级</x:v>
+      </x:c>
+      <x:c r="E59" s="146" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F59" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G59" s="146" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H59" s="146" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="I59" s="146"/>
+      <x:c r="J59" s="146" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="K59" s="146" t="str">
+        <x:v>1,024K 上下文</x:v>
+      </x:c>
+      <x:c r="L59" s="146" t="str">
+        <x:v>缓存存储 ¥0.017/百万 Token/小时</x:v>
+      </x:c>
+      <x:c r="M59" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="N59" s="146" t="str">
+        <x:v>https://docs.volcengine.com/docs/82379/1544106?lang=zh</x:v>
+      </x:c>
+      <x:c r="O59" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="54" customHeight="1">
+      <x:c r="A60" s="146" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B60" s="146" t="str">
+        <x:v>阶跃星辰 StepFun</x:v>
+      </x:c>
+      <x:c r="C60" s="146" t="str">
+        <x:v>Step-3.7 Flash</x:v>
+      </x:c>
+      <x:c r="D60" s="146" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="E60" s="146" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F60" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G60" s="146" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="H60" s="146" t="n">
+        <x:v>0.27</x:v>
+      </x:c>
+      <x:c r="I60" s="146"/>
+      <x:c r="J60" s="146" t="n">
+        <x:v>8.1</x:v>
+      </x:c>
+      <x:c r="K60" s="146" t="str">
+        <x:v>256K；原生图像/视频理解</x:v>
+      </x:c>
+      <x:c r="L60" s="146" t="str">
+        <x:v>搜索与工具成本另计</x:v>
+      </x:c>
+      <x:c r="M60" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="N60" s="146" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
+      </x:c>
+      <x:c r="O60" s="146" t="str">
         <x:v>官方价格页</x:v>
       </x:c>
     </x:row>
@@ -7442,7 +8025,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raed858df767d44b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R308c72477ebe4fa9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8995,45 +9578,45 @@
         <x:v>DeepSeek</x:v>
       </x:c>
       <x:c r="C36" s="127" t="str">
-        <x:v>DeepSeek V4 Flash</x:v>
+        <x:v>DeepSeek V4.1 Flash</x:v>
       </x:c>
       <x:c r="D36" s="127" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="E36" s="128" t="n">
-        <x:v>1.5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F36" s="128" t="n">
-        <x:v>0.05</x:v>
+        <x:v>0.02</x:v>
       </x:c>
       <x:c r="G36" s="128" t="n">
-        <x:v>4.5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H36" s="129" t="n">
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="I36" s="130" t="n">
         <x:f>$B$4/1000000*($B$2*((1-$B$5)*E36+$B$5*IF(F36="",E36,F36))+$B$3*G36)*(1-$B$7)</x:f>
-        <x:v>438</x:v>
+        <x:v>341.20000000000005</x:v>
       </x:c>
       <x:c r="J36" s="130" t="n">
         <x:f>IF(D36="USD",I36*$B$6,I36)</x:f>
-        <x:v>438</x:v>
+        <x:v>341.20000000000005</x:v>
       </x:c>
       <x:c r="K36" s="130" t="n">
         <x:f>J36/$B$4*1000</x:f>
-        <x:v>4.38</x:v>
+        <x:v>3.4120000000000004</x:v>
       </x:c>
       <x:c r="L36" s="130" t="n">
         <x:f>IFERROR(J36/($B$4*H36),"")</x:f>
-        <x:v>0.0051529411764705884</x:v>
+        <x:v>0.004014117647058824</x:v>
       </x:c>
       <x:c r="M36" s="127" t="str">
         <x:f>IF(H36&lt;0.7,"先修质量",IF(L36&lt;0.01,"极低成本",IF(L36&lt;0.1,"低成本","需看价值")))</x:f>
         <x:v>极低成本</x:v>
       </x:c>
       <x:c r="N36" s="134" t="str">
-        <x:v>https://api-docs.deepseek.com/quick_start/pricing</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing/</x:v>
       </x:c>
       <x:c r="O36" s="127"/>
     </x:row>
@@ -10130,6 +10713,304 @@
       <x:c r="M59"/>
       <x:c r="N59"/>
       <x:c r="O59"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>GPT-5.6 Cyber</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E60" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F60" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="G60" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="H60" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I60" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E60+$B$5*IF(F60="",E60,F60))+$B$3*G60)*(1-$B$7)</x:f>
+        <x:v>5575</x:v>
+      </x:c>
+      <x:c r="J60" t="n">
+        <x:f>IF(D60="USD",I60*$B$6,I60)</x:f>
+        <x:v>40140</x:v>
+      </x:c>
+      <x:c r="K60" t="n">
+        <x:f>J60/$B$4*1000</x:f>
+        <x:v>401.4</x:v>
+      </x:c>
+      <x:c r="L60" t="n">
+        <x:f>IFERROR(J60/($B$4*H60),"")</x:f>
+        <x:v>0.4722352941176471</x:v>
+      </x:c>
+      <x:c r="M60" t="str">
+        <x:f>IF(H60&lt;0.7,"先修质量",IF(L60&lt;0.01,"极低成本",IF(L60&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>需看价值</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-cyber</x:v>
+      </x:c>
+      <x:c r="O60"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>GPT-Rosalind</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E61" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F61" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="G61" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H61" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I61" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E61+$B$5*IF(F61="",E61,F61))+$B$3*G61)*(1-$B$7)</x:f>
+        <x:v>1980</x:v>
+      </x:c>
+      <x:c r="J61" t="n">
+        <x:f>IF(D61="USD",I61*$B$6,I61)</x:f>
+        <x:v>14256</x:v>
+      </x:c>
+      <x:c r="K61" t="n">
+        <x:f>J61/$B$4*1000</x:f>
+        <x:v>142.56</x:v>
+      </x:c>
+      <x:c r="L61" t="n">
+        <x:f>IFERROR(J61/($B$4*H61),"")</x:f>
+        <x:v>0.16771764705882353</x:v>
+      </x:c>
+      <x:c r="M61" t="str">
+        <x:f>IF(H61&lt;0.7,"先修质量",IF(L61&lt;0.01,"极低成本",IF(L61&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>需看价值</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="O61"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>海外</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>Meta</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>Muse Spark 1.3</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="E62" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="F62" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="G62" t="n">
+        <x:v>4.25</x:v>
+      </x:c>
+      <x:c r="H62" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I62" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E62+$B$5*IF(F62="",E62,F62))+$B$3*G62)*(1-$B$7)</x:f>
+        <x:v>396.5</x:v>
+      </x:c>
+      <x:c r="J62" t="n">
+        <x:f>IF(D62="USD",I62*$B$6,I62)</x:f>
+        <x:v>2854.8</x:v>
+      </x:c>
+      <x:c r="K62" t="n">
+        <x:f>J62/$B$4*1000</x:f>
+        <x:v>28.548000000000002</x:v>
+      </x:c>
+      <x:c r="L62" t="n">
+        <x:f>IFERROR(J62/($B$4*H62),"")</x:f>
+        <x:v>0.03358588235294118</x:v>
+      </x:c>
+      <x:c r="M62" t="str">
+        <x:f>IF(H62&lt;0.7,"先修质量",IF(L62&lt;0.01,"极低成本",IF(L62&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>低成本</x:v>
+      </x:c>
+      <x:c r="N62" t="str">
+        <x:v>https://developer.meta.com/ai/products/muse-code/</x:v>
+      </x:c>
+      <x:c r="O62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>阿里云 / 通义千问 Qwen</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>Qwen3.8-Flash</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E63" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="F63"/>
+      <x:c r="G63" t="n">
+        <x:v>2.7</x:v>
+      </x:c>
+      <x:c r="H63" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I63" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E63+$B$5*IF(F63="",E63,F63))+$B$3*G63)*(1-$B$7)</x:f>
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="J63" t="n">
+        <x:f>IF(D63="USD",I63*$B$6,I63)</x:f>
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="K63" t="n">
+        <x:f>J63/$B$4*1000</x:f>
+        <x:v>2.9499999999999997</x:v>
+      </x:c>
+      <x:c r="L63" t="n">
+        <x:f>IFERROR(J63/($B$4*H63),"")</x:f>
+        <x:v>0.0034705882352941177</x:v>
+      </x:c>
+      <x:c r="M63" t="str">
+        <x:f>IF(H63&lt;0.7,"先修质量",IF(L63&lt;0.01,"极低成本",IF(L63&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>极低成本</x:v>
+      </x:c>
+      <x:c r="N63" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
+      </x:c>
+      <x:c r="O63"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>字节跳动 / 豆包 Seed</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>Seed-Evolving</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E64" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F64" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="G64" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="H64" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I64" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E64+$B$5*IF(F64="",E64,F64))+$B$3*G64)*(1-$B$7)</x:f>
+        <x:v>2412</x:v>
+      </x:c>
+      <x:c r="J64" t="n">
+        <x:f>IF(D64="USD",I64*$B$6,I64)</x:f>
+        <x:v>2412</x:v>
+      </x:c>
+      <x:c r="K64" t="n">
+        <x:f>J64/$B$4*1000</x:f>
+        <x:v>24.119999999999997</x:v>
+      </x:c>
+      <x:c r="L64" t="n">
+        <x:f>IFERROR(J64/($B$4*H64),"")</x:f>
+        <x:v>0.028376470588235295</x:v>
+      </x:c>
+      <x:c r="M64" t="str">
+        <x:f>IF(H64&lt;0.7,"先修质量",IF(L64&lt;0.01,"极低成本",IF(L64&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>低成本</x:v>
+      </x:c>
+      <x:c r="N64" t="str">
+        <x:v>https://docs.volcengine.com/docs/82379/1544106?lang=zh</x:v>
+      </x:c>
+      <x:c r="O64"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>阶跃星辰 StepFun</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>Step-3.7 Flash</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E65" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="F65" t="n">
+        <x:v>0.27</x:v>
+      </x:c>
+      <x:c r="G65" t="n">
+        <x:v>8.1</x:v>
+      </x:c>
+      <x:c r="H65" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I65" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E65+$B$5*IF(F65="",E65,F65))+$B$3*G65)*(1-$B$7)</x:f>
+        <x:v>610.2</x:v>
+      </x:c>
+      <x:c r="J65" t="n">
+        <x:f>IF(D65="USD",I65*$B$6,I65)</x:f>
+        <x:v>610.2</x:v>
+      </x:c>
+      <x:c r="K65" t="n">
+        <x:f>J65/$B$4*1000</x:f>
+        <x:v>6.102</x:v>
+      </x:c>
+      <x:c r="L65" t="n">
+        <x:f>IFERROR(J65/($B$4*H65),"")</x:f>
+        <x:v>0.007178823529411765</x:v>
+      </x:c>
+      <x:c r="M65" t="str">
+        <x:f>IF(H65&lt;0.7,"先修质量",IF(L65&lt;0.01,"极低成本",IF(L65&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>极低成本</x:v>
+      </x:c>
+      <x:c r="N65" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
+      </x:c>
+      <x:c r="O65"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -10143,7 +11024,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6abdd04caea4a9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6e468b7a4124d91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10399,22 +11280,22 @@
         <x:v>Anthropic</x:v>
       </x:c>
       <x:c r="D8" s="64" t="str">
-        <x:v>Claude 3.5 Haiku + Sonnet</x:v>
+        <x:v>Claude 3.5 Haiku（实时代码补全）+ Claude 3.5 Sonnet（架构解释与复杂代码）</x:v>
       </x:c>
       <x:c r="E8" s="64" t="str">
-        <x:v>低延迟补全、复杂代码聊天与安全开发</x:v>
+        <x:v>低延迟补全、IDE 对话、复杂代码生成与安全开发</x:v>
       </x:c>
       <x:c r="F8" s="64" t="str">
-        <x:v>功能交付快 20%-30%；初级开发者集成任务快 70%</x:v>
+        <x:v>功能开发速度提升 20%-30%；新开发者入职由数月缩短至数周；已导入 2,500 名开发者，计划增至 3,500 名</x:v>
       </x:c>
       <x:c r="G8" s="64" t="str">
         <x:v>A｜官方案例</x:v>
       </x:c>
       <x:c r="H8" s="64" t="str">
-        <x:v>自报指标，模型和工具链共同贡献</x:v>
+        <x:v>客户自报；模型、IDE 与内部工程流程共同贡献</x:v>
       </x:c>
       <x:c r="I8" s="64" t="str">
-        <x:v>2024-2025</x:v>
+        <x:v>2024-2026</x:v>
       </x:c>
       <x:c r="J8" s="136" t="str">
         <x:v>https://www.claude.com/customers/palo-alto-networks</x:v>
@@ -10751,19 +11632,19 @@
         <x:v>Meta</x:v>
       </x:c>
       <x:c r="D19" s="64" t="str">
-        <x:v>微调 Llama 3.1 70B/405B</x:v>
+        <x:v>微调 Llama 3.1 Instruct 70B / 405B</x:v>
       </x:c>
       <x:c r="E19" s="64" t="str">
         <x:v>企业代码助手</x:v>
       </x:c>
       <x:c r="F19" s="64" t="str">
-        <x:v>官方称单张 H100 可支持最多约 1,000 名工程师，突出低 TCO</x:v>
+        <x:v>官方称较可比模型成本效率高 90%、延迟低 3×，且准确率更高</x:v>
       </x:c>
       <x:c r="G19" s="64" t="str">
         <x:v>A｜Meta 官方案例</x:v>
       </x:c>
       <x:c r="H19" s="64" t="str">
-        <x:v>吞吐取决于上下文、量化、并发和补全长度</x:v>
+        <x:v>厂商比较；吞吐与成本取决于上下文、量化、并发和补全长度</x:v>
       </x:c>
       <x:c r="I19" s="64" t="str">
         <x:v>2024</x:v>
@@ -10783,13 +11664,13 @@
         <x:v>百度</x:v>
       </x:c>
       <x:c r="D20" s="64" t="str">
-        <x:v>文心大模型 + RAG（版本未披露）</x:v>
+        <x:v>百度智能云大模型 + RAG（版本未披露）</x:v>
       </x:c>
       <x:c r="E20" s="64" t="str">
         <x:v>游戏客服、问题分流</x:v>
       </x:c>
       <x:c r="F20" s="64" t="str">
-        <x:v>复杂问题路由能力提升 2.4×；SLA 提升 38.3 个百分点至 99.3%</x:v>
+        <x:v>复杂问题分流准确率提升 2.4×；SLA 达成率提升 38.3 个百分点至 99.3%</x:v>
       </x:c>
       <x:c r="G20" s="64" t="str">
         <x:v>B｜官方案例</x:v>
@@ -11026,6 +11907,38 @@
       </x:c>
       <x:c r="J27" s="137" t="str">
         <x:v>https://www.minimax.io/news/minimax-m25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="54" customHeight="1">
+      <x:c r="A28" s="146" t="str">
+        <x:v>供应链 Agent</x:v>
+      </x:c>
+      <x:c r="B28" s="146" t="str">
+        <x:v>Palantir Foundry</x:v>
+      </x:c>
+      <x:c r="C28" s="146" t="str">
+        <x:v>NVIDIA / Palantir</x:v>
+      </x:c>
+      <x:c r="D28" s="146" t="str">
+        <x:v>后训练 Nemotron 3.5 Lightning + Palantir Foundry</x:v>
+      </x:c>
+      <x:c r="E28" s="146" t="str">
+        <x:v>供应链分配与专家知识编码</x:v>
+      </x:c>
+      <x:c r="F28" s="146" t="str">
+        <x:v>受限任务开发基准 86.7%；对照 Nemotron Ultra 55.5%、原始 Lightning 17.5%</x:v>
+      </x:c>
+      <x:c r="G28" s="146" t="str">
+        <x:v>A｜NVIDIA 官方案例</x:v>
+      </x:c>
+      <x:c r="H28" s="146" t="str">
+        <x:v>后训练与 Palantir 工作流共同贡献；仅适用于文中受限任务，不外推全局模型优劣</x:v>
+      </x:c>
+      <x:c r="I28" s="146" t="str">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="J28" s="146" t="str">
+        <x:v>https://developer.nvidia.com/blog/from-wafer-out-to-first-token-codifying-supply-chain-expertise-with-nemotron-and-palantir-foundry/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11034,7 +11947,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re20631e52f9b49b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7295ce44d5f9436d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11139,7 +12052,7 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="C4" s="64" t="str">
-        <x:v>GPT-6 Astra / GPT-5.6；Claude Sonnet/Opus/Fable；Grok 4.6；Qwen Coder；DeepSeek V4；GLM-5.3；Kimi K2.7 Code；MiniMax M3</x:v>
+        <x:v>GPT-6 Astra / GPT-5.6；Claude；Grok 4.6；Muse Code；Qwen Coder；DeepSeek V4.1；GLM-5.3；Kimi Code K2.8；MiniMax M3</x:v>
       </x:c>
       <x:c r="D4" s="64" t="str">
         <x:v>代码库级修改、测试、终端与多文件工作</x:v>
@@ -11191,7 +12104,7 @@
         <x:v>高</x:v>
       </x:c>
       <x:c r="C6" s="64" t="str">
-        <x:v>GPT-5.6 Luna；Gemini Flash-Lite；Mistral Small 4；DeepSeek V4 Flash；Step Flash；ERNIE 4.5 Turbo；Hy3</x:v>
+        <x:v>GPT-5.6 Luna；Gemini Flash-Lite；Mistral Small 4；DeepSeek V4.1 Flash；Step-3.5 Flash；Qwen3.8 Flash；ERNIE 4.5 Turbo；Hy3</x:v>
       </x:c>
       <x:c r="D6" s="64" t="str">
         <x:v>分类、抽取、改写、简单问答、执行层子任务</x:v>
@@ -11217,7 +12130,7 @@
         <x:v>中高</x:v>
       </x:c>
       <x:c r="C7" s="64" t="str">
-        <x:v>Claude 5；GPT-6 Astra / GPT-5.6；Gemini；Qwen3.8；DeepSeek V4；GLM-5.3；Kimi K3；MiniMax M3</x:v>
+        <x:v>Claude 5；GPT-6 Astra / GPT-5.6；Gemini；Qwen3.8；DeepSeek V4.1；GLM-5.3；Kimi K3；MiniMax M3</x:v>
       </x:c>
       <x:c r="D7" s="64" t="str">
         <x:v>代码库、合同包、研究资料、多轮 Agent 历史</x:v>
@@ -11295,7 +12208,7 @@
         <x:v>中高</x:v>
       </x:c>
       <x:c r="C10" s="64" t="str">
-        <x:v>Grok Voice；OpenAI Realtime；Gemini Live；Amazon Nova Sonic；讯飞；MiniMax Speech</x:v>
+        <x:v>GPT-Live 1 / OpenAI Realtime；Grok Voice；Gemini Live；Amazon Nova Sonic；讯飞；MiniMax Speech</x:v>
       </x:c>
       <x:c r="D10" s="64" t="str">
         <x:v>电话客服、销售、车载、陪伴与实时翻译</x:v>
@@ -11423,7 +12336,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R539eb51245714128"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d736f9cfa9343e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11563,13 +12476,13 @@
         <x:v>GPT-6 Astra、当前产品与模型入口</x:v>
       </x:c>
       <x:c r="D13" s="95" t="str">
-        <x:v>https://developers.openai.com/api/docs/models/gpt-6-astra</x:v>
+        <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-cyber</x:v>
       </x:c>
       <x:c r="E13" s="88" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F13" s="89" t="str">
-        <x:v>【公开事实】当前目录与价格按查询日快照</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -11623,13 +12536,13 @@
         <x:v>Llama、Muse 系列与第一方 Model API</x:v>
       </x:c>
       <x:c r="D16" s="96" t="str">
-        <x:v>https://developer.meta.com/ai</x:v>
+        <x:v>https://developer.meta.com/ai/products/muse-code/</x:v>
       </x:c>
       <x:c r="E16" s="64" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F16" s="91" t="str">
-        <x:v>【公开事实】开放权重不等于零成本</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -11683,13 +12596,13 @@
         <x:v>Command A+ 与免费限速档</x:v>
       </x:c>
       <x:c r="D19" s="96" t="str">
-        <x:v>https://docs.cohere.com/docs/command-a-plus</x:v>
+        <x:v>https://docs.cohere.com/docs/models</x:v>
       </x:c>
       <x:c r="E19" s="64" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F19" s="91" t="str">
-        <x:v>【公开事实】适合把生成与检索组件组合评测</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -11703,13 +12616,13 @@
         <x:v>Bedrock 与 Claude Fable 5.1 可用性</x:v>
       </x:c>
       <x:c r="D20" s="96" t="str">
-        <x:v>https://aws.amazon.com/about-aws/whats-new/2026/09/claude-fable-5-1-aws/</x:v>
+        <x:v>https://aws.amazon.com/blogs/machine-learning/take-on-your-most-ambitious-work-with-gpt-6-astra-on-amazon-bedrock/</x:v>
       </x:c>
       <x:c r="E20" s="64" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F20" s="91" t="str">
-        <x:v>【公开事实】Bedrock 案例常使用第三方底模</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -11723,13 +12636,13 @@
         <x:v>MAI-Transcribe-2 与 Foundry Astra</x:v>
       </x:c>
       <x:c r="D21" s="96" t="str">
-        <x:v>https://microsoft.ai/news/introducing-mai-transcribe-2/</x:v>
+        <x:v>https://microsoft.ai/news/mai-transcribe-2-is-the-fastest-most-accurate-and-cheapest-speech-recognition-model-in-the-world/</x:v>
       </x:c>
       <x:c r="E21" s="64" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F21" s="91" t="str">
-        <x:v>【公开事实】MAI 生产 API 价未统一公开</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -11803,13 +12716,13 @@
         <x:v>官网、当前产品与模型入口</x:v>
       </x:c>
       <x:c r="D25" s="96" t="str">
-        <x:v>https://seed.bytedance.com/</x:v>
+        <x:v>https://docs.volcengine.com/docs/82379/1544106?lang=zh</x:v>
       </x:c>
       <x:c r="E25" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F25" s="91" t="str">
-        <x:v>【公开事实】活动/节省计划价需与刊例价分开</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -11863,13 +12776,13 @@
         <x:v>DeepSeek V4 峰谷与缓存价格</x:v>
       </x:c>
       <x:c r="D28" s="96" t="str">
-        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing/</x:v>
       </x:c>
       <x:c r="E28" s="64" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F28" s="91" t="str">
-        <x:v>【公开事实】缓存命中价格极低但不能假设必定命中</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -11883,13 +12796,13 @@
         <x:v>官网、当前产品与模型入口</x:v>
       </x:c>
       <x:c r="D29" s="96" t="str">
-        <x:v>https://platform.kimi.com/</x:v>
+        <x:v>https://www.kimi.com/code/docs/kimi-code/whats-new.html</x:v>
       </x:c>
       <x:c r="E29" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F29" s="91" t="str">
-        <x:v>【公开事实】国内外 API 币种与价格页可能不同</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -11986,10 +12899,10 @@
         <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
       </x:c>
       <x:c r="E34" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F34" s="91" t="str">
-        <x:v>【公开事实】具体模型可用性以平台目录为准</x:v>
+        <x:v>官方页面</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -13897,16 +14810,16 @@
         <x:v>价格</x:v>
       </x:c>
       <x:c r="B130" s="64" t="str">
-        <x:v>DeepSeek｜DeepSeek V4 Flash</x:v>
+        <x:v>DeepSeek｜DeepSeek V4.1 Flash</x:v>
       </x:c>
       <x:c r="C130" s="64" t="str">
-        <x:v>当前价格与计费条件</x:v>
+        <x:v>闲时 ¥1/¥0.02/¥4；忙时 ¥2/¥0.04/¥8</x:v>
       </x:c>
       <x:c r="D130" s="96" t="str">
         <x:v>https://api-docs.deepseek.com/quick_start/pricing</x:v>
       </x:c>
       <x:c r="E130" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F130" s="91" t="str">
         <x:v>官方价格页</x:v>
@@ -14020,13 +14933,13 @@
         <x:v>Palo Alto Networks</x:v>
       </x:c>
       <x:c r="C136" s="64" t="str">
-        <x:v>Claude 3.5 Haiku + Sonnet｜低延迟补全、复杂代码聊天与安全开发</x:v>
+        <x:v>Claude 3.5 Haiku + Sonnet｜代码补全、复杂代码与开发者入职</x:v>
       </x:c>
       <x:c r="D136" s="96" t="str">
         <x:v>https://www.anthropic.com/customers/palo-alto-networks</x:v>
       </x:c>
       <x:c r="E136" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F136" s="91" t="str">
         <x:v>A｜官方案例</x:v>
@@ -14226,7 +15139,7 @@
         <x:v>https://ai.meta.com/blog/codeium-ai-coding-assistant-llama/</x:v>
       </x:c>
       <x:c r="E146" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F146" s="91" t="str">
         <x:v>A｜Meta 官方案例</x:v>
@@ -14240,13 +15153,13 @@
         <x:v>三七互娱</x:v>
       </x:c>
       <x:c r="C147" s="64" t="str">
-        <x:v>文心大模型 + RAG（版本未披露）｜游戏客服、问题分流</x:v>
+        <x:v>百度智能云大模型 + RAG｜游戏客服与问题分流</x:v>
       </x:c>
       <x:c r="D147" s="96" t="str">
         <x:v>https://cloud.baidu.com/customer/case/sanqihuyu.html</x:v>
       </x:c>
       <x:c r="E147" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F147" s="91" t="str">
         <x:v>B｜官方案例</x:v>
@@ -14480,13 +15393,13 @@
         <x:v>MiniMax｜MiniMax M3 ≤512K</x:v>
       </x:c>
       <x:c r="C159" t="str">
-        <x:v>当前价格与计费条件</x:v>
+        <x:v>永久五折价格与计费条件</x:v>
       </x:c>
       <x:c r="D159" t="str">
         <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
       </x:c>
       <x:c r="E159" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F159" t="str">
         <x:v>官方价格页</x:v>
@@ -14520,16 +15433,396 @@
         <x:v>MiniMax｜MiniMax M3 &gt;512K</x:v>
       </x:c>
       <x:c r="C161" t="str">
-        <x:v>当前价格与计费条件</x:v>
+        <x:v>永久五折价格与计费条件</x:v>
       </x:c>
       <x:c r="D161" t="str">
         <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
       </x:c>
       <x:c r="E161" t="str">
-        <x:v>2026-09-07</x:v>
+        <x:v>2026-09-14</x:v>
       </x:c>
       <x:c r="F161" t="str">
         <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="36" customHeight="1">
+      <x:c r="A162" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B162" s="146" t="str">
+        <x:v>OpenAI｜GPT Image 2.5 Sunburst / Flare</x:v>
+      </x:c>
+      <x:c r="C162" s="146" t="str">
+        <x:v>2026-09-08｜图像生成与编辑；新增 xhigh / max 质量档</x:v>
+      </x:c>
+      <x:c r="D162" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="E162" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F162" s="146" t="str">
+        <x:v>公开事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="36" customHeight="1">
+      <x:c r="A163" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B163" s="146" t="str">
+        <x:v>OpenAI｜GPT-Rosalind</x:v>
+      </x:c>
+      <x:c r="C163" s="146" t="str">
+        <x:v>2026-09-08｜trusted access GA；获批内部生命科学研究</x:v>
+      </x:c>
+      <x:c r="D163" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="E163" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F163" s="146" t="str">
+        <x:v>公开事实2026-10-05 起计费</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="36" customHeight="1">
+      <x:c r="A164" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B164" s="146" t="str">
+        <x:v>OpenAI｜GPT-Live 1</x:v>
+      </x:c>
+      <x:c r="C164" s="146" t="str">
+        <x:v>2026-09-10｜全双工语音 API GA；会话 $0.05/分钟</x:v>
+      </x:c>
+      <x:c r="D164" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="E164" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F164" s="146" t="str">
+        <x:v>公开事实后端模型与工具另计</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="36" customHeight="1">
+      <x:c r="A165" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B165" s="146" t="str">
+        <x:v>OpenAI｜GPT-5.4-Cyber → GPT-5.6 Cyber</x:v>
+      </x:c>
+      <x:c r="C165" s="146" t="str">
+        <x:v>2026-09-11 / 10-01｜旧版宣布弃用，10 月 1 日移除</x:v>
+      </x:c>
+      <x:c r="D165" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/deprecations</x:v>
+      </x:c>
+      <x:c r="E165" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F165" s="146" t="str">
+        <x:v>公开事实需迁移；GPT-5.6 Cyber 单独审批</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="36" customHeight="1">
+      <x:c r="A166" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B166" s="146" t="str">
+        <x:v>Cohere｜North Small Translate 1.0</x:v>
+      </x:c>
+      <x:c r="C166" s="146" t="str">
+        <x:v>2026-09-09｜50+ 语言翻译；218B 总参数 / 25B active MoE；16K</x:v>
+      </x:c>
+      <x:c r="D166" s="146" t="str">
+        <x:v>https://docs.cohere.com/v2/changelog</x:v>
+      </x:c>
+      <x:c r="E166" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F166" s="146" t="str">
+        <x:v>公开事实免费层仅评估，生产需商业许可</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="36" customHeight="1">
+      <x:c r="A167" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B167" s="146" t="str">
+        <x:v>Amazon / AWS｜GPT-6 Astra on Bedrock</x:v>
+      </x:c>
+      <x:c r="C167" s="146" t="str">
+        <x:v>2026-09-08｜在 Amazon Bedrock GA</x:v>
+      </x:c>
+      <x:c r="D167" s="146" t="str">
+        <x:v>https://aws.amazon.com/blogs/machine-learning/take-on-your-most-ambitious-work-with-gpt-6-astra-on-amazon-bedrock/</x:v>
+      </x:c>
+      <x:c r="E167" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F167" s="146" t="str">
+        <x:v>公开事实｜地区与精确价格需控制台复核</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="36" customHeight="1">
+      <x:c r="A168" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B168" s="146" t="str">
+        <x:v>DeepSeek｜DeepSeek V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="C168" s="146" t="str">
+        <x:v>2026-09-10｜原生视觉、1M 上下文、384K 最大输出；旧 V4 Flash 临时兼容路由</x:v>
+      </x:c>
+      <x:c r="D168" s="146" t="str">
+        <x:v>https://api-docs.deepseek.com/zh-cn/updates/</x:v>
+      </x:c>
+      <x:c r="E168" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F168" s="146" t="str">
+        <x:v>公开事实模型 ID 为 deepseek-flash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="36" customHeight="1">
+      <x:c r="A169" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B169" s="146" t="str">
+        <x:v>字节跳动 / 豆包 Seed｜Seed-Evolving</x:v>
+      </x:c>
+      <x:c r="C169" s="146" t="str">
+        <x:v>2026-09-09｜滚动升级模型 ID；1,024K 上下文、256K 最大输出</x:v>
+      </x:c>
+      <x:c r="D169" s="146" t="str">
+        <x:v>https://docs.volcengine.com/docs/82379/2549861?lang=zh</x:v>
+      </x:c>
+      <x:c r="E169" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F169" s="146" t="str">
+        <x:v>公开事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="36" customHeight="1">
+      <x:c r="A170" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B170" s="146" t="str">
+        <x:v>月之暗面 / Kimi｜Kimi Code K2.8 Preview</x:v>
+      </x:c>
+      <x:c r="C170" s="146" t="str">
+        <x:v>2026-09-11｜全量上线；全会员档支持 1M 上下文</x:v>
+      </x:c>
+      <x:c r="D170" s="146" t="str">
+        <x:v>https://www.kimi.com/code/docs/kimi-code/whats-new.html</x:v>
+      </x:c>
+      <x:c r="E170" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F170" s="146" t="str">
+        <x:v>公开事实模型 ID 仍为 kimi-for-coding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="36" customHeight="1">
+      <x:c r="A171" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B171" s="146" t="str">
+        <x:v>腾讯云 TokenHub｜DeepSeek V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="C171" s="146" t="str">
+        <x:v>2026-09-10｜新增原厂模型并沿用原厂闲时 / 忙时价格</x:v>
+      </x:c>
+      <x:c r="D171" s="146" t="str">
+        <x:v>https://cloud.tencent.com/document/product/1823/130675</x:v>
+      </x:c>
+      <x:c r="E171" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F171" s="146" t="str">
+        <x:v>公开事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="36" customHeight="1">
+      <x:c r="A172" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B172" s="146" t="str">
+        <x:v>阿里云百炼｜DeepSeek V4.1 Flash</x:v>
+      </x:c>
+      <x:c r="C172" s="146" t="str">
+        <x:v>2026-09-13｜新增原厂模型托管</x:v>
+      </x:c>
+      <x:c r="D172" s="146" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/newly-released-models</x:v>
+      </x:c>
+      <x:c r="E172" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F172" s="146" t="str">
+        <x:v>公开事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="36" customHeight="1">
+      <x:c r="A173" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B173" s="146" t="str">
+        <x:v>阶跃星辰 StepFun｜step-2x-large / step-image-edit-2 / step-1x-edit</x:v>
+      </x:c>
+      <x:c r="C173" s="146" t="str">
+        <x:v>2026-10-10 / 已退役｜前两者计划 10 月 10 日退役；step-1x-edit 已退役</x:v>
+      </x:c>
+      <x:c r="D173" s="146" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/image-offline-notice</x:v>
+      </x:c>
+      <x:c r="E173" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F173" s="146" t="str">
+        <x:v>公开事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="36" customHeight="1">
+      <x:c r="A174" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B174" s="146" t="str">
+        <x:v>OpenAI｜GPT-5.6 Cyber</x:v>
+      </x:c>
+      <x:c r="C174" s="146" t="str">
+        <x:v>12.5/1.25/75 USD/百万tokens</x:v>
+      </x:c>
+      <x:c r="D174" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-cyber</x:v>
+      </x:c>
+      <x:c r="E174" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F174" s="146" t="str">
+        <x:v>官方模型与价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="36" customHeight="1">
+      <x:c r="A175" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B175" s="146" t="str">
+        <x:v>OpenAI｜GPT-Rosalind</x:v>
+      </x:c>
+      <x:c r="C175" s="146" t="str">
+        <x:v>5/0.5/25 USD/百万tokens</x:v>
+      </x:c>
+      <x:c r="D175" s="146" t="str">
+        <x:v>https://developers.openai.com/api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="E175" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F175" s="146" t="str">
+        <x:v>官方变更日志</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="36" customHeight="1">
+      <x:c r="A176" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B176" s="146" t="str">
+        <x:v>Meta｜Muse Spark 1.3</x:v>
+      </x:c>
+      <x:c r="C176" s="146" t="str">
+        <x:v>1.25/0.15/4.25 USD/百万tokens</x:v>
+      </x:c>
+      <x:c r="D176" s="146" t="str">
+        <x:v>https://developer.meta.com/ai/products/muse-code/</x:v>
+      </x:c>
+      <x:c r="E176" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F176" s="146" t="str">
+        <x:v>官方产品页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="36" customHeight="1">
+      <x:c r="A177" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B177" s="146" t="str">
+        <x:v>阿里云 / 通义千问 Qwen｜Qwen3.8-Flash</x:v>
+      </x:c>
+      <x:c r="C177" s="146" t="str">
+        <x:v>0.8/—/2.7 CNY/百万tokens</x:v>
+      </x:c>
+      <x:c r="D177" s="146" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
+      </x:c>
+      <x:c r="E177" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F177" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="36" customHeight="1">
+      <x:c r="A178" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B178" s="146" t="str">
+        <x:v>字节跳动 / 豆包 Seed｜Seed-Evolving</x:v>
+      </x:c>
+      <x:c r="C178" s="146" t="str">
+        <x:v>6/1.2/30 CNY/百万tokens</x:v>
+      </x:c>
+      <x:c r="D178" s="146" t="str">
+        <x:v>https://docs.volcengine.com/docs/82379/1544106?lang=zh</x:v>
+      </x:c>
+      <x:c r="E178" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F178" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="36" customHeight="1">
+      <x:c r="A179" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B179" s="146" t="str">
+        <x:v>阶跃星辰 StepFun｜Step-3.7 Flash</x:v>
+      </x:c>
+      <x:c r="C179" s="146" t="str">
+        <x:v>1.35/0.27/8.1 CNY/百万tokens</x:v>
+      </x:c>
+      <x:c r="D179" s="146" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
+      </x:c>
+      <x:c r="E179" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F179" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="36" customHeight="1">
+      <x:c r="A180" s="146" t="str">
+        <x:v>应用案例</x:v>
+      </x:c>
+      <x:c r="B180" s="146" t="str">
+        <x:v>Palantir Foundry</x:v>
+      </x:c>
+      <x:c r="C180" s="146" t="str">
+        <x:v>Nemotron 3.5 Lightning + Palantir Foundry｜供应链分配与专家知识编码</x:v>
+      </x:c>
+      <x:c r="D180" s="146" t="str">
+        <x:v>https://developer.nvidia.com/blog/from-wafer-out-to-first-token-codifying-supply-chain-expertise-with-nemotron-and-palantir-foundry/</x:v>
+      </x:c>
+      <x:c r="E180" s="146" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="F180" s="146" t="str">
+        <x:v>A｜NVIDIA 官方案例</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14538,7 +15831,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27cbe2e31c74499e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf97678a9b73454f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
data: refresh models and pricing for 2026-09-21
</commit_message>
<xml_diff>
--- a/public/AI模型厂商全景_2023-2026.xlsx
+++ b/public/AI模型厂商全景_2023-2026.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rd01a4dee867144c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="厂商地图" sheetId="2" r:id="Rc76cd3d5ec954741"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型时间轴" sheetId="3" r:id="Radcf04a74a444c96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前定价" sheetId="4" r:id="R0b00338896624fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本计算器" sheetId="5" r:id="R5b0d104946be471b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用案例" sheetId="6" r:id="R40a6e509ba1b4ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景选型" sheetId="7" r:id="R3407b46b6c444fd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料来源" sheetId="8" r:id="Rc81f718795e74ff7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Raeb40d54464140fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="厂商地图" sheetId="2" r:id="R99ad2fb1924848f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型时间轴" sheetId="3" r:id="Rf23f4a4a9c464560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前定价" sheetId="4" r:id="R1d4badf09e124805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成本计算器" sheetId="5" r:id="Rc386f314934b425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="应用案例" sheetId="6" r:id="R2c3c3ca5d7514dcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="场景选型" sheetId="7" r:id="R2b46578effde42b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料来源" sheetId="8" r:id="Re0db60aefb8a47fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -137,7 +137,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -187,6 +187,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF9E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCDEFFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCDF5D6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -336,7 +346,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="147">
+  <x:cellXfs count="149">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -668,6 +678,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1069,7 +1085,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
-        <x:v>研究日：2026-09-14｜范围：24 家代表厂商｜价格与产品为查询日快照，采购前请复核来源</x:v>
+        <x:v>研究日：2026-09-21｜范围：24 家代表厂商｜价格与产品为查询日快照，采购前请复核来源</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -1095,19 +1111,19 @@
         <x:v>时间轴节点</x:v>
       </x:c>
       <x:c r="E4" s="15" t="n">
-        <x:v>108</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="G4" s="14" t="str">
         <x:v>当前价格行</x:v>
       </x:c>
       <x:c r="H4" s="15" t="n">
-        <x:v>58</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="J4" s="14" t="str">
         <x:v>公开案例</x:v>
       </x:c>
       <x:c r="K4" s="15" t="n">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1496,7 +1512,7 @@
         <x:v>证据/限制</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="54" customHeight="1">
+    <x:row r="3" ht="70" customHeight="1">
       <x:c r="A3" s="87" t="str">
         <x:v>海外</x:v>
       </x:c>
@@ -1507,10 +1523,10 @@
         <x:v>从 GPT-4 的多模态能力，演进到 GPT-4o 的实时多模态、o1 的推理范式、GPT-5/5.6 的统一推理与 Agent 工具栈；2026-09 又推出 Astra、GPT-Live、Image 2.5、Rosalind 与 Cyber 专业模型。</x:v>
       </x:c>
       <x:c r="D3" s="88" t="str">
-        <x:v>GPT-6 Astra；GPT-5.6 Sol / Terra / Luna / Cyber；GPT-Live 1；GPT Image 2.5</x:v>
+        <x:v>GPT-6 Astra / Astra Law；GPT-5.6 Sol / Terra / Luna / Cyber；GPT-Live 1；GPT Image 2.5</x:v>
       </x:c>
       <x:c r="E3" s="88" t="str">
-        <x:v>ChatGPT、Responses API、Codex、Sora、Daybreak</x:v>
+        <x:v>ChatGPT、Responses API、Codex、Sora、Daybreak；Astra Law 仅 Trusted Access</x:v>
       </x:c>
       <x:c r="F3" s="88" t="str">
         <x:v>复杂推理、代码、工具调用、计算机使用、多模态</x:v>
@@ -1531,7 +1547,7 @@
         <x:v>https://developers.openai.com/api/docs/models/gpt-5.6-cyber</x:v>
       </x:c>
       <x:c r="L3" s="89" t="str">
-        <x:v>【公开事实】Cyber 需 Daybreak 单独审批；&gt;272K 输入/缓存 2×、输出 1.5×</x:v>
+        <x:v>【公开事实】Astra Law API 尚未开放；Cyber 需 Daybreak 单独审批</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
@@ -1572,7 +1588,7 @@
         <x:v>【公开事实】Fable 缓存写入与 US-only inference、Batch 档需单独核算</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="54" customHeight="1">
+    <x:row r="5" ht="70" customHeight="1">
       <x:c r="A5" s="90" t="str">
         <x:v>海外</x:v>
       </x:c>
@@ -1583,7 +1599,7 @@
         <x:v>以 Gemini 1 建立原生多模态路线，Gemini 1.5 扩展长上下文，2.x/3.x 强化推理、搜索与 Agent；2026-09 推出 3.8 Flash 与 Lyria 3.5。</x:v>
       </x:c>
       <x:c r="D5" s="64" t="str">
-        <x:v>Gemini 3.8 Flash / 3.7 Flash / 3.5 Flash-Lite；Lyria 3.5；Gemma</x:v>
+        <x:v>Gemini 3.8 Flash / Live；Antigravity Preview 09-2026；Lyria 3.5；Gemma</x:v>
       </x:c>
       <x:c r="E5" s="64" t="str">
         <x:v>Gemini、AI Studio、Vertex AI、Workspace、Android/Pixel</x:v>
@@ -1648,7 +1664,7 @@
         <x:v>【公开事实】Muse Spark contributor 档需允许数据用于改进产品；开放权重与第一方 API 为不同成本口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="54" customHeight="1">
+    <x:row r="7" ht="70" customHeight="1">
       <x:c r="A7" s="90" t="str">
         <x:v>海外</x:v>
       </x:c>
@@ -1659,7 +1675,7 @@
         <x:v>从 Grok 1 的实时信息与 X 数据差异化，演进到 Grok 3/4 的推理与代码，再到 Grok 4.6、Voice、Imagine 与 Build。</x:v>
       </x:c>
       <x:c r="D7" s="64" t="str">
-        <x:v>Grok 4.6；Grok Voice Think Fast 2.0；Imagine 2.0</x:v>
+        <x:v>Grok 4.6；Grok Voice Transcribe 2.0；Imagine 2.0</x:v>
       </x:c>
       <x:c r="E7" s="64" t="str">
         <x:v>Grok、Grok Build、Grok Voice、Imagine、X</x:v>
@@ -1876,7 +1892,7 @@
         <x:v>【公开事实】应测算 GPU 利用率与运维 TCO</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="54" customHeight="1">
+    <x:row r="13" ht="70" customHeight="1">
       <x:c r="A13" s="90" t="str">
         <x:v>国内</x:v>
       </x:c>
@@ -1887,7 +1903,7 @@
         <x:v>从 Qwen-7B/VL 开源起步，形成通用、代码、视觉、音频、数学的开放生态；Qwen3 后强化混合思考和 Agent。</x:v>
       </x:c>
       <x:c r="D13" s="64" t="str">
-        <x:v>Qwen3.8-Max / Qwen3-Max / Qwen3-Coder；开放 Qwen 系列</x:v>
+        <x:v>Qwen3.8 Max / Flash / Omni Flash；Qwen Coder；VL</x:v>
       </x:c>
       <x:c r="E13" s="64" t="str">
         <x:v>千问、Qwen Chat、QwenWork、阿里云百炼、钉钉/通义生态</x:v>
@@ -1902,7 +1918,7 @@
         <x:v>百炼 API、开源自建、专属部署</x:v>
       </x:c>
       <x:c r="I13" s="64" t="str">
-        <x:v>Qwen3.8-Max $12/$36；Qwen3.8-Flash ¥0.8/¥2.7；Qwen3-Max ¥2.5/¥10</x:v>
+        <x:v>Qwen3.8 Max ≤1M ¥12/¥36；Omni Flash ¥0.8/¥2.7（输入/输出，CNY/百万tokens）</x:v>
       </x:c>
       <x:c r="J13" s="64" t="str">
         <x:v>中文 Agent、代码、企业知识、私有化、底模微调</x:v>
@@ -2028,7 +2044,7 @@
         <x:v>【公开事实】Hy4 为 Preview；原混元售卖入口逐步迁移 TokenHub</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="54" customHeight="1">
+    <x:row r="17" ht="70" customHeight="1">
       <x:c r="A17" s="90" t="str">
         <x:v>国内</x:v>
       </x:c>
@@ -2039,7 +2055,7 @@
         <x:v>以 ChatGLM 开源生态和 BigModel MaaS 切入，GLM-4.5 后重点转向代码、Agent 与长周期工程任务。</x:v>
       </x:c>
       <x:c r="D17" s="64" t="str">
-        <x:v>GLM-5.3 / 5.2；GLM-5V-Turbo；GLM-4.7-FlashX</x:v>
+        <x:v>GLM-5.3；GLM-5.3-Flash；GLM Coding</x:v>
       </x:c>
       <x:c r="E17" s="64" t="str">
         <x:v>智谱清言、AutoGLM、GLM Coding Plan、开放平台</x:v>
@@ -2054,7 +2070,7 @@
         <x:v>BigModel API、私有化、代码订阅</x:v>
       </x:c>
       <x:c r="I17" s="64" t="str">
-        <x:v>GLM-5.3 ¥8/¥28，缓存 ¥2；GLM-4.7-FlashX ¥0.5/¥3</x:v>
+        <x:v>GLM-5.3 ¥8/¥28；5.3-Flash 标准 ¥0.8/¥2.8（输入/输出，CNY/百万tokens）</x:v>
       </x:c>
       <x:c r="J17" s="64" t="str">
         <x:v>代码 Agent、企业知识库、工单/合同、视觉操作</x:v>
@@ -2063,10 +2079,10 @@
         <x:v>https://bigmodel.cn/pricing</x:v>
       </x:c>
       <x:c r="L17" s="91" t="str">
-        <x:v>【公开事实】免费模型受配额/稳定性条件限制</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="54" customHeight="1">
+        <x:v>【公开事实】Flash 限时五折未披露截止日，标准价与促销价分开</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="70" customHeight="1">
       <x:c r="A18" s="90" t="str">
         <x:v>国内</x:v>
       </x:c>
@@ -2092,7 +2108,7 @@
         <x:v>第一方 API、自建、云平台托管</x:v>
       </x:c>
       <x:c r="I18" s="64" t="str">
-        <x:v>V4.1 Flash 闲时 ¥1/¥4，缓存 ¥0.02；忙时 ¥2/¥8，缓存 ¥0.04</x:v>
+        <x:v>V4.1 Flash 闲时 ¥1/¥4；V4 Pro 闲时 ¥4.5/¥13.5；忙时另计（CNY/百万tokens）</x:v>
       </x:c>
       <x:c r="J18" s="64" t="str">
         <x:v>低成本 Agent、代码、推理、底模蒸馏、私有化</x:v>
@@ -2142,7 +2158,7 @@
         <x:v>【公开事实】Kimi Code 模型 ID 不变；全会员档支持 1M 上下文</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="54" customHeight="1">
+    <x:row r="20" ht="70" customHeight="1">
       <x:c r="A20" s="90" t="str">
         <x:v>国内</x:v>
       </x:c>
@@ -2153,7 +2169,7 @@
         <x:v>从多模态和社交/陪伴产品扩展到超长上下文、推理与 Agent Coding，同时保留海螺视频、语音、音乐能力。</x:v>
       </x:c>
       <x:c r="D20" s="64" t="str">
-        <x:v>MiniMax M3 / M2.7；Hailuo 2.3；Speech/Music</x:v>
+        <x:v>MiniMax M3 / M2.7；H3 视频；Speech</x:v>
       </x:c>
       <x:c r="E20" s="64" t="str">
         <x:v>MiniMax Agent、海螺 AI、开放平台、Talkie</x:v>
@@ -2168,13 +2184,13 @@
         <x:v>API、订阅 Token Plan、专属部署</x:v>
       </x:c>
       <x:c r="I20" s="64" t="str">
-        <x:v>M3 ≤512K 永久五折 ¥2.1/¥8.4；M2.7 ¥2.1/¥8.4</x:v>
+        <x:v>M3 ≤512K 永久五折 ¥2.1/¥8.4（百万tokens）；H3 768P 输出 ¥0.50/秒，输入另计</x:v>
       </x:c>
       <x:c r="J20" s="64" t="str">
         <x:v>Agent、代码、Office 交付、视频/语音、角色互动</x:v>
       </x:c>
       <x:c r="K20" s="96" t="str">
-        <x:v>https://platform.minimaxi.com/docs/guides/pricing-paygo</x:v>
+        <x:v>https://platform.minimax.cn/docs/guides/pricing-paygo</x:v>
       </x:c>
       <x:c r="L20" s="91" t="str">
         <x:v>【公开事实】M3 永久五折；高速版、长上下文与 Token Plan 另计</x:v>
@@ -2294,7 +2310,7 @@
         <x:v>【公开事实】Beta 免费额度与生产 SLA、长期定价需分开看</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="54" customHeight="1">
+    <x:row r="24" ht="70" customHeight="1">
       <x:c r="A24" s="90" t="str">
         <x:v>国内</x:v>
       </x:c>
@@ -2305,7 +2321,7 @@
         <x:v>从 Step-1/1V/2 的通用和多模态，发展到 Step-3/3.5/3.7 Flash 的高吞吐 Agent 与本地部署路线。</x:v>
       </x:c>
       <x:c r="D24" s="64" t="str">
-        <x:v>Step-3.7 Flash；Step-3.5 Flash；Step Audio</x:v>
+        <x:v>Step 5 Preview；Step-3.7 Flash；Step Audio</x:v>
       </x:c>
       <x:c r="E24" s="64" t="str">
         <x:v>跃问、StepFun 开放平台、Agent/MCP 示例</x:v>
@@ -2320,7 +2336,7 @@
         <x:v>API、自建、本地工作站/DGX</x:v>
       </x:c>
       <x:c r="I24" s="64" t="str">
-        <x:v>Step-3.7 Flash ¥1.35/¥8.1，缓存 ¥0.27；Step-3.5 Flash ¥0.7/¥2.1</x:v>
+        <x:v>Step 5 Preview ¥7/¥20；Step-3.7 Flash ¥1.35/¥8.1（输入/输出，CNY/百万tokens）</x:v>
       </x:c>
       <x:c r="J24" s="64" t="str">
         <x:v>低成本 Agent、MCP 工具链、多模态、私有部署</x:v>
@@ -2329,7 +2345,7 @@
         <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
       </x:c>
       <x:c r="L24" s="91" t="str">
-        <x:v>【公开事实】Step-3.7 Flash 256K，原生图像/视频理解；具体首发日待核</x:v>
+        <x:v>【公开事实】Step 5 仍为 Preview；开放权重计划 2026-10-15</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
@@ -2414,7 +2430,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf4a0077e4a4f63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd19b302691a433a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5293,13 +5309,143 @@
         <x:v>【公开事实】</x:v>
       </x:c>
     </x:row>
+    <x:row r="111" ht="68" customHeight="1">
+      <x:c r="A111" s="147" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B111" s="147" t="str">
+        <x:v>Google DeepMind</x:v>
+      </x:c>
+      <x:c r="C111" s="147" t="str">
+        <x:v>2026-09-15</x:v>
+      </x:c>
+      <x:c r="D111" s="147" t="str">
+        <x:v>Gemini 3.8 Live / Extended Thinking</x:v>
+      </x:c>
+      <x:c r="E111" s="147" t="str">
+        <x:v>两个实时语音模型转 GA</x:v>
+      </x:c>
+      <x:c r="F111" s="147" t="str">
+        <x:v>Gemini Live API</x:v>
+      </x:c>
+      <x:c r="G111" s="147" t="str">
+        <x:v>https://ai.google.dev/gemini-api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="H111" s="147" t="str">
+        <x:v>【公开事实】</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="68" customHeight="1">
+      <x:c r="A112" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B112" s="146" t="str">
+        <x:v>Google DeepMind</x:v>
+      </x:c>
+      <x:c r="C112" s="146" t="str">
+        <x:v>2026-09-17 / 10-05</x:v>
+      </x:c>
+      <x:c r="D112" s="146" t="str">
+        <x:v>Antigravity Preview 09-2026</x:v>
+      </x:c>
+      <x:c r="E112" s="146" t="str">
+        <x:v>9 月版发布；05-2026 旧版已弃用，计划 10 月 5 日停用</x:v>
+      </x:c>
+      <x:c r="F112" s="146" t="str">
+        <x:v>Gemini API</x:v>
+      </x:c>
+      <x:c r="G112" s="146" t="str">
+        <x:v>https://ai.google.dev/gemini-api/docs/deprecations</x:v>
+      </x:c>
+      <x:c r="H112" s="146" t="str">
+        <x:v>【公开事实】旧版尚未退役</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="68" customHeight="1">
+      <x:c r="A113" s="147" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B113" s="147" t="str">
+        <x:v>xAI / SpaceXAI</x:v>
+      </x:c>
+      <x:c r="C113" s="147" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="D113" s="147" t="str">
+        <x:v>grok-voice-transcribe-2.0</x:v>
+      </x:c>
+      <x:c r="E113" s="147" t="str">
+        <x:v>新版语音转写上线；默认仍为 1.0</x:v>
+      </x:c>
+      <x:c r="F113" s="147" t="str">
+        <x:v>xAI Voice API</x:v>
+      </x:c>
+      <x:c r="G113" s="147" t="str">
+        <x:v>https://docs.x.ai/developers/release-notes</x:v>
+      </x:c>
+      <x:c r="H113" s="147" t="str">
+        <x:v>【公开事实】</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="68" customHeight="1">
+      <x:c r="A114" s="146" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B114" s="146" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="C114" s="146" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="D114" s="146" t="str">
+        <x:v>GPT-6 Astra Law</x:v>
+      </x:c>
+      <x:c r="E114" s="146" t="str">
+        <x:v>法律搜索与指令组合系统；获选机构 Trusted Access，API 即将推出</x:v>
+      </x:c>
+      <x:c r="F114" s="146" t="str">
+        <x:v>ChatGPT / Codex</x:v>
+      </x:c>
+      <x:c r="G114" s="146" t="str">
+        <x:v>https://openai.com/index/astra-for-law/</x:v>
+      </x:c>
+      <x:c r="H114" s="146" t="str">
+        <x:v>【公开事实】非公开 API GA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="68" customHeight="1">
+      <x:c r="A115" s="147" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B115" s="147" t="str">
+        <x:v>阶跃星辰 StepFun</x:v>
+      </x:c>
+      <x:c r="C115" s="147" t="str">
+        <x:v>2026-09（具体日未披露）</x:v>
+      </x:c>
+      <x:c r="D115" s="147" t="str">
+        <x:v>Step 5 Preview</x:v>
+      </x:c>
+      <x:c r="E115" s="147" t="str">
+        <x:v>1M 上下文、64K 输出；开放权重计划 10 月 15 日</x:v>
+      </x:c>
+      <x:c r="F115" s="147" t="str">
+        <x:v>StepFun API</x:v>
+      </x:c>
+      <x:c r="G115" s="147" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/models/step-5-preview.md</x:v>
+      </x:c>
+      <x:c r="H115" s="147" t="str">
+        <x:v>【公开事实｜Preview】</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c697578c0ea4ff0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4ec4e70cca54e8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5327,7 +5473,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>当前代表模型 API 价格（查询日快照；默认标准短上下文）</x:v>
+        <x:v>当前代表模型 API 价格（查询日快照；计价单位见各行）</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
         <x:v>当前代表模型 API 价格（查询日快照；默认标准短上下文）</x:v>
@@ -6742,26 +6888,26 @@
         <x:v>每百万tokens</x:v>
       </x:c>
       <x:c r="G32" s="102" t="n">
-        <x:v>3</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="H32" s="102" t="n">
-        <x:v>0.025</x:v>
+        <x:v>0.15</x:v>
       </x:c>
       <x:c r="I32" s="102"/>
       <x:c r="J32" s="102" t="n">
-        <x:v>6</x:v>
+        <x:v>13.5</x:v>
       </x:c>
       <x:c r="K32" s="64" t="str">
-        <x:v>1M</x:v>
+        <x:v>原厂 V4-Pro-0813 闲时</x:v>
       </x:c>
       <x:c r="L32" s="64" t="str">
-        <x:v>原厂 USD 价与人民币页面略有四舍五入</x:v>
+        <x:v>忙时输入/缓存/输出 ¥9/¥0.30/¥27；云平台托管价不同</x:v>
       </x:c>
       <x:c r="M32" s="64" t="str">
-        <x:v>2026-08-24</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
       <x:c r="N32" s="96" t="str">
-        <x:v>https://api-docs.deepseek.com/quick_start/pricing</x:v>
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing/</x:v>
       </x:c>
       <x:c r="O32" s="91" t="str">
         <x:v>官方价格页</x:v>
@@ -8017,6 +8163,227 @@
       </x:c>
       <x:c r="O60" s="146" t="str">
         <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="56" customHeight="1">
+      <x:c r="A61" s="147" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B61" s="147" t="str">
+        <x:v>阶跃星辰 StepFun</x:v>
+      </x:c>
+      <x:c r="C61" s="147" t="str">
+        <x:v>Step 5 Preview</x:v>
+      </x:c>
+      <x:c r="D61" s="147" t="str">
+        <x:v>Preview</x:v>
+      </x:c>
+      <x:c r="E61" s="147" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F61" s="147" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G61" s="147" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H61" s="147" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="I61" s="147"/>
+      <x:c r="J61" s="147" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K61" s="147" t="str">
+        <x:v>1M 上下文；64K 输出</x:v>
+      </x:c>
+      <x:c r="L61" s="147" t="str">
+        <x:v>模型 ID step-5-preview；当前未开放权重</x:v>
+      </x:c>
+      <x:c r="M61" s="147" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="N61" s="147" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
+      </x:c>
+      <x:c r="O61" s="147" t="str">
+        <x:v>官方价格 / 模型页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="56" customHeight="1">
+      <x:c r="A62" s="146" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B62" s="146" t="str">
+        <x:v>智谱 AI / GLM</x:v>
+      </x:c>
+      <x:c r="C62" s="146" t="str">
+        <x:v>GLM-5.3-Flash</x:v>
+      </x:c>
+      <x:c r="D62" s="146" t="str">
+        <x:v>公开可用</x:v>
+      </x:c>
+      <x:c r="E62" s="146" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F62" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G62" s="146" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H62" s="146" t="n">
+        <x:v>0.23</x:v>
+      </x:c>
+      <x:c r="I62" s="146"/>
+      <x:c r="J62" s="146" t="n">
+        <x:v>2.8</x:v>
+      </x:c>
+      <x:c r="K62" s="146" t="str">
+        <x:v>标准价；1M 上下文</x:v>
+      </x:c>
+      <x:c r="L62" s="146" t="str">
+        <x:v>限时五折 ¥0.4/¥0.115/¥1.4，截止日未披露</x:v>
+      </x:c>
+      <x:c r="M62" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="N62" s="146" t="str">
+        <x:v>https://bigmodel.cn/pricing</x:v>
+      </x:c>
+      <x:c r="O62" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="56" customHeight="1">
+      <x:c r="A63" s="147" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B63" s="147" t="str">
+        <x:v>阿里云 / 通义千问 Qwen</x:v>
+      </x:c>
+      <x:c r="C63" s="147" t="str">
+        <x:v>Qwen3.8 Omni Flash</x:v>
+      </x:c>
+      <x:c r="D63" s="147" t="str">
+        <x:v>公开可用</x:v>
+      </x:c>
+      <x:c r="E63" s="147" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F63" s="147" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G63" s="147" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H63" s="147" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="I63" s="147"/>
+      <x:c r="J63" s="147" t="n">
+        <x:v>2.7</x:v>
+      </x:c>
+      <x:c r="K63" s="147" t="str">
+        <x:v>中国内地；qwen3.8-omni-flash</x:v>
+      </x:c>
+      <x:c r="L63" s="147" t="str">
+        <x:v>多模态输入需按官方计量规则复核</x:v>
+      </x:c>
+      <x:c r="M63" s="147" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="N63" s="147" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
+      </x:c>
+      <x:c r="O63" s="147" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="56" customHeight="1">
+      <x:c r="A64" s="146" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B64" s="146" t="str">
+        <x:v>腾讯云 TokenHub</x:v>
+      </x:c>
+      <x:c r="C64" s="146" t="str">
+        <x:v>Kimi K2.8 Preview</x:v>
+      </x:c>
+      <x:c r="D64" s="146" t="str">
+        <x:v>Preview</x:v>
+      </x:c>
+      <x:c r="E64" s="146" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F64" s="146" t="str">
+        <x:v>每百万tokens</x:v>
+      </x:c>
+      <x:c r="G64" s="146" t="n">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="H64" s="146" t="n">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="I64" s="146"/>
+      <x:c r="J64" s="146" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="K64" s="146" t="str">
+        <x:v>腾讯云托管版</x:v>
+      </x:c>
+      <x:c r="L64" s="146" t="str">
+        <x:v>与 Kimi 原厂 K2.7 Code 及其缓存价不可混用</x:v>
+      </x:c>
+      <x:c r="M64" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="N64" s="146" t="str">
+        <x:v>https://cloud.tencent.com/document/product/1823/130055</x:v>
+      </x:c>
+      <x:c r="O64" s="146" t="str">
+        <x:v>TokenHub 价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="76" customHeight="1">
+      <x:c r="A65" s="147" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B65" s="147" t="str">
+        <x:v>MiniMax</x:v>
+      </x:c>
+      <x:c r="C65" s="147" t="str">
+        <x:v>MiniMax H3 视频 768P</x:v>
+      </x:c>
+      <x:c r="D65" s="147" t="str">
+        <x:v>公开可用</x:v>
+      </x:c>
+      <x:c r="E65" s="147" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="F65" s="147" t="str">
+        <x:v>每秒输出视频</x:v>
+      </x:c>
+      <x:c r="G65" s="147"/>
+      <x:c r="H65" s="147"/>
+      <x:c r="I65" s="147"/>
+      <x:c r="J65" s="147" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="K65" s="147" t="str">
+        <x:v>768P；2K ¥0.80/秒</x:v>
+      </x:c>
+      <x:c r="L65" s="147" t="str">
+        <x:v>H3 Max 480P ¥0.33/秒、768P ¥0.50/秒；输入视频/超额图片另计；不纳入 Token 成本计算器</x:v>
+      </x:c>
+      <x:c r="M65" s="147" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="N65" s="147" t="str">
+        <x:v>https://platform.minimax.cn/docs/guides/pricing-paygo</x:v>
+      </x:c>
+      <x:c r="O65" s="147" t="str">
+        <x:v>官方视频 API 价格页</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8025,7 +8392,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R308c72477ebe4fa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5f08b0376d44f13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11012,6 +11379,206 @@
       </x:c>
       <x:c r="O65"/>
     </x:row>
+    <x:row r="66" ht="32" customHeight="1">
+      <x:c r="A66" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>阶跃星辰 StepFun</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>Step 5 Preview</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E66" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F66" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="G66" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H66" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I66" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E66+$B$5*IF(F66="",E66,F66))+$B$3*G66)*(1-$B$7)</x:f>
+        <x:v>2001</x:v>
+      </x:c>
+      <x:c r="J66" t="n">
+        <x:f>IF(D66="USD",I66*$B$6,I66)</x:f>
+        <x:v>2001</x:v>
+      </x:c>
+      <x:c r="K66" t="n">
+        <x:f>J66/$B$4*1000</x:f>
+        <x:v>20.01</x:v>
+      </x:c>
+      <x:c r="L66" t="n">
+        <x:f>IFERROR(J66/($B$4*H66),"")</x:f>
+        <x:v>0.023541176470588236</x:v>
+      </x:c>
+      <x:c r="M66" t="str">
+        <x:f>IF(H66&lt;0.7,"先修质量",IF(L66&lt;0.01,"极低成本",IF(L66&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>低成本</x:v>
+      </x:c>
+      <x:c r="N66" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
+      </x:c>
+      <x:c r="O66"/>
+    </x:row>
+    <x:row r="67" ht="32" customHeight="1">
+      <x:c r="A67" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>智谱 AI / GLM</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>GLM-5.3-Flash</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E67" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="F67" t="n">
+        <x:v>0.23</x:v>
+      </x:c>
+      <x:c r="G67" t="n">
+        <x:v>2.8</x:v>
+      </x:c>
+      <x:c r="H67" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I67" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E67+$B$5*IF(F67="",E67,F67))+$B$3*G67)*(1-$B$7)</x:f>
+        <x:v>265.8</x:v>
+      </x:c>
+      <x:c r="J67" t="n">
+        <x:f>IF(D67="USD",I67*$B$6,I67)</x:f>
+        <x:v>265.8</x:v>
+      </x:c>
+      <x:c r="K67" t="n">
+        <x:f>J67/$B$4*1000</x:f>
+        <x:v>2.6580000000000004</x:v>
+      </x:c>
+      <x:c r="L67" t="n">
+        <x:f>IFERROR(J67/($B$4*H67),"")</x:f>
+        <x:v>0.003127058823529412</x:v>
+      </x:c>
+      <x:c r="M67" t="str">
+        <x:f>IF(H67&lt;0.7,"先修质量",IF(L67&lt;0.01,"极低成本",IF(L67&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>极低成本</x:v>
+      </x:c>
+      <x:c r="N67" t="str">
+        <x:v>https://bigmodel.cn/pricing</x:v>
+      </x:c>
+      <x:c r="O67"/>
+    </x:row>
+    <x:row r="68" ht="32" customHeight="1">
+      <x:c r="A68" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>阿里云 / 通义千问 Qwen</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>Qwen3.8 Omni Flash</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E68" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="F68" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="G68" t="n">
+        <x:v>2.7</x:v>
+      </x:c>
+      <x:c r="H68" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I68" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E68+$B$5*IF(F68="",E68,F68))+$B$3*G68)*(1-$B$7)</x:f>
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="J68" t="n">
+        <x:f>IF(D68="USD",I68*$B$6,I68)</x:f>
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="K68" t="n">
+        <x:f>J68/$B$4*1000</x:f>
+        <x:v>2.5300000000000002</x:v>
+      </x:c>
+      <x:c r="L68" t="n">
+        <x:f>IFERROR(J68/($B$4*H68),"")</x:f>
+        <x:v>0.002976470588235294</x:v>
+      </x:c>
+      <x:c r="M68" t="str">
+        <x:f>IF(H68&lt;0.7,"先修质量",IF(L68&lt;0.01,"极低成本",IF(L68&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>极低成本</x:v>
+      </x:c>
+      <x:c r="N68" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
+      </x:c>
+      <x:c r="O68"/>
+    </x:row>
+    <x:row r="69" ht="32" customHeight="1">
+      <x:c r="A69" t="str">
+        <x:v>国内</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>腾讯云 TokenHub</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>Kimi K2.8 Preview</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="E69" t="n">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="F69" t="n">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="G69" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="H69" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I69" t="n">
+        <x:f>$B$4/1000000*($B$2*((1-$B$5)*E69+$B$5*IF(F69="",E69,F69))+$B$3*G69)*(1-$B$7)</x:f>
+        <x:v>2362</x:v>
+      </x:c>
+      <x:c r="J69" t="n">
+        <x:f>IF(D69="USD",I69*$B$6,I69)</x:f>
+        <x:v>2362</x:v>
+      </x:c>
+      <x:c r="K69" t="n">
+        <x:f>J69/$B$4*1000</x:f>
+        <x:v>23.619999999999997</x:v>
+      </x:c>
+      <x:c r="L69" t="n">
+        <x:f>IFERROR(J69/($B$4*H69),"")</x:f>
+        <x:v>0.02778823529411765</x:v>
+      </x:c>
+      <x:c r="M69" t="str">
+        <x:f>IF(H69&lt;0.7,"先修质量",IF(L69&lt;0.01,"极低成本",IF(L69&lt;0.1,"低成本","需看价值")))</x:f>
+        <x:v>低成本</x:v>
+      </x:c>
+      <x:c r="N69" t="str">
+        <x:v>https://cloud.tencent.com/document/product/1823/130055</x:v>
+      </x:c>
+      <x:c r="O69"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
@@ -11024,7 +11591,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6e468b7a4124d91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14e835d626b847a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11237,7 +11804,7 @@
         <x:v>https://openai.com/index/ada/</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="54" customHeight="1">
+    <x:row r="7" ht="63" customHeight="1">
       <x:c r="A7" s="90" t="str">
         <x:v>企业搜索</x:v>
       </x:c>
@@ -11248,25 +11815,25 @@
         <x:v>Anthropic</x:v>
       </x:c>
       <x:c r="D7" s="64" t="str">
-        <x:v>Claude + 检索 + Prompt Caching</x:v>
+        <x:v>Claude / Opus 4.6 + 检索 + Prompt Caching</x:v>
       </x:c>
       <x:c r="E7" s="64" t="str">
-        <x:v>企业搜索、问答、写作</x:v>
+        <x:v>企业搜索、问答、写作；Notion Agent 并行任务</x:v>
       </x:c>
       <x:c r="F7" s="64" t="str">
-        <x:v>Osaka Gas 搜索时间降 35%；Remote 每次搜索约节省 10 分钟</x:v>
+        <x:v>Osaka Gas 搜索时间降 35%；Remote 每次约省 10 分钟；Managed Agents 支持 30+ 并行任务；缓存成本降 90%、延迟最多降 85%</x:v>
       </x:c>
       <x:c r="G7" s="64" t="str">
         <x:v>A｜官方案例</x:v>
       </x:c>
       <x:c r="H7" s="64" t="str">
-        <x:v>不同客户场景与统计口径不同</x:v>
+        <x:v>不同客户和时期；缓存指标属于系统工程，不可只归因底模</x:v>
       </x:c>
       <x:c r="I7" s="64" t="str">
-        <x:v>2024-2025</x:v>
+        <x:v>2024-2026</x:v>
       </x:c>
       <x:c r="J7" s="136" t="str">
-        <x:v>https://www.anthropic.com/customers/notion</x:v>
+        <x:v>https://claude.com/customers/notion</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -11330,7 +11897,7 @@
         <x:v>2024-2025</x:v>
       </x:c>
       <x:c r="J9" s="136" t="str">
-        <x:v>https://www.anthropic.com/customers/replit</x:v>
+        <x:v>https://claude.com/customers/replit?from_blog=true</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -11472,13 +12039,13 @@
         <x:v>Google</x:v>
       </x:c>
       <x:c r="D14" s="64" t="str">
-        <x:v>基于 Gemma 3 的 4B/27B 医疗开放模型</x:v>
+        <x:v>基于 Gemma 3 的 MedGemma 4B / 27B Text 医疗开放模型</x:v>
       </x:c>
       <x:c r="E14" s="64" t="str">
         <x:v>医疗文本、影像与边缘研究</x:v>
       </x:c>
       <x:c r="F14" s="64" t="str">
-        <x:v>官方报告 4B/27B 在 MedQA 为 64.4%/87.7%；强调较低推理成本</x:v>
+        <x:v>官方报告 4B / 27B Text 在 MedQA 为 64.4% / 87.7%；不代表所有 27B 变体</x:v>
       </x:c>
       <x:c r="G14" s="64" t="str">
         <x:v>A｜模型卡/研究</x:v>
@@ -11824,13 +12391,13 @@
         <x:v>字节跳动</x:v>
       </x:c>
       <x:c r="D25" s="64" t="str">
-        <x:v>Seed 2.0/2.1 系列</x:v>
+        <x:v>Seed 2.0 Pro / Code</x:v>
       </x:c>
       <x:c r="E25" s="64" t="str">
         <x:v>搜索、代码、GUI、多模态 Agent</x:v>
       </x:c>
       <x:c r="F25" s="64" t="str">
-        <x:v>官方确认模型进入豆包与 TRAE；无独立业务指标</x:v>
+        <x:v>官方确认 Seed 2.0 接入豆包与 TRAE；无独立业务指标</x:v>
       </x:c>
       <x:c r="G25" s="64" t="str">
         <x:v>B｜官方产品事实</x:v>
@@ -11888,7 +12455,7 @@
         <x:v>MiniMax</x:v>
       </x:c>
       <x:c r="D27" s="93" t="str">
-        <x:v>M2.5/M2.7</x:v>
+        <x:v>M2.7</x:v>
       </x:c>
       <x:c r="E27" s="93" t="str">
         <x:v>代码、检索、Word/PPT/Excel Office Skills</x:v>
@@ -11906,7 +12473,7 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="J27" s="137" t="str">
-        <x:v>https://www.minimax.io/news/minimax-m25</x:v>
+        <x:v>https://www.minimax.io/news/minimax-m27-en</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
@@ -11939,6 +12506,38 @@
       </x:c>
       <x:c r="J28" s="146" t="str">
         <x:v>https://developer.nvidia.com/blog/from-wafer-out-to-first-token-codifying-supply-chain-expertise-with-nemotron-and-palantir-foundry/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="76" customHeight="1">
+      <x:c r="A29" s="147" t="str">
+        <x:v>代码 Agent</x:v>
+      </x:c>
+      <x:c r="B29" s="147" t="str">
+        <x:v>Perplexity</x:v>
+      </x:c>
+      <x:c r="C29" s="147" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="D29" s="147" t="str">
+        <x:v>GPT-6 Astra</x:v>
+      </x:c>
+      <x:c r="E29" s="147" t="str">
+        <x:v>编写通信内容、修改和监控生产系统、生成端到端模拟测试</x:v>
+      </x:c>
+      <x:c r="F29" s="147" t="str">
+        <x:v>官方称减少人工盯守；未披露统一量化业务指标</x:v>
+      </x:c>
+      <x:c r="G29" s="147" t="str">
+        <x:v>A｜OpenAI 官方案例</x:v>
+      </x:c>
+      <x:c r="H29" s="147" t="str">
+        <x:v>多工具与工程流程共同贡献，不外推独立底模效果</x:v>
+      </x:c>
+      <x:c r="I29" s="147" t="str">
+        <x:v>2026-09-14</x:v>
+      </x:c>
+      <x:c r="J29" s="147" t="str">
+        <x:v>https://openai.com/index/perplexity-improving-accuracy-with-astra/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11947,7 +12546,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7295ce44d5f9436d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d50b159ed7548f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12336,7 +12935,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d736f9cfa9343e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5247eb20dcb4446d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12394,7 +12993,7 @@
         <x:v>时间范围</x:v>
       </x:c>
       <x:c r="B4" s="91" t="str">
-        <x:v>2023-01-01 至 2026-09-07；时间轴保留关键代际和产品变化，不穷尽每个快照、实验版或区域别名。</x:v>
+        <x:v>2023-01-01 至 2026-09-21；时间轴保留关键代际和产品变化，不穷尽每个快照、实验版或区域别名。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -15823,6 +16422,406 @@
       </x:c>
       <x:c r="F180" s="146" t="str">
         <x:v>A｜NVIDIA 官方案例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="56" customHeight="1">
+      <x:c r="A181" s="148" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B181" s="148" t="str">
+        <x:v>Google｜Gemini 3.8 Live</x:v>
+      </x:c>
+      <x:c r="C181" s="148" t="str">
+        <x:v>2026-09-15｜两个实时语音模型 GA</x:v>
+      </x:c>
+      <x:c r="D181" s="148" t="str">
+        <x:v>https://ai.google.dev/gemini-api/docs/changelog</x:v>
+      </x:c>
+      <x:c r="E181" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F181" s="148" t="str">
+        <x:v>公开事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="56" customHeight="1">
+      <x:c r="A182" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B182" s="146" t="str">
+        <x:v>Google｜Antigravity Preview</x:v>
+      </x:c>
+      <x:c r="C182" s="146" t="str">
+        <x:v>2026-09-17｜新版发布；旧版计划 10 月 5 日停用</x:v>
+      </x:c>
+      <x:c r="D182" s="146" t="str">
+        <x:v>https://ai.google.dev/gemini-api/docs/deprecations</x:v>
+      </x:c>
+      <x:c r="E182" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F182" s="146" t="str">
+        <x:v>公开事实｜尚未退役</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="56" customHeight="1">
+      <x:c r="A183" s="148" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B183" s="148" t="str">
+        <x:v>xAI｜Voice Transcribe 2.0</x:v>
+      </x:c>
+      <x:c r="C183" s="148" t="str">
+        <x:v>2026-09-17｜新版上线，默认仍为 1.0</x:v>
+      </x:c>
+      <x:c r="D183" s="148" t="str">
+        <x:v>https://docs.x.ai/developers/release-notes</x:v>
+      </x:c>
+      <x:c r="E183" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F183" s="148" t="str">
+        <x:v>公开事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="56" customHeight="1">
+      <x:c r="A184" s="146" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B184" s="146" t="str">
+        <x:v>OpenAI｜GPT-6 Astra Law</x:v>
+      </x:c>
+      <x:c r="C184" s="146" t="str">
+        <x:v>2026-09-17｜部分机构 Trusted Access；API 即将推出</x:v>
+      </x:c>
+      <x:c r="D184" s="146" t="str">
+        <x:v>https://openai.com/index/astra-for-law/</x:v>
+      </x:c>
+      <x:c r="E184" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F184" s="146" t="str">
+        <x:v>公开事实｜非公开 API GA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="56" customHeight="1">
+      <x:c r="A185" s="148" t="str">
+        <x:v>模型时间轴</x:v>
+      </x:c>
+      <x:c r="B185" s="148" t="str">
+        <x:v>阶跃星辰｜Step 5 Preview</x:v>
+      </x:c>
+      <x:c r="C185" s="148" t="str">
+        <x:v>1M 上下文、64K 输出；具体发布日期未披露</x:v>
+      </x:c>
+      <x:c r="D185" s="148" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/models/step-5-preview.md</x:v>
+      </x:c>
+      <x:c r="E185" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F185" s="148" t="str">
+        <x:v>公开事实｜Preview</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="56" customHeight="1">
+      <x:c r="A186" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B186" s="146" t="str">
+        <x:v>DeepSeek｜V4 Pro 原厂</x:v>
+      </x:c>
+      <x:c r="C186" s="146" t="str">
+        <x:v>闲时 4.5/0.15/13.5；忙时 9/0.30/27 CNY/百万tokens</x:v>
+      </x:c>
+      <x:c r="D186" s="146" t="str">
+        <x:v>https://api-docs.deepseek.com/zh-cn/quick_start/pricing/</x:v>
+      </x:c>
+      <x:c r="E186" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F186" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="56" customHeight="1">
+      <x:c r="A187" s="148" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B187" s="148" t="str">
+        <x:v>阶跃星辰｜Step 5 Preview</x:v>
+      </x:c>
+      <x:c r="C187" s="148" t="str">
+        <x:v>7/0.35/20 CNY/百万tokens</x:v>
+      </x:c>
+      <x:c r="D187" s="148" t="str">
+        <x:v>https://platform.stepfun.com/docs/zh/guides/pricing/details</x:v>
+      </x:c>
+      <x:c r="E187" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F187" s="148" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="56" customHeight="1">
+      <x:c r="A188" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B188" s="146" t="str">
+        <x:v>智谱｜GLM-5.3-Flash</x:v>
+      </x:c>
+      <x:c r="C188" s="146" t="str">
+        <x:v>标准 0.8/0.23/2.8 CNY/百万tokens；促销截止日未公布</x:v>
+      </x:c>
+      <x:c r="D188" s="146" t="str">
+        <x:v>https://bigmodel.cn/pricing</x:v>
+      </x:c>
+      <x:c r="E188" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F188" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="56" customHeight="1">
+      <x:c r="A189" s="148" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B189" s="148" t="str">
+        <x:v>阿里云｜Qwen3.8 Omni Flash</x:v>
+      </x:c>
+      <x:c r="C189" s="148" t="str">
+        <x:v>0.8/0.1/2.7 CNY/百万tokens</x:v>
+      </x:c>
+      <x:c r="D189" s="148" t="str">
+        <x:v>https://help.aliyun.com/zh/model-studio/model-pricing</x:v>
+      </x:c>
+      <x:c r="E189" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F189" s="148" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="56" customHeight="1">
+      <x:c r="A190" s="146" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B190" s="146" t="str">
+        <x:v>腾讯云｜Kimi K2.8 Preview</x:v>
+      </x:c>
+      <x:c r="C190" s="146" t="str">
+        <x:v>6.5/1.7/27 CNY/百万tokens；仅 TokenHub 托管价</x:v>
+      </x:c>
+      <x:c r="D190" s="146" t="str">
+        <x:v>https://cloud.tencent.com/document/product/1823/130055</x:v>
+      </x:c>
+      <x:c r="E190" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F190" s="146" t="str">
+        <x:v>官方价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="56" customHeight="1">
+      <x:c r="A191" s="148" t="str">
+        <x:v>价格</x:v>
+      </x:c>
+      <x:c r="B191" s="148" t="str">
+        <x:v>MiniMax｜H3 视频 768P</x:v>
+      </x:c>
+      <x:c r="C191" s="148" t="str">
+        <x:v>输出 0.50 CNY/秒；输入视频/超额图片另计</x:v>
+      </x:c>
+      <x:c r="D191" s="148" t="str">
+        <x:v>https://platform.minimax.cn/docs/guides/pricing-paygo</x:v>
+      </x:c>
+      <x:c r="E191" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F191" s="148" t="str">
+        <x:v>官方视频价格页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="56" customHeight="1">
+      <x:c r="A192" s="146" t="str">
+        <x:v>应用案例</x:v>
+      </x:c>
+      <x:c r="B192" s="146" t="str">
+        <x:v>Notion AI</x:v>
+      </x:c>
+      <x:c r="C192" s="146" t="str">
+        <x:v>Opus 4.6、Managed Agents 与历史客户搜索指标</x:v>
+      </x:c>
+      <x:c r="D192" s="146" t="str">
+        <x:v>https://claude.com/customers/notion</x:v>
+      </x:c>
+      <x:c r="E192" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F192" s="146" t="str">
+        <x:v>A｜Claude 官方案例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="56" customHeight="1">
+      <x:c r="A193" s="148" t="str">
+        <x:v>应用案例</x:v>
+      </x:c>
+      <x:c r="B193" s="148" t="str">
+        <x:v>Replit Agent 历史案例</x:v>
+      </x:c>
+      <x:c r="C193" s="148" t="str">
+        <x:v>旧 Vertex AI / Cloud Run 案例的官方历史页</x:v>
+      </x:c>
+      <x:c r="D193" s="148" t="str">
+        <x:v>https://claude.com/customers/replit?from_blog=true</x:v>
+      </x:c>
+      <x:c r="E193" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F193" s="148" t="str">
+        <x:v>A｜Claude 官方案例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="56" customHeight="1">
+      <x:c r="A194" s="146" t="str">
+        <x:v>应用案例</x:v>
+      </x:c>
+      <x:c r="B194" s="146" t="str">
+        <x:v>MedGemma</x:v>
+      </x:c>
+      <x:c r="C194" s="146" t="str">
+        <x:v>MedQA 87.7% 对应 27B Text 变体</x:v>
+      </x:c>
+      <x:c r="D194" s="146" t="str">
+        <x:v>https://research.google/blog/medgemma-our-most-capable-open-models-for-health-ai-development/</x:v>
+      </x:c>
+      <x:c r="E194" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F194" s="146" t="str">
+        <x:v>A｜Google Research</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="56" customHeight="1">
+      <x:c r="A195" s="148" t="str">
+        <x:v>应用案例</x:v>
+      </x:c>
+      <x:c r="B195" s="148" t="str">
+        <x:v>MiniMax Agent</x:v>
+      </x:c>
+      <x:c r="C195" s="148" t="str">
+        <x:v>M2.7 支持 Word/Excel/PPT 多轮编辑</x:v>
+      </x:c>
+      <x:c r="D195" s="148" t="str">
+        <x:v>https://www.minimax.io/news/minimax-m27-en</x:v>
+      </x:c>
+      <x:c r="E195" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F195" s="148" t="str">
+        <x:v>B｜官方产品事实</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="56" customHeight="1">
+      <x:c r="A196" s="146" t="str">
+        <x:v>应用案例</x:v>
+      </x:c>
+      <x:c r="B196" s="146" t="str">
+        <x:v>Perplexity</x:v>
+      </x:c>
+      <x:c r="C196" s="146" t="str">
+        <x:v>GPT-6 Astra 用于生产系统与端到端模拟测试</x:v>
+      </x:c>
+      <x:c r="D196" s="146" t="str">
+        <x:v>https://openai.com/index/perplexity-improving-accuracy-with-astra/</x:v>
+      </x:c>
+      <x:c r="E196" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F196" s="146" t="str">
+        <x:v>A｜OpenAI 官方案例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="56" customHeight="1">
+      <x:c r="A197" s="148" t="str">
+        <x:v>订阅权益</x:v>
+      </x:c>
+      <x:c r="B197" s="148" t="str">
+        <x:v>ChatGPT Pro 5× / 20×</x:v>
+      </x:c>
+      <x:c r="C197" s="148" t="str">
+        <x:v>精确 Pro 消息限额；20× 暂停新购另见帮助中心</x:v>
+      </x:c>
+      <x:c r="D197" s="148" t="str">
+        <x:v>https://help.openai.com/en/articles/20001354-gpt-56-and-gpt-6-pro-in-chatgpt</x:v>
+      </x:c>
+      <x:c r="E197" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F197" s="148" t="str">
+        <x:v>官方帮助中心</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="56" customHeight="1">
+      <x:c r="A198" s="146" t="str">
+        <x:v>订阅权益</x:v>
+      </x:c>
+      <x:c r="B198" s="146" t="str">
+        <x:v>Claude Pro</x:v>
+      </x:c>
+      <x:c r="C198" s="146" t="str">
+        <x:v>Slides / Docs / Microsoft 365 权益</x:v>
+      </x:c>
+      <x:c r="D198" s="146" t="str">
+        <x:v>https://claude.com/pricing</x:v>
+      </x:c>
+      <x:c r="E198" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F198" s="146" t="str">
+        <x:v>官方定价页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="56" customHeight="1">
+      <x:c r="A199" s="148" t="str">
+        <x:v>订阅权益</x:v>
+      </x:c>
+      <x:c r="B199" s="148" t="str">
+        <x:v>Mistral Vibe Pro</x:v>
+      </x:c>
+      <x:c r="C199" s="148" t="str">
+        <x:v>普通每月 $30、教育每月 $15 API credits</x:v>
+      </x:c>
+      <x:c r="D199" s="148" t="str">
+        <x:v>https://mistral.ai/pricing/</x:v>
+      </x:c>
+      <x:c r="E199" s="148" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F199" s="148" t="str">
+        <x:v>官方定价页</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="56" customHeight="1">
+      <x:c r="A200" s="146" t="str">
+        <x:v>订阅权益</x:v>
+      </x:c>
+      <x:c r="B200" s="146" t="str">
+        <x:v>Kimi 会员</x:v>
+      </x:c>
+      <x:c r="C200" s="146" t="str">
+        <x:v>共享 Token 额度池；Kimi Code 5 小时/周</x:v>
+      </x:c>
+      <x:c r="D200" s="146" t="str">
+        <x:v>https://www.kimi.com/help/membership/membership-pricing</x:v>
+      </x:c>
+      <x:c r="E200" s="146" t="str">
+        <x:v>2026-09-21</x:v>
+      </x:c>
+      <x:c r="F200" s="146" t="str">
+        <x:v>官方会员页</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15831,7 +16830,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf97678a9b73454f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8841d9e851834dde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>